<commit_message>
Recover seven institutional Quran specifications
</commit_message>
<xml_diff>
--- a/قائمة_المقررات_التخصصية_المفقودة_2026-09-10.xlsx
+++ b/قائمة_المقررات_التخصصية_المفقودة_2026-09-10.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الملخص" sheetId="1" r:id="R543ef7c7721a491d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="المقررات المفقودة" sheetId="2" r:id="Rfbc63b27ce4042e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="مواضع الخطط" sheetId="3" r:id="R6b82ed7f74454a9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الملخص" sheetId="1" r:id="R544b04a06e2e4fbf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="المقررات المفقودة" sheetId="2" r:id="Rcd8d97c65e294443"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="مواضع الخطط" sheetId="3" r:id="R7cca6474166148fe"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -274,7 +274,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="MissingCourseIdentities" displayName="MissingCourseIdentities" ref="A5:L106" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="MissingCourseIdentities" displayName="MissingCourseIdentities" ref="A5:L105" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="م"/>
     <x:tableColumn id="2" name="رمز المقرر"/>
@@ -294,7 +294,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="MissingCourseOccurrences" displayName="MissingCourseOccurrences" ref="A5:O136" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="MissingCourseOccurrences" displayName="MissingCourseOccurrences" ref="A5:O126" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="15">
     <x:tableColumn id="1" name="م"/>
     <x:tableColumn id="2" name="البرنامج"/>
@@ -525,15 +525,42 @@
     <x:col min="9" max="9" width="13.329999923706055" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1"/>
+      <x:c r="B1"/>
+      <x:c r="C1"/>
+      <x:c r="D1"/>
+      <x:c r="E1"/>
+      <x:c r="F1"/>
+      <x:c r="G1"/>
+      <x:c r="H1"/>
+      <x:c r="I1"/>
+    </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="3" t="str">
         <x:v>المقررات التخصصية المفقودة من توصيفات برامج كلية الشريعة والأنظمة</x:v>
       </x:c>
+      <x:c r="B2"/>
+      <x:c r="C2"/>
+      <x:c r="D2"/>
+      <x:c r="E2"/>
+      <x:c r="F2"/>
+      <x:c r="G2"/>
+      <x:c r="H2"/>
+      <x:c r="I2"/>
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>المصدر: data.json في مستودع التوصيفات، بتاريخ 2026-09-10. النطاق: رموز 200* والاستثناء القديم 101221-2، دون الرسالة والاختبار الشامل أو مقررات الأقسام الخارجية.</x:v>
-      </x:c>
+        <x:v>المصدر: data.json في مستودع التوصيفات، بتاريخ 2026-09-11. النطاق: رموز 200* والاستثناء القديم 101221-2، دون الرسالة والاختبار الشامل أو مقررات الأقسام الخارجية.</x:v>
+      </x:c>
+      <x:c r="B3"/>
+      <x:c r="C3"/>
+      <x:c r="D3"/>
+      <x:c r="E3"/>
+      <x:c r="F3"/>
+      <x:c r="G3"/>
+      <x:c r="H3"/>
+      <x:c r="I3"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="7"/>
@@ -589,22 +616,18 @@
         <x:v>99</x:v>
       </x:c>
       <x:c r="E6" s="29" t="n">
-        <x:f>D6-F6</x:f>
         <x:v>76</x:v>
       </x:c>
       <x:c r="F6" s="29" t="n">
-        <x:f>COUNTIFS('مواضع الخطط'!$B$6:$B$145,A6,'مواضع الخطط'!$C$6:$C$145,B6)</x:f>
         <x:v>23</x:v>
       </x:c>
       <x:c r="G6" s="35" t="n">
-        <x:f>E6/D6</x:f>
         <x:v>0.7676767676767676</x:v>
       </x:c>
       <x:c r="H6" s="29" t="n">
         <x:v>23</x:v>
       </x:c>
       <x:c r="I6" s="32" t="str">
-        <x:f>IF(F6=0,"مكتمل","يحتاج استكمال")</x:f>
         <x:v>يحتاج استكمال</x:v>
       </x:c>
     </x:row>
@@ -634,7 +657,6 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="I7" s="33" t="str">
-        <x:f>IF(F7=0,"مكتمل","يحتاج استكمال")</x:f>
         <x:v>يحتاج استكمال</x:v>
       </x:c>
     </x:row>
@@ -652,22 +674,18 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="E8" s="30" t="n">
-        <x:f>D8-F8</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="F8" s="30" t="n">
-        <x:f>COUNTIFS('مواضع الخطط'!$B$6:$B$145,A8,'مواضع الخطط'!$C$6:$C$145,B8)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G8" s="36" t="n">
-        <x:f>E8/D8</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="H8" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I8" s="33" t="str">
-        <x:f>IF(F8=0,"مكتمل","يحتاج استكمال")</x:f>
         <x:v>مكتمل</x:v>
       </x:c>
     </x:row>
@@ -685,22 +703,18 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="E9" s="30" t="n">
-        <x:f>D9-F9</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="F9" s="30" t="n">
-        <x:f>COUNTIFS('مواضع الخطط'!$B$6:$B$145,A9,'مواضع الخطط'!$C$6:$C$145,B9)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G9" s="36" t="n">
-        <x:f>E9/D9</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="H9" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I9" s="33" t="str">
-        <x:f>IF(F9=0,"مكتمل","يحتاج استكمال")</x:f>
         <x:v>مكتمل</x:v>
       </x:c>
     </x:row>
@@ -718,22 +732,18 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="E10" s="30" t="n">
-        <x:f>D10-F10</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="F10" s="30" t="n">
-        <x:f>COUNTIFS('مواضع الخطط'!$B$6:$B$145,A10,'مواضع الخطط'!$C$6:$C$145,B10)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G10" s="36" t="n">
-        <x:f>E10/D10</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="H10" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I10" s="33" t="str">
-        <x:f>IF(F10=0,"مكتمل","يحتاج استكمال")</x:f>
         <x:v>مكتمل</x:v>
       </x:c>
     </x:row>
@@ -751,22 +761,18 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="E11" s="30" t="n">
-        <x:f>D11-F11</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="F11" s="30" t="n">
-        <x:f>COUNTIFS('مواضع الخطط'!$B$6:$B$145,A11,'مواضع الخطط'!$C$6:$C$145,B11)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G11" s="36" t="n">
-        <x:f>E11/D11</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="H11" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I11" s="33" t="str">
-        <x:f>IF(F11=0,"مكتمل","يحتاج استكمال")</x:f>
         <x:v>مكتمل</x:v>
       </x:c>
     </x:row>
@@ -796,7 +802,6 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="I12" s="33" t="str">
-        <x:f>IF(F12=0,"مكتمل","يحتاج استكمال")</x:f>
         <x:v>يحتاج استكمال</x:v>
       </x:c>
     </x:row>
@@ -814,22 +819,18 @@
         <x:v>113</x:v>
       </x:c>
       <x:c r="E13" s="30" t="n">
-        <x:f>D13-F13</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="F13" s="30" t="n">
-        <x:f>COUNTIFS('مواضع الخطط'!$B$6:$B$145,A13,'مواضع الخطط'!$C$6:$C$145,B13)</x:f>
         <x:v>23</x:v>
       </x:c>
       <x:c r="G13" s="36" t="n">
-        <x:f>E13/D13</x:f>
         <x:v>0.7964601769911505</x:v>
       </x:c>
       <x:c r="H13" s="30" t="n">
         <x:v>22</x:v>
       </x:c>
       <x:c r="I13" s="33" t="str">
-        <x:f>IF(F13=0,"مكتمل","يحتاج استكمال")</x:f>
         <x:v>يحتاج استكمال</x:v>
       </x:c>
     </x:row>
@@ -847,22 +848,18 @@
         <x:v>120</x:v>
       </x:c>
       <x:c r="E14" s="30" t="n">
-        <x:f>D14-F14</x:f>
-        <x:v>96</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="F14" s="30" t="n">
-        <x:f>COUNTIFS('مواضع الخطط'!$B$6:$B$145,A14,'مواضع الخطط'!$C$6:$C$145,B14)</x:f>
-        <x:v>24</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G14" s="36" t="n">
-        <x:f>E14/D14</x:f>
-        <x:v>0.8</x:v>
+        <x:v>0.8833333333333333</x:v>
       </x:c>
       <x:c r="H14" s="30" t="n">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="I14" s="33" t="str">
-        <x:f>IF(F14=0,"مكتمل","يحتاج استكمال")</x:f>
         <x:v>يحتاج استكمال</x:v>
       </x:c>
     </x:row>
@@ -880,22 +877,18 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="E15" s="30" t="n">
-        <x:f>D15-F15</x:f>
         <x:v>15</x:v>
       </x:c>
       <x:c r="F15" s="30" t="n">
-        <x:f>COUNTIFS('مواضع الخطط'!$B$6:$B$145,A15,'مواضع الخطط'!$C$6:$C$145,B15)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G15" s="36" t="n">
-        <x:f>E15/D15</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="H15" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I15" s="33" t="str">
-        <x:f>IF(F15=0,"مكتمل","يحتاج استكمال")</x:f>
         <x:v>مكتمل</x:v>
       </x:c>
     </x:row>
@@ -913,22 +906,18 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="E16" s="30" t="n">
-        <x:f>D16-F16</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="F16" s="30" t="n">
-        <x:f>COUNTIFS('مواضع الخطط'!$B$6:$B$145,A16,'مواضع الخطط'!$C$6:$C$145,B16)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="G16" s="36" t="n">
-        <x:f>E16/D16</x:f>
         <x:v>0.9333333333333333</x:v>
       </x:c>
       <x:c r="H16" s="30" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="I16" s="33" t="str">
-        <x:f>IF(F16=0,"مكتمل","يحتاج استكمال")</x:f>
         <x:v>يحتاج استكمال</x:v>
       </x:c>
     </x:row>
@@ -946,22 +935,18 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="E17" s="30" t="n">
-        <x:f>D17-F17</x:f>
         <x:v>21</x:v>
       </x:c>
       <x:c r="F17" s="30" t="n">
-        <x:f>COUNTIFS('مواضع الخطط'!$B$6:$B$145,A17,'مواضع الخطط'!$C$6:$C$145,B17)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G17" s="36" t="n">
-        <x:f>E17/D17</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="H17" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I17" s="33" t="str">
-        <x:f>IF(F17=0,"مكتمل","يحتاج استكمال")</x:f>
         <x:v>مكتمل</x:v>
       </x:c>
     </x:row>
@@ -979,22 +964,18 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="E18" s="30" t="n">
-        <x:f>D18-F18</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="F18" s="30" t="n">
-        <x:f>COUNTIFS('مواضع الخطط'!$B$6:$B$145,A18,'مواضع الخطط'!$C$6:$C$145,B18)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G18" s="36" t="n">
-        <x:f>E18/D18</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="H18" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I18" s="33" t="str">
-        <x:f>IF(F18=0,"مكتمل","يحتاج استكمال")</x:f>
         <x:v>مكتمل</x:v>
       </x:c>
     </x:row>
@@ -1012,22 +993,18 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="E19" s="30" t="n">
-        <x:f>D19-F19</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="F19" s="30" t="n">
-        <x:f>COUNTIFS('مواضع الخطط'!$B$6:$B$145,A19,'مواضع الخطط'!$C$6:$C$145,B19)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G19" s="36" t="n">
-        <x:f>E19/D19</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="H19" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I19" s="33" t="str">
-        <x:f>IF(F19=0,"مكتمل","يحتاج استكمال")</x:f>
         <x:v>مكتمل</x:v>
       </x:c>
     </x:row>
@@ -1045,22 +1022,18 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="E20" s="30" t="n">
-        <x:f>D20-F20</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="F20" s="30" t="n">
-        <x:f>COUNTIFS('مواضع الخطط'!$B$6:$B$145,A20,'مواضع الخطط'!$C$6:$C$145,B20)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="G20" s="36" t="n">
-        <x:f>E20/D20</x:f>
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="H20" s="30" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="I20" s="33" t="str">
-        <x:f>IF(F20=0,"مكتمل","يحتاج استكمال")</x:f>
         <x:v>يحتاج استكمال</x:v>
       </x:c>
     </x:row>
@@ -1071,20 +1044,19 @@
       <x:c r="B21" s="31"/>
       <x:c r="C21" s="31"/>
       <x:c r="D21" s="31" t="n">
-        <x:f>SUM(D6:D20)</x:f>
         <x:v>756</x:v>
       </x:c>
       <x:c r="E21" s="31" t="n">
-        <x:v>625</x:v>
+        <x:v>635</x:v>
       </x:c>
       <x:c r="F21" s="31" t="n">
-        <x:v>131</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="G21" s="37" t="n">
-        <x:v>0.8267195767195767</x:v>
+        <x:v>0.83994708994709</x:v>
       </x:c>
       <x:c r="H21" s="31" t="n">
-        <x:v>101</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="I21" s="34" t="str">
         <x:v>قائمة العمل الحالية</x:v>
@@ -1129,15 +1101,51 @@
     <x:col min="12" max="12" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1"/>
+      <x:c r="B1"/>
+      <x:c r="C1"/>
+      <x:c r="D1"/>
+      <x:c r="E1"/>
+      <x:c r="F1"/>
+      <x:c r="G1"/>
+      <x:c r="H1"/>
+      <x:c r="I1"/>
+      <x:c r="J1"/>
+      <x:c r="K1"/>
+      <x:c r="L1"/>
+    </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="3" t="str">
         <x:v>قائمة المقررات التخصصية المفقودة دون تكرار</x:v>
       </x:c>
+      <x:c r="B2"/>
+      <x:c r="C2"/>
+      <x:c r="D2"/>
+      <x:c r="E2"/>
+      <x:c r="F2"/>
+      <x:c r="G2"/>
+      <x:c r="H2"/>
+      <x:c r="I2"/>
+      <x:c r="J2"/>
+      <x:c r="K2"/>
+      <x:c r="L2"/>
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>عدد الهويات الفريدة: 101. قد يظهر المقرر نفسه في أكثر من برنامج أو خطة، وتوضح الأعمدة جميع المواضع المتأثرة.</x:v>
-      </x:c>
+        <x:v>عدد الهويات الفريدة: 100. قد يظهر المقرر نفسه في أكثر من برنامج أو خطة، وتوضح الأعمدة جميع المواضع المتأثرة.</x:v>
+      </x:c>
+      <x:c r="B3"/>
+      <x:c r="C3"/>
+      <x:c r="D3"/>
+      <x:c r="E3"/>
+      <x:c r="F3"/>
+      <x:c r="G3"/>
+      <x:c r="H3"/>
+      <x:c r="I3"/>
+      <x:c r="J3"/>
+      <x:c r="K3"/>
+      <x:c r="L3"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="7"/>
@@ -1528,28 +1536,28 @@
         <x:v>أصول الفقه (2)</x:v>
       </x:c>
       <x:c r="D15" s="39" t="str">
-        <x:v>الأنظمة، القرآن وعلومه</x:v>
+        <x:v>الأنظمة</x:v>
       </x:c>
       <x:c r="E15" s="39" t="str">
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F15" s="39" t="str">
-        <x:v>الأنظمة: قديمة 38
-القرآن وعلومه: جديدة 47
-القرآن وعلومه: قديمة 39</x:v>
+        <x:v>الأنظمة: قديمة 38</x:v>
       </x:c>
       <x:c r="G15" s="39" t="str">
-        <x:v>3، 6</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H15" s="39" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I15" s="39" t="str">
-        <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
-      </x:c>
-      <x:c r="J15" s="39"/>
+        <x:v>يوجد توصيف مؤسسي لبرنامج القرآن وعلومه فقط</x:v>
+      </x:c>
+      <x:c r="J15" s="39" t="str">
+        <x:v>institutional-recovery-20260911/2001330-2.pdf</x:v>
+      </x:c>
       <x:c r="K15" s="39" t="str">
-        <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
+        <x:v>الحصول على دليل خاص ببرنامج الأنظمة، ثم ربط مخرجاته في نطاقه فقط</x:v>
       </x:c>
       <x:c r="L15" s="39" t="str">
         <x:v>2001330-2||اصولالفقه2</x:v>
@@ -3847,27 +3855,28 @@
         <x:v>الحديث (1)</x:v>
       </x:c>
       <x:c r="D79" s="39" t="str">
-        <x:v>القراءات، القرآن وعلومه</x:v>
+        <x:v>القراءات</x:v>
       </x:c>
       <x:c r="E79" s="39" t="str">
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F79" s="39" t="str">
-        <x:v>القراءات: قديمة 38
-القرآن وعلومه: قديمة 39</x:v>
+        <x:v>القراءات: قديمة 38</x:v>
       </x:c>
       <x:c r="G79" s="39" t="str">
         <x:v>3</x:v>
       </x:c>
       <x:c r="H79" s="39" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I79" s="39" t="str">
-        <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
-      </x:c>
-      <x:c r="J79" s="39"/>
+        <x:v>يوجد توصيف مؤسسي لبرنامج القرآن وعلومه فقط</x:v>
+      </x:c>
+      <x:c r="J79" s="39" t="str">
+        <x:v>institutional-recovery-20260911/2001205-2.pdf</x:v>
+      </x:c>
       <x:c r="K79" s="39" t="str">
-        <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
+        <x:v>الحصول على دليل خاص ببرنامج القراءات، ثم ربط مخرجاته في نطاقه فقط</x:v>
       </x:c>
       <x:c r="L79" s="39" t="str">
         <x:v>2001205-2||الحديث1</x:v>
@@ -3884,27 +3893,28 @@
         <x:v>الحديث (2)</x:v>
       </x:c>
       <x:c r="D80" s="39" t="str">
-        <x:v>القراءات، القرآن وعلومه</x:v>
+        <x:v>القراءات</x:v>
       </x:c>
       <x:c r="E80" s="39" t="str">
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F80" s="39" t="str">
-        <x:v>القراءات: قديمة 38
-القرآن وعلومه: قديمة 39</x:v>
+        <x:v>القراءات: قديمة 38</x:v>
       </x:c>
       <x:c r="G80" s="39" t="str">
         <x:v>4</x:v>
       </x:c>
       <x:c r="H80" s="39" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I80" s="39" t="str">
-        <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
-      </x:c>
-      <x:c r="J80" s="39"/>
+        <x:v>يوجد توصيف مؤسسي لبرنامج القرآن وعلومه فقط</x:v>
+      </x:c>
+      <x:c r="J80" s="39" t="str">
+        <x:v>institutional-recovery-20260911/2001209-2.pdf</x:v>
+      </x:c>
       <x:c r="K80" s="39" t="str">
-        <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
+        <x:v>الحصول على دليل خاص ببرنامج القراءات، ثم ربط مخرجاته في نطاقه فقط</x:v>
       </x:c>
       <x:c r="L80" s="39" t="str">
         <x:v>2001209-2||الحديث2</x:v>
@@ -3921,28 +3931,28 @@
         <x:v>الفقه (1)</x:v>
       </x:c>
       <x:c r="D81" s="39" t="str">
-        <x:v>القراءات، القرآن وعلومه</x:v>
+        <x:v>القراءات</x:v>
       </x:c>
       <x:c r="E81" s="39" t="str">
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F81" s="39" t="str">
-        <x:v>القراءات: جديدة 47
-القراءات: قديمة 38
-القرآن وعلومه: جديدة 47</x:v>
+        <x:v>القراءات: جديدة 47؛ القراءات: قديمة 38</x:v>
       </x:c>
       <x:c r="G81" s="39" t="str">
         <x:v>3</x:v>
       </x:c>
       <x:c r="H81" s="39" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I81" s="39" t="str">
-        <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
-      </x:c>
-      <x:c r="J81" s="39"/>
+        <x:v>يوجد توصيف مؤسسي لبرنامج القرآن وعلومه فقط</x:v>
+      </x:c>
+      <x:c r="J81" s="39" t="str">
+        <x:v>institutional-recovery-20260911/2001221-2.pdf</x:v>
+      </x:c>
       <x:c r="K81" s="39" t="str">
-        <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
+        <x:v>الحصول على دليل خاص ببرنامج القراءات، ثم ربط مخرجاته في نطاقه فقط</x:v>
       </x:c>
       <x:c r="L81" s="39" t="str">
         <x:v>2001221-2||الفقه1</x:v>
@@ -3995,27 +4005,28 @@
         <x:v>الحديث (3)</x:v>
       </x:c>
       <x:c r="D83" s="39" t="str">
-        <x:v>القراءات، القرآن وعلومه</x:v>
+        <x:v>القراءات</x:v>
       </x:c>
       <x:c r="E83" s="39" t="str">
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F83" s="39" t="str">
-        <x:v>القراءات: قديمة 38
-القرآن وعلومه: قديمة 39</x:v>
+        <x:v>القراءات: قديمة 38</x:v>
       </x:c>
       <x:c r="G83" s="39" t="str">
         <x:v>6</x:v>
       </x:c>
       <x:c r="H83" s="39" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I83" s="39" t="str">
-        <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
-      </x:c>
-      <x:c r="J83" s="39"/>
+        <x:v>يوجد توصيف مؤسسي لبرنامج القرآن وعلومه فقط</x:v>
+      </x:c>
+      <x:c r="J83" s="39" t="str">
+        <x:v>institutional-recovery-20260911/2001320-2.pdf</x:v>
+      </x:c>
       <x:c r="K83" s="39" t="str">
-        <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
+        <x:v>الحصول على دليل خاص ببرنامج القراءات، ثم ربط مخرجاته في نطاقه فقط</x:v>
       </x:c>
       <x:c r="L83" s="39" t="str">
         <x:v>2001320-2||الحديث3</x:v>
@@ -4032,28 +4043,28 @@
         <x:v>الفقه (2)</x:v>
       </x:c>
       <x:c r="D84" s="39" t="str">
-        <x:v>القراءات، القرآن وعلومه</x:v>
+        <x:v>القراءات</x:v>
       </x:c>
       <x:c r="E84" s="39" t="str">
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F84" s="39" t="str">
-        <x:v>القراءات: قديمة 38
-القرآن وعلومه: جديدة 47
-القرآن وعلومه: قديمة 39</x:v>
+        <x:v>القراءات: قديمة 38</x:v>
       </x:c>
       <x:c r="G84" s="39" t="str">
         <x:v>4</x:v>
       </x:c>
       <x:c r="H84" s="39" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I84" s="39" t="str">
-        <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
-      </x:c>
-      <x:c r="J84" s="39"/>
+        <x:v>يوجد توصيف مؤسسي لبرنامج القرآن وعلومه فقط</x:v>
+      </x:c>
+      <x:c r="J84" s="39" t="str">
+        <x:v>institutional-recovery-20260911/2001322-2.pdf</x:v>
+      </x:c>
       <x:c r="K84" s="39" t="str">
-        <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
+        <x:v>الحصول على دليل خاص ببرنامج القراءات، ثم ربط مخرجاته في نطاقه فقط</x:v>
       </x:c>
       <x:c r="L84" s="39" t="str">
         <x:v>2001322-2||الفقه2</x:v>
@@ -4717,10 +4728,10 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="B103" s="33" t="str">
-        <x:v>2001317-2</x:v>
+        <x:v>2001424-2</x:v>
       </x:c>
       <x:c r="C103" s="39" t="str">
-        <x:v>الفقه (3)</x:v>
+        <x:v>الفقه (4)</x:v>
       </x:c>
       <x:c r="D103" s="39" t="str">
         <x:v>القرآن وعلومه</x:v>
@@ -4729,14 +4740,13 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F103" s="39" t="str">
-        <x:v>القرآن وعلومه: جديدة 47
-القرآن وعلومه: قديمة 39</x:v>
+        <x:v>القرآن وعلومه: قديمة 39</x:v>
       </x:c>
       <x:c r="G103" s="39" t="str">
-        <x:v>5</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H103" s="39" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I103" s="39" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
@@ -4746,7 +4756,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L103" s="39" t="str">
-        <x:v>2001317-2||الفقه3</x:v>
+        <x:v>2001424-2||الفقه4</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="42" customHeight="1">
@@ -4754,10 +4764,10 @@
         <x:v>99</x:v>
       </x:c>
       <x:c r="B104" s="33" t="str">
-        <x:v>2001424-2</x:v>
+        <x:v>2002266-5</x:v>
       </x:c>
       <x:c r="C104" s="39" t="str">
-        <x:v>الفقه (4)</x:v>
+        <x:v>التدريب التعاوني</x:v>
       </x:c>
       <x:c r="D104" s="39" t="str">
         <x:v>القرآن وعلومه</x:v>
@@ -4766,7 +4776,7 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F104" s="39" t="str">
-        <x:v>القرآن وعلومه: قديمة 39</x:v>
+        <x:v>القرآن وعلومه: جديدة 47</x:v>
       </x:c>
       <x:c r="G104" s="39" t="str">
         <x:v>8</x:v>
@@ -4782,7 +4792,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L104" s="39" t="str">
-        <x:v>2001424-2||الفقه4</x:v>
+        <x:v>2002266-5||التدريبالتعاوني</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="42" customHeight="1">
@@ -4790,10 +4800,10 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="B105" s="33" t="str">
-        <x:v>2002266-5</x:v>
+        <x:v>20024101-2</x:v>
       </x:c>
       <x:c r="C105" s="39" t="str">
-        <x:v>التدريب التعاوني</x:v>
+        <x:v>قاعة بحث</x:v>
       </x:c>
       <x:c r="D105" s="39" t="str">
         <x:v>القرآن وعلومه</x:v>
@@ -4805,7 +4815,7 @@
         <x:v>القرآن وعلومه: جديدة 47</x:v>
       </x:c>
       <x:c r="G105" s="39" t="str">
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="H105" s="39" t="n">
         <x:v>1</x:v>
@@ -4818,44 +4828,22 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L105" s="39" t="str">
-        <x:v>2002266-5||التدريبالتعاوني</x:v>
+        <x:v>20024101-2||قاعةبحث</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="42" customHeight="1">
-      <x:c r="A106" s="33" t="n">
-        <x:v>101</x:v>
-      </x:c>
-      <x:c r="B106" s="33" t="str">
-        <x:v>20024101-2</x:v>
-      </x:c>
-      <x:c r="C106" s="39" t="str">
-        <x:v>قاعة بحث</x:v>
-      </x:c>
-      <x:c r="D106" s="39" t="str">
-        <x:v>القرآن وعلومه</x:v>
-      </x:c>
-      <x:c r="E106" s="39" t="str">
-        <x:v>بكالوريوس</x:v>
-      </x:c>
-      <x:c r="F106" s="39" t="str">
-        <x:v>القرآن وعلومه: جديدة 47</x:v>
-      </x:c>
-      <x:c r="G106" s="39" t="str">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="H106" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I106" s="39" t="str">
-        <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
-      </x:c>
+      <x:c r="A106" s="33"/>
+      <x:c r="B106" s="33"/>
+      <x:c r="C106" s="39"/>
+      <x:c r="D106" s="39"/>
+      <x:c r="E106" s="39"/>
+      <x:c r="F106" s="39"/>
+      <x:c r="G106" s="39"/>
+      <x:c r="H106" s="39"/>
+      <x:c r="I106" s="39"/>
       <x:c r="J106" s="39"/>
-      <x:c r="K106" s="39" t="str">
-        <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
-      </x:c>
-      <x:c r="L106" s="39" t="str">
-        <x:v>20024101-2||قاعةبحث</x:v>
-      </x:c>
+      <x:c r="K106" s="39"/>
+      <x:c r="L106" s="39"/>
     </x:row>
     <x:row r="107" ht="42" customHeight="1">
       <x:c r="A107" s="33"/>
@@ -4934,7 +4922,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47649aa9885d4953"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c1afe0f4ade4f17"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4963,15 +4951,60 @@
     <x:col min="15" max="15" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1"/>
+      <x:c r="B1"/>
+      <x:c r="C1"/>
+      <x:c r="D1"/>
+      <x:c r="E1"/>
+      <x:c r="F1"/>
+      <x:c r="G1"/>
+      <x:c r="H1"/>
+      <x:c r="I1"/>
+      <x:c r="J1"/>
+      <x:c r="K1"/>
+      <x:c r="L1"/>
+      <x:c r="M1"/>
+      <x:c r="N1"/>
+      <x:c r="O1"/>
+    </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="3" t="str">
         <x:v>مواضع المقررات التخصصية المفقودة في الخطط</x:v>
       </x:c>
+      <x:c r="B2"/>
+      <x:c r="C2"/>
+      <x:c r="D2"/>
+      <x:c r="E2"/>
+      <x:c r="F2"/>
+      <x:c r="G2"/>
+      <x:c r="H2"/>
+      <x:c r="I2"/>
+      <x:c r="J2"/>
+      <x:c r="K2"/>
+      <x:c r="L2"/>
+      <x:c r="M2"/>
+      <x:c r="N2"/>
+      <x:c r="O2"/>
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>عدد المواضع: 131. كل صف يمثل ظهور مقرر في برنامج وخطة وإصدار محدد.</x:v>
-      </x:c>
+        <x:v>عدد المواضع: 121. كل صف يمثل ظهور مقرر في برنامج وخطة وإصدار محدد.</x:v>
+      </x:c>
+      <x:c r="B3"/>
+      <x:c r="C3"/>
+      <x:c r="D3"/>
+      <x:c r="E3"/>
+      <x:c r="F3"/>
+      <x:c r="G3"/>
+      <x:c r="H3"/>
+      <x:c r="I3"/>
+      <x:c r="J3"/>
+      <x:c r="K3"/>
+      <x:c r="L3"/>
+      <x:c r="M3"/>
+      <x:c r="N3"/>
+      <x:c r="O3"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="7"/>
@@ -9737,10 +9770,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G110" s="43" t="str">
-        <x:v>2001221-2</x:v>
+        <x:v>2003220-2</x:v>
       </x:c>
       <x:c r="H110" s="42" t="str">
-        <x:v>الفقه (1)</x:v>
+        <x:v>المدخل لدراسة الأنظمة</x:v>
       </x:c>
       <x:c r="I110" s="43" t="n">
         <x:v>2</x:v>
@@ -9759,7 +9792,7 @@
       </x:c>
       <x:c r="N110" s="42"/>
       <x:c r="O110" s="42" t="str">
-        <x:v>2001221-2||الفقه1</x:v>
+        <x:v>2003220-2||المدخللدراسةالانظمة</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="34" customHeight="1">
@@ -9782,10 +9815,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G111" s="43" t="str">
-        <x:v>2003220-2</x:v>
+        <x:v>2004205-2</x:v>
       </x:c>
       <x:c r="H111" s="42" t="str">
-        <x:v>المدخل لدراسة الأنظمة</x:v>
+        <x:v>الحديث (1)</x:v>
       </x:c>
       <x:c r="I111" s="43" t="n">
         <x:v>2</x:v>
@@ -9794,7 +9827,7 @@
         <x:v>نظري</x:v>
       </x:c>
       <x:c r="K111" s="42" t="str">
-        <x:v>إجبارية القسم</x:v>
+        <x:v>متطلبات الكلية</x:v>
       </x:c>
       <x:c r="L111" s="42" t="str">
         <x:v>القرآن وعلومه 47.pdf</x:v>
@@ -9804,7 +9837,7 @@
       </x:c>
       <x:c r="N111" s="42"/>
       <x:c r="O111" s="42" t="str">
-        <x:v>2003220-2||المدخللدراسةالانظمة</x:v>
+        <x:v>2004205-2||الحديث1</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="34" customHeight="1">
@@ -9824,13 +9857,13 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="F112" s="43" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G112" s="43" t="str">
-        <x:v>2004205-2</x:v>
+        <x:v>2004209-2</x:v>
       </x:c>
       <x:c r="H112" s="42" t="str">
-        <x:v>الحديث (1)</x:v>
+        <x:v>الحديث (2)</x:v>
       </x:c>
       <x:c r="I112" s="43" t="n">
         <x:v>2</x:v>
@@ -9849,7 +9882,7 @@
       </x:c>
       <x:c r="N112" s="42"/>
       <x:c r="O112" s="42" t="str">
-        <x:v>2004205-2||الحديث1</x:v>
+        <x:v>2004209-2||الحديث2</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="34" customHeight="1">
@@ -9869,13 +9902,13 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="F113" s="43" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G113" s="43" t="str">
-        <x:v>2001322-2</x:v>
+        <x:v>2001113-2</x:v>
       </x:c>
       <x:c r="H113" s="42" t="str">
-        <x:v>الفقه (2)</x:v>
+        <x:v>أصول الفقه (1)</x:v>
       </x:c>
       <x:c r="I113" s="43" t="n">
         <x:v>2</x:v>
@@ -9894,7 +9927,7 @@
       </x:c>
       <x:c r="N113" s="42"/>
       <x:c r="O113" s="42" t="str">
-        <x:v>2001322-2||الفقه2</x:v>
+        <x:v>2001113-2||اصولالفقه1</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="34" customHeight="1">
@@ -9914,13 +9947,13 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="F114" s="43" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G114" s="43" t="str">
-        <x:v>2004209-2</x:v>
+        <x:v>2004320-2</x:v>
       </x:c>
       <x:c r="H114" s="42" t="str">
-        <x:v>الحديث (2)</x:v>
+        <x:v>الحديث (3)</x:v>
       </x:c>
       <x:c r="I114" s="43" t="n">
         <x:v>2</x:v>
@@ -9939,7 +9972,7 @@
       </x:c>
       <x:c r="N114" s="42"/>
       <x:c r="O114" s="42" t="str">
-        <x:v>2004209-2||الحديث2</x:v>
+        <x:v>2004320-2||الحديث3</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="34" customHeight="1">
@@ -9959,13 +9992,13 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="F115" s="43" t="n">
-        <x:v>5</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G115" s="43" t="str">
-        <x:v>2001113-2</x:v>
+        <x:v>2004403-2</x:v>
       </x:c>
       <x:c r="H115" s="42" t="str">
-        <x:v>أصول الفقه (1)</x:v>
+        <x:v>الأديان والفرق والمذاهب المعاصرة</x:v>
       </x:c>
       <x:c r="I115" s="43" t="n">
         <x:v>2</x:v>
@@ -9974,7 +10007,7 @@
         <x:v>نظري</x:v>
       </x:c>
       <x:c r="K115" s="42" t="str">
-        <x:v>إجبارية القسم</x:v>
+        <x:v>متطلبات الكلية</x:v>
       </x:c>
       <x:c r="L115" s="42" t="str">
         <x:v>القرآن وعلومه 47.pdf</x:v>
@@ -9984,7 +10017,7 @@
       </x:c>
       <x:c r="N115" s="42"/>
       <x:c r="O115" s="42" t="str">
-        <x:v>2001113-2||اصولالفقه1</x:v>
+        <x:v>2004403-2||الاديانوالفرقوالمذاهبالمعاصرة</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="34" customHeight="1">
@@ -10004,13 +10037,13 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="F116" s="43" t="n">
-        <x:v>5</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G116" s="43" t="str">
-        <x:v>2001317-2</x:v>
+        <x:v>20024101-2</x:v>
       </x:c>
       <x:c r="H116" s="42" t="str">
-        <x:v>الفقه (3)</x:v>
+        <x:v>قاعة بحث</x:v>
       </x:c>
       <x:c r="I116" s="43" t="n">
         <x:v>2</x:v>
@@ -10029,7 +10062,7 @@
       </x:c>
       <x:c r="N116" s="42"/>
       <x:c r="O116" s="42" t="str">
-        <x:v>2001317-2||الفقه3</x:v>
+        <x:v>20024101-2||قاعةبحث</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="34" customHeight="1">
@@ -10049,22 +10082,22 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="F117" s="43" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G117" s="43" t="str">
+        <x:v>2002266-5</x:v>
+      </x:c>
+      <x:c r="H117" s="42" t="str">
+        <x:v>التدريب التعاوني</x:v>
+      </x:c>
+      <x:c r="I117" s="43" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G117" s="43" t="str">
-        <x:v>2004320-2</x:v>
-      </x:c>
-      <x:c r="H117" s="42" t="str">
-        <x:v>الحديث (3)</x:v>
-      </x:c>
-      <x:c r="I117" s="43" t="n">
-        <x:v>2</x:v>
-      </x:c>
       <x:c r="J117" s="42" t="str">
-        <x:v>نظري</x:v>
+        <x:v>تدريب</x:v>
       </x:c>
       <x:c r="K117" s="42" t="str">
-        <x:v>متطلبات الكلية</x:v>
+        <x:v>إجبارية القسم</x:v>
       </x:c>
       <x:c r="L117" s="42" t="str">
         <x:v>القرآن وعلومه 47.pdf</x:v>
@@ -10074,7 +10107,7 @@
       </x:c>
       <x:c r="N117" s="42"/>
       <x:c r="O117" s="42" t="str">
-        <x:v>2004320-2||الحديث3</x:v>
+        <x:v>2002266-5||التدريبالتعاوني</x:v>
       </x:c>
     </x:row>
     <x:row r="118" ht="34" customHeight="1">
@@ -10088,19 +10121,19 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="D118" s="42" t="str">
-        <x:v>جديدة</x:v>
+        <x:v>قديمة</x:v>
       </x:c>
       <x:c r="E118" s="43" t="n">
-        <x:v>47</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="F118" s="43" t="n">
-        <x:v>6</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G118" s="43" t="str">
-        <x:v>2001330-2</x:v>
+        <x:v>2001160-2</x:v>
       </x:c>
       <x:c r="H118" s="42" t="str">
-        <x:v>أصول الفقه (2)</x:v>
+        <x:v>المدخل لدراسة الشريعة</x:v>
       </x:c>
       <x:c r="I118" s="43" t="n">
         <x:v>2</x:v>
@@ -10112,14 +10145,14 @@
         <x:v>إجبارية القسم</x:v>
       </x:c>
       <x:c r="L118" s="42" t="str">
-        <x:v>القرآن وعلومه 47.pdf</x:v>
+        <x:v>القرآن وعلومه 39.pdf</x:v>
       </x:c>
       <x:c r="M118" s="42" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
       </x:c>
       <x:c r="N118" s="42"/>
       <x:c r="O118" s="42" t="str">
-        <x:v>2001330-2||اصولالفقه2</x:v>
+        <x:v>2001160-2||المدخللدراسةالشريعة</x:v>
       </x:c>
     </x:row>
     <x:row r="119" ht="34" customHeight="1">
@@ -10133,19 +10166,19 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="D119" s="42" t="str">
-        <x:v>جديدة</x:v>
+        <x:v>قديمة</x:v>
       </x:c>
       <x:c r="E119" s="43" t="n">
-        <x:v>47</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="F119" s="43" t="n">
-        <x:v>7</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G119" s="43" t="str">
-        <x:v>2004403-2</x:v>
+        <x:v>101221-2</x:v>
       </x:c>
       <x:c r="H119" s="42" t="str">
-        <x:v>الأديان والفرق والمذاهب المعاصرة</x:v>
+        <x:v>الفقه (1)</x:v>
       </x:c>
       <x:c r="I119" s="43" t="n">
         <x:v>2</x:v>
@@ -10154,17 +10187,17 @@
         <x:v>نظري</x:v>
       </x:c>
       <x:c r="K119" s="42" t="str">
-        <x:v>متطلبات الكلية</x:v>
+        <x:v>إجبارية القسم</x:v>
       </x:c>
       <x:c r="L119" s="42" t="str">
-        <x:v>القرآن وعلومه 47.pdf</x:v>
+        <x:v>القرآن وعلومه 39.pdf</x:v>
       </x:c>
       <x:c r="M119" s="42" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
       </x:c>
       <x:c r="N119" s="42"/>
       <x:c r="O119" s="42" t="str">
-        <x:v>2004403-2||الاديانوالفرقوالمذاهبالمعاصرة</x:v>
+        <x:v>101221-2||الفقه1</x:v>
       </x:c>
     </x:row>
     <x:row r="120" ht="34" customHeight="1">
@@ -10178,19 +10211,19 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="D120" s="42" t="str">
-        <x:v>جديدة</x:v>
+        <x:v>قديمة</x:v>
       </x:c>
       <x:c r="E120" s="43" t="n">
-        <x:v>47</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="F120" s="43" t="n">
-        <x:v>7</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G120" s="43" t="str">
-        <x:v>20024101-2</x:v>
+        <x:v>2003220-2</x:v>
       </x:c>
       <x:c r="H120" s="42" t="str">
-        <x:v>قاعة بحث</x:v>
+        <x:v>المدخل لدراسة الأنظمة</x:v>
       </x:c>
       <x:c r="I120" s="43" t="n">
         <x:v>2</x:v>
@@ -10202,14 +10235,14 @@
         <x:v>إجبارية القسم</x:v>
       </x:c>
       <x:c r="L120" s="42" t="str">
-        <x:v>القرآن وعلومه 47.pdf</x:v>
+        <x:v>القرآن وعلومه 39.pdf</x:v>
       </x:c>
       <x:c r="M120" s="42" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
       </x:c>
       <x:c r="N120" s="42"/>
       <x:c r="O120" s="42" t="str">
-        <x:v>20024101-2||قاعةبحث</x:v>
+        <x:v>2003220-2||المدخللدراسةالانظمة</x:v>
       </x:c>
     </x:row>
     <x:row r="121" ht="34" customHeight="1">
@@ -10223,38 +10256,38 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="D121" s="42" t="str">
-        <x:v>جديدة</x:v>
+        <x:v>قديمة</x:v>
       </x:c>
       <x:c r="E121" s="43" t="n">
-        <x:v>47</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="F121" s="43" t="n">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G121" s="43" t="str">
-        <x:v>2002266-5</x:v>
+        <x:v>2001113-2</x:v>
       </x:c>
       <x:c r="H121" s="42" t="str">
-        <x:v>التدريب التعاوني</x:v>
+        <x:v>أصول الفقه (1)</x:v>
       </x:c>
       <x:c r="I121" s="43" t="n">
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J121" s="42" t="str">
-        <x:v>تدريب</x:v>
+        <x:v>نظري</x:v>
       </x:c>
       <x:c r="K121" s="42" t="str">
         <x:v>إجبارية القسم</x:v>
       </x:c>
       <x:c r="L121" s="42" t="str">
-        <x:v>القرآن وعلومه 47.pdf</x:v>
+        <x:v>القرآن وعلومه 39.pdf</x:v>
       </x:c>
       <x:c r="M121" s="42" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
       </x:c>
       <x:c r="N121" s="42"/>
       <x:c r="O121" s="42" t="str">
-        <x:v>2002266-5||التدريبالتعاوني</x:v>
+        <x:v>2001113-2||اصولالفقه1</x:v>
       </x:c>
     </x:row>
     <x:row r="122" ht="34" customHeight="1">
@@ -10274,13 +10307,13 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="F122" s="43" t="n">
-        <x:v>1</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G122" s="43" t="str">
-        <x:v>2001160-2</x:v>
+        <x:v>2001424-2</x:v>
       </x:c>
       <x:c r="H122" s="42" t="str">
-        <x:v>المدخل لدراسة الشريعة</x:v>
+        <x:v>الفقه (4)</x:v>
       </x:c>
       <x:c r="I122" s="43" t="n">
         <x:v>2</x:v>
@@ -10299,7 +10332,7 @@
       </x:c>
       <x:c r="N122" s="42"/>
       <x:c r="O122" s="42" t="str">
-        <x:v>2001160-2||المدخللدراسةالشريعة</x:v>
+        <x:v>2001424-2||الفقه4</x:v>
       </x:c>
     </x:row>
     <x:row r="123" ht="34" customHeight="1">
@@ -10307,25 +10340,25 @@
         <x:v>118</x:v>
       </x:c>
       <x:c r="B123" s="42" t="str">
-        <x:v>القرآن وعلومه</x:v>
+        <x:v>أصول الفقه</x:v>
       </x:c>
       <x:c r="C123" s="42" t="str">
-        <x:v>بكالوريوس</x:v>
+        <x:v>دكتوراه</x:v>
       </x:c>
       <x:c r="D123" s="42" t="str">
-        <x:v>قديمة</x:v>
+        <x:v>جديدة</x:v>
       </x:c>
       <x:c r="E123" s="43" t="n">
-        <x:v>39</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F123" s="43" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G123" s="43" t="str">
-        <x:v>101221-2</x:v>
+        <x:v>2001901-2</x:v>
       </x:c>
       <x:c r="H123" s="42" t="str">
-        <x:v>الفقه (1)</x:v>
+        <x:v>دراسات مقاصدية</x:v>
       </x:c>
       <x:c r="I123" s="43" t="n">
         <x:v>2</x:v>
@@ -10337,14 +10370,14 @@
         <x:v>إجبارية القسم</x:v>
       </x:c>
       <x:c r="L123" s="42" t="str">
-        <x:v>القرآن وعلومه 39.pdf</x:v>
+        <x:v>الدكتوراه في أصول الفقه.pdf</x:v>
       </x:c>
       <x:c r="M123" s="42" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
       </x:c>
       <x:c r="N123" s="42"/>
       <x:c r="O123" s="42" t="str">
-        <x:v>101221-2||الفقه1</x:v>
+        <x:v>2001901-2||دراساتمقاصدية</x:v>
       </x:c>
     </x:row>
     <x:row r="124" ht="34" customHeight="1">
@@ -10352,28 +10385,28 @@
         <x:v>119</x:v>
       </x:c>
       <x:c r="B124" s="42" t="str">
-        <x:v>القرآن وعلومه</x:v>
+        <x:v>أصول الفقه</x:v>
       </x:c>
       <x:c r="C124" s="42" t="str">
-        <x:v>بكالوريوس</x:v>
+        <x:v>دكتوراه</x:v>
       </x:c>
       <x:c r="D124" s="42" t="str">
-        <x:v>قديمة</x:v>
+        <x:v>جديدة</x:v>
       </x:c>
       <x:c r="E124" s="43" t="n">
-        <x:v>39</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F124" s="43" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G124" s="43" t="str">
+        <x:v>2001902-3</x:v>
+      </x:c>
+      <x:c r="H124" s="42" t="str">
+        <x:v>دراسة تحليلية أصولية</x:v>
+      </x:c>
+      <x:c r="I124" s="43" t="n">
         <x:v>3</x:v>
-      </x:c>
-      <x:c r="G124" s="43" t="str">
-        <x:v>2001205-2</x:v>
-      </x:c>
-      <x:c r="H124" s="42" t="str">
-        <x:v>الحديث (1)</x:v>
-      </x:c>
-      <x:c r="I124" s="43" t="n">
-        <x:v>2</x:v>
       </x:c>
       <x:c r="J124" s="42" t="str">
         <x:v>نظري</x:v>
@@ -10382,14 +10415,14 @@
         <x:v>إجبارية القسم</x:v>
       </x:c>
       <x:c r="L124" s="42" t="str">
-        <x:v>القرآن وعلومه 39.pdf</x:v>
+        <x:v>الدكتوراه في أصول الفقه.pdf</x:v>
       </x:c>
       <x:c r="M124" s="42" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
       </x:c>
       <x:c r="N124" s="42"/>
       <x:c r="O124" s="42" t="str">
-        <x:v>2001205-2||الحديث1</x:v>
+        <x:v>2001902-3||دراسةتحليليةاصولية</x:v>
       </x:c>
     </x:row>
     <x:row r="125" ht="34" customHeight="1">
@@ -10397,28 +10430,28 @@
         <x:v>120</x:v>
       </x:c>
       <x:c r="B125" s="42" t="str">
-        <x:v>القرآن وعلومه</x:v>
+        <x:v>أصول الفقه</x:v>
       </x:c>
       <x:c r="C125" s="42" t="str">
-        <x:v>بكالوريوس</x:v>
+        <x:v>دكتوراه</x:v>
       </x:c>
       <x:c r="D125" s="42" t="str">
-        <x:v>قديمة</x:v>
+        <x:v>جديدة</x:v>
       </x:c>
       <x:c r="E125" s="43" t="n">
-        <x:v>39</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F125" s="43" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G125" s="43" t="str">
+        <x:v>2001903-4</x:v>
+      </x:c>
+      <x:c r="H125" s="42" t="str">
+        <x:v>الاجتهاد الاستدلالي والفتوى</x:v>
+      </x:c>
+      <x:c r="I125" s="43" t="n">
         <x:v>4</x:v>
-      </x:c>
-      <x:c r="G125" s="43" t="str">
-        <x:v>2001209-2</x:v>
-      </x:c>
-      <x:c r="H125" s="42" t="str">
-        <x:v>الحديث (2)</x:v>
-      </x:c>
-      <x:c r="I125" s="43" t="n">
-        <x:v>2</x:v>
       </x:c>
       <x:c r="J125" s="42" t="str">
         <x:v>نظري</x:v>
@@ -10427,14 +10460,14 @@
         <x:v>إجبارية القسم</x:v>
       </x:c>
       <x:c r="L125" s="42" t="str">
-        <x:v>القرآن وعلومه 39.pdf</x:v>
+        <x:v>الدكتوراه في أصول الفقه.pdf</x:v>
       </x:c>
       <x:c r="M125" s="42" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
       </x:c>
       <x:c r="N125" s="42"/>
       <x:c r="O125" s="42" t="str">
-        <x:v>2001209-2||الحديث2</x:v>
+        <x:v>2001903-4||الاجتهادالاستدلاليوالفتوي</x:v>
       </x:c>
     </x:row>
     <x:row r="126" ht="34" customHeight="1">
@@ -10442,25 +10475,25 @@
         <x:v>121</x:v>
       </x:c>
       <x:c r="B126" s="42" t="str">
-        <x:v>القرآن وعلومه</x:v>
+        <x:v>الفقه</x:v>
       </x:c>
       <x:c r="C126" s="42" t="str">
-        <x:v>بكالوريوس</x:v>
+        <x:v>ماجستير</x:v>
       </x:c>
       <x:c r="D126" s="42" t="str">
-        <x:v>قديمة</x:v>
+        <x:v>جديدة</x:v>
       </x:c>
       <x:c r="E126" s="43" t="n">
-        <x:v>39</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F126" s="43" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G126" s="43" t="str">
-        <x:v>2001322-2</x:v>
+        <x:v>2003880-2</x:v>
       </x:c>
       <x:c r="H126" s="42" t="str">
-        <x:v>الفقه (2)</x:v>
+        <x:v>الأنظمة العدلية في السعودية</x:v>
       </x:c>
       <x:c r="I126" s="43" t="n">
         <x:v>2</x:v>
@@ -10472,465 +10505,185 @@
         <x:v>إجبارية القسم</x:v>
       </x:c>
       <x:c r="L126" s="42" t="str">
-        <x:v>القرآن وعلومه 39.pdf</x:v>
+        <x:v>الماجستير في الفقه.pdf</x:v>
       </x:c>
       <x:c r="M126" s="42" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
       </x:c>
       <x:c r="N126" s="42"/>
       <x:c r="O126" s="42" t="str">
-        <x:v>2001322-2||الفقه2</x:v>
+        <x:v>2003880-2||الانظمةالعدليةفيالسعودية</x:v>
       </x:c>
     </x:row>
     <x:row r="127" ht="34" customHeight="1">
-      <x:c r="A127" s="33" t="n">
-        <x:v>122</x:v>
-      </x:c>
-      <x:c r="B127" s="42" t="str">
-        <x:v>القرآن وعلومه</x:v>
-      </x:c>
-      <x:c r="C127" s="42" t="str">
-        <x:v>بكالوريوس</x:v>
-      </x:c>
-      <x:c r="D127" s="42" t="str">
-        <x:v>قديمة</x:v>
-      </x:c>
-      <x:c r="E127" s="43" t="n">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="F127" s="43" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="G127" s="43" t="str">
-        <x:v>2003220-2</x:v>
-      </x:c>
-      <x:c r="H127" s="42" t="str">
-        <x:v>المدخل لدراسة الأنظمة</x:v>
-      </x:c>
-      <x:c r="I127" s="43" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="J127" s="42" t="str">
-        <x:v>نظري</x:v>
-      </x:c>
-      <x:c r="K127" s="42" t="str">
-        <x:v>إجبارية القسم</x:v>
-      </x:c>
-      <x:c r="L127" s="42" t="str">
-        <x:v>القرآن وعلومه 39.pdf</x:v>
-      </x:c>
-      <x:c r="M127" s="42" t="str">
-        <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
-      </x:c>
+      <x:c r="A127" s="33"/>
+      <x:c r="B127" s="42"/>
+      <x:c r="C127" s="42"/>
+      <x:c r="D127" s="42"/>
+      <x:c r="E127" s="43"/>
+      <x:c r="F127" s="43"/>
+      <x:c r="G127" s="43"/>
+      <x:c r="H127" s="42"/>
+      <x:c r="I127" s="43"/>
+      <x:c r="J127" s="42"/>
+      <x:c r="K127" s="42"/>
+      <x:c r="L127" s="42"/>
+      <x:c r="M127" s="42"/>
       <x:c r="N127" s="42"/>
-      <x:c r="O127" s="42" t="str">
-        <x:v>2003220-2||المدخللدراسةالانظمة</x:v>
-      </x:c>
+      <x:c r="O127" s="42"/>
     </x:row>
     <x:row r="128" ht="34" customHeight="1">
-      <x:c r="A128" s="33" t="n">
-        <x:v>123</x:v>
-      </x:c>
-      <x:c r="B128" s="42" t="str">
-        <x:v>القرآن وعلومه</x:v>
-      </x:c>
-      <x:c r="C128" s="42" t="str">
-        <x:v>بكالوريوس</x:v>
-      </x:c>
-      <x:c r="D128" s="42" t="str">
-        <x:v>قديمة</x:v>
-      </x:c>
-      <x:c r="E128" s="43" t="n">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="F128" s="43" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="G128" s="43" t="str">
-        <x:v>2001113-2</x:v>
-      </x:c>
-      <x:c r="H128" s="42" t="str">
-        <x:v>أصول الفقه (1)</x:v>
-      </x:c>
-      <x:c r="I128" s="43" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="J128" s="42" t="str">
-        <x:v>نظري</x:v>
-      </x:c>
-      <x:c r="K128" s="42" t="str">
-        <x:v>إجبارية القسم</x:v>
-      </x:c>
-      <x:c r="L128" s="42" t="str">
-        <x:v>القرآن وعلومه 39.pdf</x:v>
-      </x:c>
-      <x:c r="M128" s="42" t="str">
-        <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
-      </x:c>
+      <x:c r="A128" s="33"/>
+      <x:c r="B128" s="42"/>
+      <x:c r="C128" s="42"/>
+      <x:c r="D128" s="42"/>
+      <x:c r="E128" s="43"/>
+      <x:c r="F128" s="43"/>
+      <x:c r="G128" s="43"/>
+      <x:c r="H128" s="42"/>
+      <x:c r="I128" s="43"/>
+      <x:c r="J128" s="42"/>
+      <x:c r="K128" s="42"/>
+      <x:c r="L128" s="42"/>
+      <x:c r="M128" s="42"/>
       <x:c r="N128" s="42"/>
-      <x:c r="O128" s="42" t="str">
-        <x:v>2001113-2||اصولالفقه1</x:v>
-      </x:c>
+      <x:c r="O128" s="42"/>
     </x:row>
     <x:row r="129" ht="34" customHeight="1">
-      <x:c r="A129" s="33" t="n">
-        <x:v>124</x:v>
-      </x:c>
-      <x:c r="B129" s="42" t="str">
-        <x:v>القرآن وعلومه</x:v>
-      </x:c>
-      <x:c r="C129" s="42" t="str">
-        <x:v>بكالوريوس</x:v>
-      </x:c>
-      <x:c r="D129" s="42" t="str">
-        <x:v>قديمة</x:v>
-      </x:c>
-      <x:c r="E129" s="43" t="n">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="F129" s="43" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="G129" s="43" t="str">
-        <x:v>2001317-2</x:v>
-      </x:c>
-      <x:c r="H129" s="42" t="str">
-        <x:v>الفقه (3)</x:v>
-      </x:c>
-      <x:c r="I129" s="43" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="J129" s="42" t="str">
-        <x:v>نظري</x:v>
-      </x:c>
-      <x:c r="K129" s="42" t="str">
-        <x:v>إجبارية القسم</x:v>
-      </x:c>
-      <x:c r="L129" s="42" t="str">
-        <x:v>القرآن وعلومه 39.pdf</x:v>
-      </x:c>
-      <x:c r="M129" s="42" t="str">
-        <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
-      </x:c>
+      <x:c r="A129" s="33"/>
+      <x:c r="B129" s="42"/>
+      <x:c r="C129" s="42"/>
+      <x:c r="D129" s="42"/>
+      <x:c r="E129" s="43"/>
+      <x:c r="F129" s="43"/>
+      <x:c r="G129" s="43"/>
+      <x:c r="H129" s="42"/>
+      <x:c r="I129" s="43"/>
+      <x:c r="J129" s="42"/>
+      <x:c r="K129" s="42"/>
+      <x:c r="L129" s="42"/>
+      <x:c r="M129" s="42"/>
       <x:c r="N129" s="42"/>
-      <x:c r="O129" s="42" t="str">
-        <x:v>2001317-2||الفقه3</x:v>
-      </x:c>
+      <x:c r="O129" s="42"/>
     </x:row>
     <x:row r="130" ht="34" customHeight="1">
-      <x:c r="A130" s="33" t="n">
-        <x:v>125</x:v>
-      </x:c>
-      <x:c r="B130" s="42" t="str">
-        <x:v>القرآن وعلومه</x:v>
-      </x:c>
-      <x:c r="C130" s="42" t="str">
-        <x:v>بكالوريوس</x:v>
-      </x:c>
-      <x:c r="D130" s="42" t="str">
-        <x:v>قديمة</x:v>
-      </x:c>
-      <x:c r="E130" s="43" t="n">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="F130" s="43" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="G130" s="43" t="str">
-        <x:v>2001320-2</x:v>
-      </x:c>
-      <x:c r="H130" s="42" t="str">
-        <x:v>الحديث (3)</x:v>
-      </x:c>
-      <x:c r="I130" s="43" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="J130" s="42" t="str">
-        <x:v>نظري</x:v>
-      </x:c>
-      <x:c r="K130" s="42" t="str">
-        <x:v>إجبارية القسم</x:v>
-      </x:c>
-      <x:c r="L130" s="42" t="str">
-        <x:v>القرآن وعلومه 39.pdf</x:v>
-      </x:c>
-      <x:c r="M130" s="42" t="str">
-        <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
-      </x:c>
+      <x:c r="A130" s="33"/>
+      <x:c r="B130" s="42"/>
+      <x:c r="C130" s="42"/>
+      <x:c r="D130" s="42"/>
+      <x:c r="E130" s="43"/>
+      <x:c r="F130" s="43"/>
+      <x:c r="G130" s="43"/>
+      <x:c r="H130" s="42"/>
+      <x:c r="I130" s="43"/>
+      <x:c r="J130" s="42"/>
+      <x:c r="K130" s="42"/>
+      <x:c r="L130" s="42"/>
+      <x:c r="M130" s="42"/>
       <x:c r="N130" s="42"/>
-      <x:c r="O130" s="42" t="str">
-        <x:v>2001320-2||الحديث3</x:v>
-      </x:c>
+      <x:c r="O130" s="42"/>
     </x:row>
     <x:row r="131" ht="34" customHeight="1">
-      <x:c r="A131" s="33" t="n">
-        <x:v>126</x:v>
-      </x:c>
-      <x:c r="B131" s="42" t="str">
-        <x:v>القرآن وعلومه</x:v>
-      </x:c>
-      <x:c r="C131" s="42" t="str">
-        <x:v>بكالوريوس</x:v>
-      </x:c>
-      <x:c r="D131" s="42" t="str">
-        <x:v>قديمة</x:v>
-      </x:c>
-      <x:c r="E131" s="43" t="n">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="F131" s="43" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="G131" s="43" t="str">
-        <x:v>2001330-2</x:v>
-      </x:c>
-      <x:c r="H131" s="42" t="str">
-        <x:v>أصول الفقه (2)</x:v>
-      </x:c>
-      <x:c r="I131" s="43" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="J131" s="42" t="str">
-        <x:v>نظري</x:v>
-      </x:c>
-      <x:c r="K131" s="42" t="str">
-        <x:v>إجبارية القسم</x:v>
-      </x:c>
-      <x:c r="L131" s="42" t="str">
-        <x:v>القرآن وعلومه 39.pdf</x:v>
-      </x:c>
-      <x:c r="M131" s="42" t="str">
-        <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
-      </x:c>
+      <x:c r="A131" s="33"/>
+      <x:c r="B131" s="42"/>
+      <x:c r="C131" s="42"/>
+      <x:c r="D131" s="42"/>
+      <x:c r="E131" s="43"/>
+      <x:c r="F131" s="43"/>
+      <x:c r="G131" s="43"/>
+      <x:c r="H131" s="42"/>
+      <x:c r="I131" s="43"/>
+      <x:c r="J131" s="42"/>
+      <x:c r="K131" s="42"/>
+      <x:c r="L131" s="42"/>
+      <x:c r="M131" s="42"/>
       <x:c r="N131" s="42"/>
-      <x:c r="O131" s="42" t="str">
-        <x:v>2001330-2||اصولالفقه2</x:v>
-      </x:c>
+      <x:c r="O131" s="42"/>
     </x:row>
     <x:row r="132" ht="34" customHeight="1">
-      <x:c r="A132" s="33" t="n">
-        <x:v>127</x:v>
-      </x:c>
-      <x:c r="B132" s="42" t="str">
-        <x:v>القرآن وعلومه</x:v>
-      </x:c>
-      <x:c r="C132" s="42" t="str">
-        <x:v>بكالوريوس</x:v>
-      </x:c>
-      <x:c r="D132" s="42" t="str">
-        <x:v>قديمة</x:v>
-      </x:c>
-      <x:c r="E132" s="43" t="n">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="F132" s="43" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="G132" s="43" t="str">
-        <x:v>2001424-2</x:v>
-      </x:c>
-      <x:c r="H132" s="42" t="str">
-        <x:v>الفقه (4)</x:v>
-      </x:c>
-      <x:c r="I132" s="43" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="J132" s="42" t="str">
-        <x:v>نظري</x:v>
-      </x:c>
-      <x:c r="K132" s="42" t="str">
-        <x:v>إجبارية القسم</x:v>
-      </x:c>
-      <x:c r="L132" s="42" t="str">
-        <x:v>القرآن وعلومه 39.pdf</x:v>
-      </x:c>
-      <x:c r="M132" s="42" t="str">
-        <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
-      </x:c>
+      <x:c r="A132" s="33"/>
+      <x:c r="B132" s="42"/>
+      <x:c r="C132" s="42"/>
+      <x:c r="D132" s="42"/>
+      <x:c r="E132" s="43"/>
+      <x:c r="F132" s="43"/>
+      <x:c r="G132" s="43"/>
+      <x:c r="H132" s="42"/>
+      <x:c r="I132" s="43"/>
+      <x:c r="J132" s="42"/>
+      <x:c r="K132" s="42"/>
+      <x:c r="L132" s="42"/>
+      <x:c r="M132" s="42"/>
       <x:c r="N132" s="42"/>
-      <x:c r="O132" s="42" t="str">
-        <x:v>2001424-2||الفقه4</x:v>
-      </x:c>
+      <x:c r="O132" s="42"/>
     </x:row>
     <x:row r="133" ht="34" customHeight="1">
-      <x:c r="A133" s="33" t="n">
-        <x:v>128</x:v>
-      </x:c>
-      <x:c r="B133" s="42" t="str">
-        <x:v>أصول الفقه</x:v>
-      </x:c>
-      <x:c r="C133" s="42" t="str">
-        <x:v>دكتوراه</x:v>
-      </x:c>
-      <x:c r="D133" s="42" t="str">
-        <x:v>جديدة</x:v>
-      </x:c>
-      <x:c r="E133" s="43" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F133" s="43" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G133" s="43" t="str">
-        <x:v>2001901-2</x:v>
-      </x:c>
-      <x:c r="H133" s="42" t="str">
-        <x:v>دراسات مقاصدية</x:v>
-      </x:c>
-      <x:c r="I133" s="43" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="J133" s="42" t="str">
-        <x:v>نظري</x:v>
-      </x:c>
-      <x:c r="K133" s="42" t="str">
-        <x:v>إجبارية القسم</x:v>
-      </x:c>
-      <x:c r="L133" s="42" t="str">
-        <x:v>الدكتوراه في أصول الفقه.pdf</x:v>
-      </x:c>
-      <x:c r="M133" s="42" t="str">
-        <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
-      </x:c>
+      <x:c r="A133" s="33"/>
+      <x:c r="B133" s="42"/>
+      <x:c r="C133" s="42"/>
+      <x:c r="D133" s="42"/>
+      <x:c r="E133" s="43"/>
+      <x:c r="F133" s="43"/>
+      <x:c r="G133" s="43"/>
+      <x:c r="H133" s="42"/>
+      <x:c r="I133" s="43"/>
+      <x:c r="J133" s="42"/>
+      <x:c r="K133" s="42"/>
+      <x:c r="L133" s="42"/>
+      <x:c r="M133" s="42"/>
       <x:c r="N133" s="42"/>
-      <x:c r="O133" s="42" t="str">
-        <x:v>2001901-2||دراساتمقاصدية</x:v>
-      </x:c>
+      <x:c r="O133" s="42"/>
     </x:row>
     <x:row r="134" ht="34" customHeight="1">
-      <x:c r="A134" s="33" t="n">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="B134" s="42" t="str">
-        <x:v>أصول الفقه</x:v>
-      </x:c>
-      <x:c r="C134" s="42" t="str">
-        <x:v>دكتوراه</x:v>
-      </x:c>
-      <x:c r="D134" s="42" t="str">
-        <x:v>جديدة</x:v>
-      </x:c>
-      <x:c r="E134" s="43" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F134" s="43" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G134" s="43" t="str">
-        <x:v>2001902-3</x:v>
-      </x:c>
-      <x:c r="H134" s="42" t="str">
-        <x:v>دراسة تحليلية أصولية</x:v>
-      </x:c>
-      <x:c r="I134" s="43" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="J134" s="42" t="str">
-        <x:v>نظري</x:v>
-      </x:c>
-      <x:c r="K134" s="42" t="str">
-        <x:v>إجبارية القسم</x:v>
-      </x:c>
-      <x:c r="L134" s="42" t="str">
-        <x:v>الدكتوراه في أصول الفقه.pdf</x:v>
-      </x:c>
-      <x:c r="M134" s="42" t="str">
-        <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
-      </x:c>
+      <x:c r="A134" s="33"/>
+      <x:c r="B134" s="42"/>
+      <x:c r="C134" s="42"/>
+      <x:c r="D134" s="42"/>
+      <x:c r="E134" s="43"/>
+      <x:c r="F134" s="43"/>
+      <x:c r="G134" s="43"/>
+      <x:c r="H134" s="42"/>
+      <x:c r="I134" s="43"/>
+      <x:c r="J134" s="42"/>
+      <x:c r="K134" s="42"/>
+      <x:c r="L134" s="42"/>
+      <x:c r="M134" s="42"/>
       <x:c r="N134" s="42"/>
-      <x:c r="O134" s="42" t="str">
-        <x:v>2001902-3||دراسةتحليليةاصولية</x:v>
-      </x:c>
+      <x:c r="O134" s="42"/>
     </x:row>
     <x:row r="135" ht="34" customHeight="1">
-      <x:c r="A135" s="33" t="n">
-        <x:v>130</x:v>
-      </x:c>
-      <x:c r="B135" s="42" t="str">
-        <x:v>أصول الفقه</x:v>
-      </x:c>
-      <x:c r="C135" s="42" t="str">
-        <x:v>دكتوراه</x:v>
-      </x:c>
-      <x:c r="D135" s="42" t="str">
-        <x:v>جديدة</x:v>
-      </x:c>
-      <x:c r="E135" s="43" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F135" s="43" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G135" s="43" t="str">
-        <x:v>2001903-4</x:v>
-      </x:c>
-      <x:c r="H135" s="42" t="str">
-        <x:v>الاجتهاد الاستدلالي والفتوى</x:v>
-      </x:c>
-      <x:c r="I135" s="43" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="J135" s="42" t="str">
-        <x:v>نظري</x:v>
-      </x:c>
-      <x:c r="K135" s="42" t="str">
-        <x:v>إجبارية القسم</x:v>
-      </x:c>
-      <x:c r="L135" s="42" t="str">
-        <x:v>الدكتوراه في أصول الفقه.pdf</x:v>
-      </x:c>
-      <x:c r="M135" s="42" t="str">
-        <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
-      </x:c>
+      <x:c r="A135" s="33"/>
+      <x:c r="B135" s="42"/>
+      <x:c r="C135" s="42"/>
+      <x:c r="D135" s="42"/>
+      <x:c r="E135" s="43"/>
+      <x:c r="F135" s="43"/>
+      <x:c r="G135" s="43"/>
+      <x:c r="H135" s="42"/>
+      <x:c r="I135" s="43"/>
+      <x:c r="J135" s="42"/>
+      <x:c r="K135" s="42"/>
+      <x:c r="L135" s="42"/>
+      <x:c r="M135" s="42"/>
       <x:c r="N135" s="42"/>
-      <x:c r="O135" s="42" t="str">
-        <x:v>2001903-4||الاجتهادالاستدلاليوالفتوي</x:v>
-      </x:c>
+      <x:c r="O135" s="42"/>
     </x:row>
     <x:row r="136" ht="34" customHeight="1">
-      <x:c r="A136" s="33" t="n">
-        <x:v>131</x:v>
-      </x:c>
-      <x:c r="B136" s="42" t="str">
-        <x:v>الفقه</x:v>
-      </x:c>
-      <x:c r="C136" s="42" t="str">
-        <x:v>ماجستير</x:v>
-      </x:c>
-      <x:c r="D136" s="42" t="str">
-        <x:v>جديدة</x:v>
-      </x:c>
-      <x:c r="E136" s="43" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F136" s="43" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="G136" s="43" t="str">
-        <x:v>2003880-2</x:v>
-      </x:c>
-      <x:c r="H136" s="42" t="str">
-        <x:v>الأنظمة العدلية في السعودية</x:v>
-      </x:c>
-      <x:c r="I136" s="43" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="J136" s="42" t="str">
-        <x:v>نظري</x:v>
-      </x:c>
-      <x:c r="K136" s="42" t="str">
-        <x:v>إجبارية القسم</x:v>
-      </x:c>
-      <x:c r="L136" s="42" t="str">
-        <x:v>الماجستير في الفقه.pdf</x:v>
-      </x:c>
-      <x:c r="M136" s="42" t="str">
-        <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
-      </x:c>
+      <x:c r="A136" s="33"/>
+      <x:c r="B136" s="42"/>
+      <x:c r="C136" s="42"/>
+      <x:c r="D136" s="42"/>
+      <x:c r="E136" s="43"/>
+      <x:c r="F136" s="43"/>
+      <x:c r="G136" s="43"/>
+      <x:c r="H136" s="42"/>
+      <x:c r="I136" s="43"/>
+      <x:c r="J136" s="42"/>
+      <x:c r="K136" s="42"/>
+      <x:c r="L136" s="42"/>
+      <x:c r="M136" s="42"/>
       <x:c r="N136" s="42"/>
-      <x:c r="O136" s="42" t="str">
-        <x:v>2003880-2||الانظمةالعدليةفيالسعودية</x:v>
-      </x:c>
+      <x:c r="O136" s="42"/>
     </x:row>
     <x:row r="137" ht="34" customHeight="1">
       <x:c r="A137" s="33"/>
@@ -11092,7 +10845,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb91c256e77a4ec1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfdaa02b0899b47fb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish Islamic studies takhrij course specification
</commit_message>
<xml_diff>
--- a/قائمة_المقررات_التخصصية_المفقودة_2026-09-10.xlsx
+++ b/قائمة_المقررات_التخصصية_المفقودة_2026-09-10.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الملخص" sheetId="1" r:id="R9039e5636bad42f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="المقررات المفقودة" sheetId="2" r:id="R201105e827b64770"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="مواضع الخطط" sheetId="3" r:id="Rc05d0ea49b3a4ef9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الملخص" sheetId="1" r:id="R65f444d090ce449c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="المقررات المفقودة" sheetId="2" r:id="R49a600e8d9104a13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="مواضع الخطط" sheetId="3" r:id="R40c4a15f9b4246eb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -274,7 +274,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="MissingCourseIdentities" displayName="MissingCourseIdentities" ref="A5:L93" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="MissingCourseIdentities" displayName="MissingCourseIdentities" ref="A5:L92" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="م"/>
     <x:tableColumn id="2" name="رمز المقرر"/>
@@ -294,7 +294,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="MissingCourseOccurrences" displayName="MissingCourseOccurrences" ref="A5:O107" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="MissingCourseOccurrences" displayName="MissingCourseOccurrences" ref="A5:O106" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="15">
     <x:tableColumn id="1" name="م"/>
     <x:tableColumn id="2" name="البرنامج"/>
@@ -551,7 +551,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>المصدر: data.json في مستودع التوصيفات، بتاريخ 2026-09-15. النطاق: رموز 200* والاستثناء القديم 101221-2، دون الرسالة والاختبار الشامل أو مقررات الأقسام الخارجية.</x:v>
+        <x:v>المصدر: data.json في مستودع التوصيفات، بتاريخ 2026-09-28. النطاق: رموز 200* والاستثناء القديم 101221-2، دون الرسالة والاختبار الشامل أو مقررات الأقسام الخارجية.</x:v>
       </x:c>
       <x:c r="B3"/>
       <x:c r="C3"/>
@@ -790,16 +790,16 @@
         <x:v>127</x:v>
       </x:c>
       <x:c r="E12" s="30" t="n">
-        <x:v>103</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="F12" s="30" t="n">
-        <x:v>24</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="G12" s="36" t="n">
-        <x:v>0.8110236220472441</x:v>
+        <x:v>0.8188976377952756</x:v>
       </x:c>
       <x:c r="H12" s="30" t="n">
-        <x:v>24</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="I12" s="33" t="str">
         <x:v>يحتاج استكمال</x:v>
@@ -1047,16 +1047,16 @@
         <x:v>756</x:v>
       </x:c>
       <x:c r="E21" s="31" t="n">
-        <x:v>654</x:v>
+        <x:v>655</x:v>
       </x:c>
       <x:c r="F21" s="31" t="n">
-        <x:v>102</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="G21" s="37" t="n">
-        <x:v>0.8650793650793651</x:v>
+        <x:v>0.8664021164021164</x:v>
       </x:c>
       <x:c r="H21" s="31" t="n">
-        <x:v>88</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="I21" s="34" t="str">
         <x:v>قائمة العمل الحالية</x:v>
@@ -1133,7 +1133,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>عدد الهويات الفريدة: 88. قد يظهر المقرر نفسه في أكثر من برنامج أو خطة، وتوضح الأعمدة جميع المواضع المتأثرة.</x:v>
+        <x:v>عدد الهويات الفريدة: 87. قد يظهر المقرر نفسه في أكثر من برنامج أو خطة، وتوضح الأعمدة جميع المواضع المتأثرة.</x:v>
       </x:c>
       <x:c r="B3"/>
       <x:c r="C3"/>
@@ -2394,10 +2394,10 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="B39" s="33" t="str">
-        <x:v>2004269-4</x:v>
+        <x:v>2004272-2</x:v>
       </x:c>
       <x:c r="C39" s="39" t="str">
-        <x:v>التخريج ودراسة الأسانيد</x:v>
+        <x:v>العمل الخيري</x:v>
       </x:c>
       <x:c r="D39" s="39" t="str">
         <x:v>الدراسات الإسلامية</x:v>
@@ -2422,7 +2422,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L39" s="39" t="str">
-        <x:v>2004269-4||التخريجودراسةالاسانيد</x:v>
+        <x:v>2004272-2||العملالخيري</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="42" customHeight="1">
@@ -2430,10 +2430,10 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="B40" s="33" t="str">
-        <x:v>2004272-2</x:v>
+        <x:v>2004305-4</x:v>
       </x:c>
       <x:c r="C40" s="39" t="str">
-        <x:v>العمل الخيري</x:v>
+        <x:v>أحاديث الأحكام (١)</x:v>
       </x:c>
       <x:c r="D40" s="39" t="str">
         <x:v>الدراسات الإسلامية</x:v>
@@ -2445,7 +2445,7 @@
         <x:v>الدراسات الإسلامية: جديدة 47</x:v>
       </x:c>
       <x:c r="G40" s="39" t="str">
-        <x:v>7</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H40" s="39" t="n">
         <x:v>1</x:v>
@@ -2458,7 +2458,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L40" s="39" t="str">
-        <x:v>2004272-2||العملالخيري</x:v>
+        <x:v>2004305-4||احاديثالاحكام١</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="42" customHeight="1">
@@ -2466,10 +2466,10 @@
         <x:v>36</x:v>
       </x:c>
       <x:c r="B41" s="33" t="str">
-        <x:v>2004305-4</x:v>
+        <x:v>20013101-3</x:v>
       </x:c>
       <x:c r="C41" s="39" t="str">
-        <x:v>أحاديث الأحكام (١)</x:v>
+        <x:v>الفقه (٤)</x:v>
       </x:c>
       <x:c r="D41" s="39" t="str">
         <x:v>الدراسات الإسلامية</x:v>
@@ -2481,7 +2481,7 @@
         <x:v>الدراسات الإسلامية: جديدة 47</x:v>
       </x:c>
       <x:c r="G41" s="39" t="str">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H41" s="39" t="n">
         <x:v>1</x:v>
@@ -2494,7 +2494,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L41" s="39" t="str">
-        <x:v>2004305-4||احاديثالاحكام١</x:v>
+        <x:v>20013101-3||الفقه٤</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="42" customHeight="1">
@@ -2502,10 +2502,10 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="B42" s="33" t="str">
-        <x:v>20013101-3</x:v>
+        <x:v>20013201-4</x:v>
       </x:c>
       <x:c r="C42" s="39" t="str">
-        <x:v>الفقه (٤)</x:v>
+        <x:v>الفقه (٥)</x:v>
       </x:c>
       <x:c r="D42" s="39" t="str">
         <x:v>الدراسات الإسلامية</x:v>
@@ -2517,7 +2517,7 @@
         <x:v>الدراسات الإسلامية: جديدة 47</x:v>
       </x:c>
       <x:c r="G42" s="39" t="str">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H42" s="39" t="n">
         <x:v>1</x:v>
@@ -2530,7 +2530,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L42" s="39" t="str">
-        <x:v>20013101-3||الفقه٤</x:v>
+        <x:v>20013201-4||الفقه٥</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="42" customHeight="1">
@@ -2538,10 +2538,10 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="B43" s="33" t="str">
-        <x:v>20013201-4</x:v>
+        <x:v>20042111-2</x:v>
       </x:c>
       <x:c r="C43" s="39" t="str">
-        <x:v>الفقه (٥)</x:v>
+        <x:v>العقيدة (٢)</x:v>
       </x:c>
       <x:c r="D43" s="39" t="str">
         <x:v>الدراسات الإسلامية</x:v>
@@ -2553,7 +2553,7 @@
         <x:v>الدراسات الإسلامية: جديدة 47</x:v>
       </x:c>
       <x:c r="G43" s="39" t="str">
-        <x:v>6</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H43" s="39" t="n">
         <x:v>1</x:v>
@@ -2566,7 +2566,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L43" s="39" t="str">
-        <x:v>20013201-4||الفقه٥</x:v>
+        <x:v>20042111-2||العقيدة٢</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="42" customHeight="1">
@@ -2574,10 +2574,10 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="B44" s="33" t="str">
-        <x:v>20042111-2</x:v>
+        <x:v>20043105-2</x:v>
       </x:c>
       <x:c r="C44" s="39" t="str">
-        <x:v>العقيدة (٢)</x:v>
+        <x:v>الفقه المقارن</x:v>
       </x:c>
       <x:c r="D44" s="39" t="str">
         <x:v>الدراسات الإسلامية</x:v>
@@ -2586,10 +2586,10 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F44" s="39" t="str">
-        <x:v>الدراسات الإسلامية: جديدة 47</x:v>
+        <x:v>الدراسات الإسلامية: قديمة 39</x:v>
       </x:c>
       <x:c r="G44" s="39" t="str">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H44" s="39" t="n">
         <x:v>1</x:v>
@@ -2602,7 +2602,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L44" s="39" t="str">
-        <x:v>20042111-2||العقيدة٢</x:v>
+        <x:v>20043105-2||الفقهالمقارن</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="42" customHeight="1">
@@ -2610,10 +2610,10 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="B45" s="33" t="str">
-        <x:v>20043105-2</x:v>
+        <x:v>20043108-2</x:v>
       </x:c>
       <x:c r="C45" s="39" t="str">
-        <x:v>الفقه المقارن</x:v>
+        <x:v>علم المواريث (1)</x:v>
       </x:c>
       <x:c r="D45" s="39" t="str">
         <x:v>الدراسات الإسلامية</x:v>
@@ -2638,7 +2638,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L45" s="39" t="str">
-        <x:v>20043105-2||الفقهالمقارن</x:v>
+        <x:v>20043108-2||علمالمواريث1</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="42" customHeight="1">
@@ -2646,10 +2646,10 @@
         <x:v>41</x:v>
       </x:c>
       <x:c r="B46" s="33" t="str">
-        <x:v>20043108-2</x:v>
+        <x:v>20043109-2</x:v>
       </x:c>
       <x:c r="C46" s="39" t="str">
-        <x:v>علم المواريث (1)</x:v>
+        <x:v>دراسات في سير السلف</x:v>
       </x:c>
       <x:c r="D46" s="39" t="str">
         <x:v>الدراسات الإسلامية</x:v>
@@ -2658,7 +2658,7 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F46" s="39" t="str">
-        <x:v>الدراسات الإسلامية: قديمة 39</x:v>
+        <x:v>الدراسات الإسلامية: جديدة 47</x:v>
       </x:c>
       <x:c r="G46" s="39" t="str">
         <x:v>5</x:v>
@@ -2674,7 +2674,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L46" s="39" t="str">
-        <x:v>20043108-2||علمالمواريث1</x:v>
+        <x:v>20043109-2||دراساتفيسيرالسلف</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="42" customHeight="1">
@@ -2682,10 +2682,10 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="B47" s="33" t="str">
-        <x:v>20043109-2</x:v>
+        <x:v>20043110-2</x:v>
       </x:c>
       <x:c r="C47" s="39" t="str">
-        <x:v>دراسات في سير السلف</x:v>
+        <x:v>محاسن الإسلام</x:v>
       </x:c>
       <x:c r="D47" s="39" t="str">
         <x:v>الدراسات الإسلامية</x:v>
@@ -2710,7 +2710,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L47" s="39" t="str">
-        <x:v>20043109-2||دراساتفيسيرالسلف</x:v>
+        <x:v>20043110-2||محاسنالاسلام</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="42" customHeight="1">
@@ -2718,10 +2718,10 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="B48" s="33" t="str">
-        <x:v>20043110-2</x:v>
+        <x:v>20043111-2</x:v>
       </x:c>
       <x:c r="C48" s="39" t="str">
-        <x:v>محاسن الإسلام</x:v>
+        <x:v>الأمن الفكري</x:v>
       </x:c>
       <x:c r="D48" s="39" t="str">
         <x:v>الدراسات الإسلامية</x:v>
@@ -2733,7 +2733,7 @@
         <x:v>الدراسات الإسلامية: جديدة 47</x:v>
       </x:c>
       <x:c r="G48" s="39" t="str">
-        <x:v>5</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="H48" s="39" t="n">
         <x:v>1</x:v>
@@ -2746,7 +2746,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L48" s="39" t="str">
-        <x:v>20043110-2||محاسنالاسلام</x:v>
+        <x:v>20043111-2||الامنالفكري</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="42" customHeight="1">
@@ -2754,10 +2754,10 @@
         <x:v>44</x:v>
       </x:c>
       <x:c r="B49" s="33" t="str">
-        <x:v>20043111-2</x:v>
+        <x:v>20043202-2</x:v>
       </x:c>
       <x:c r="C49" s="39" t="str">
-        <x:v>الأمن الفكري</x:v>
+        <x:v>القواعد الفقهية</x:v>
       </x:c>
       <x:c r="D49" s="39" t="str">
         <x:v>الدراسات الإسلامية</x:v>
@@ -2766,10 +2766,10 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F49" s="39" t="str">
-        <x:v>الدراسات الإسلامية: جديدة 47</x:v>
+        <x:v>الدراسات الإسلامية: قديمة 39</x:v>
       </x:c>
       <x:c r="G49" s="39" t="str">
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H49" s="39" t="n">
         <x:v>1</x:v>
@@ -2782,7 +2782,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L49" s="39" t="str">
-        <x:v>20043111-2||الامنالفكري</x:v>
+        <x:v>20043202-2||القواعدالفقهية</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="42" customHeight="1">
@@ -2790,10 +2790,10 @@
         <x:v>45</x:v>
       </x:c>
       <x:c r="B50" s="33" t="str">
-        <x:v>20043202-2</x:v>
+        <x:v>20044101-2</x:v>
       </x:c>
       <x:c r="C50" s="39" t="str">
-        <x:v>القواعد الفقهية</x:v>
+        <x:v>أصول فقه (3)</x:v>
       </x:c>
       <x:c r="D50" s="39" t="str">
         <x:v>الدراسات الإسلامية</x:v>
@@ -2805,7 +2805,7 @@
         <x:v>الدراسات الإسلامية: قديمة 39</x:v>
       </x:c>
       <x:c r="G50" s="39" t="str">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="H50" s="39" t="n">
         <x:v>1</x:v>
@@ -2818,7 +2818,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L50" s="39" t="str">
-        <x:v>20043202-2||القواعدالفقهية</x:v>
+        <x:v>20044101-2||اصولفقه3</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="42" customHeight="1">
@@ -2826,10 +2826,10 @@
         <x:v>46</x:v>
       </x:c>
       <x:c r="B51" s="33" t="str">
-        <x:v>20044101-2</x:v>
+        <x:v>20044206-2</x:v>
       </x:c>
       <x:c r="C51" s="39" t="str">
-        <x:v>أصول فقه (3)</x:v>
+        <x:v>علم المواريث (2)</x:v>
       </x:c>
       <x:c r="D51" s="39" t="str">
         <x:v>الدراسات الإسلامية</x:v>
@@ -2841,7 +2841,7 @@
         <x:v>الدراسات الإسلامية: قديمة 39</x:v>
       </x:c>
       <x:c r="G51" s="39" t="str">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H51" s="39" t="n">
         <x:v>1</x:v>
@@ -2854,7 +2854,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L51" s="39" t="str">
-        <x:v>20044101-2||اصولفقه3</x:v>
+        <x:v>20044206-2||علمالمواريث2</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="42" customHeight="1">
@@ -2862,10 +2862,10 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="B52" s="33" t="str">
-        <x:v>20044206-2</x:v>
+        <x:v>20044220-4</x:v>
       </x:c>
       <x:c r="C52" s="39" t="str">
-        <x:v>علم المواريث (2)</x:v>
+        <x:v>التدريب التعاوني</x:v>
       </x:c>
       <x:c r="D52" s="39" t="str">
         <x:v>الدراسات الإسلامية</x:v>
@@ -2874,7 +2874,7 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F52" s="39" t="str">
-        <x:v>الدراسات الإسلامية: قديمة 39</x:v>
+        <x:v>الدراسات الإسلامية: جديدة 47</x:v>
       </x:c>
       <x:c r="G52" s="39" t="str">
         <x:v>8</x:v>
@@ -2890,7 +2890,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L52" s="39" t="str">
-        <x:v>20044206-2||علمالمواريث2</x:v>
+        <x:v>20044220-4||التدريبالتعاوني</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="42" customHeight="1">
@@ -2898,25 +2898,26 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="B53" s="33" t="str">
-        <x:v>20044220-4</x:v>
+        <x:v>2001192-2</x:v>
       </x:c>
       <x:c r="C53" s="39" t="str">
-        <x:v>التدريب التعاوني</x:v>
+        <x:v>علوم الحديث (2)</x:v>
       </x:c>
       <x:c r="D53" s="39" t="str">
-        <x:v>الدراسات الإسلامية</x:v>
+        <x:v>الشريعة</x:v>
       </x:c>
       <x:c r="E53" s="39" t="str">
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F53" s="39" t="str">
-        <x:v>الدراسات الإسلامية: جديدة 47</x:v>
+        <x:v>الشريعة: قديمة 38
+الشريعة: قديمة 39</x:v>
       </x:c>
       <x:c r="G53" s="39" t="str">
-        <x:v>8</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H53" s="39" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I53" s="39" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
@@ -2926,7 +2927,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L53" s="39" t="str">
-        <x:v>20044220-4||التدريبالتعاوني</x:v>
+        <x:v>2001192-2||علومالحديث2</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="42" customHeight="1">
@@ -2934,10 +2935,10 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="B54" s="33" t="str">
-        <x:v>2001192-2</x:v>
+        <x:v>2001193-2</x:v>
       </x:c>
       <x:c r="C54" s="39" t="str">
-        <x:v>علوم الحديث (2)</x:v>
+        <x:v>علوم الحديث (1)</x:v>
       </x:c>
       <x:c r="D54" s="39" t="str">
         <x:v>الشريعة</x:v>
@@ -2950,7 +2951,7 @@
 الشريعة: قديمة 39</x:v>
       </x:c>
       <x:c r="G54" s="39" t="str">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H54" s="39" t="n">
         <x:v>2</x:v>
@@ -2963,7 +2964,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L54" s="39" t="str">
-        <x:v>2001192-2||علومالحديث2</x:v>
+        <x:v>2001193-2||علومالحديث1</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="42" customHeight="1">
@@ -2971,10 +2972,10 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="B55" s="33" t="str">
-        <x:v>2001193-2</x:v>
+        <x:v>2001217-4</x:v>
       </x:c>
       <x:c r="C55" s="39" t="str">
-        <x:v>علوم الحديث (1)</x:v>
+        <x:v>أدلة الأحكام الشرعية (2)</x:v>
       </x:c>
       <x:c r="D55" s="39" t="str">
         <x:v>الشريعة</x:v>
@@ -2987,7 +2988,7 @@
 الشريعة: قديمة 39</x:v>
       </x:c>
       <x:c r="G55" s="39" t="str">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H55" s="39" t="n">
         <x:v>2</x:v>
@@ -3000,7 +3001,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L55" s="39" t="str">
-        <x:v>2001193-2||علومالحديث1</x:v>
+        <x:v>2001217-4||ادلةالاحكامالشرعية2</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="42" customHeight="1">
@@ -3008,10 +3009,10 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="B56" s="33" t="str">
-        <x:v>2001217-4</x:v>
+        <x:v>2001218-2</x:v>
       </x:c>
       <x:c r="C56" s="39" t="str">
-        <x:v>أدلة الأحكام الشرعية (2)</x:v>
+        <x:v>قاعة بحث (تطبيقي)</x:v>
       </x:c>
       <x:c r="D56" s="39" t="str">
         <x:v>الشريعة</x:v>
@@ -3020,14 +3021,13 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F56" s="39" t="str">
-        <x:v>الشريعة: قديمة 38
-الشريعة: قديمة 39</x:v>
+        <x:v>الشريعة: قديمة 38</x:v>
       </x:c>
       <x:c r="G56" s="39" t="str">
         <x:v>4</x:v>
       </x:c>
       <x:c r="H56" s="39" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I56" s="39" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
@@ -3037,7 +3037,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L56" s="39" t="str">
-        <x:v>2001217-4||ادلةالاحكامالشرعية2</x:v>
+        <x:v>2001218-2||قاعةبحثتطبيقي</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="42" customHeight="1">
@@ -3045,10 +3045,10 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="B57" s="33" t="str">
-        <x:v>2001218-2</x:v>
+        <x:v>2001219-3</x:v>
       </x:c>
       <x:c r="C57" s="39" t="str">
-        <x:v>قاعة بحث (تطبيقي)</x:v>
+        <x:v>أدلة الأحكام الشرعية (1)</x:v>
       </x:c>
       <x:c r="D57" s="39" t="str">
         <x:v>الشريعة</x:v>
@@ -3057,13 +3057,14 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F57" s="39" t="str">
-        <x:v>الشريعة: قديمة 38</x:v>
+        <x:v>الشريعة: قديمة 38
+الشريعة: قديمة 39</x:v>
       </x:c>
       <x:c r="G57" s="39" t="str">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H57" s="39" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I57" s="39" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
@@ -3073,7 +3074,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L57" s="39" t="str">
-        <x:v>2001218-2||قاعةبحثتطبيقي</x:v>
+        <x:v>2001219-3||ادلةالاحكامالشرعية1</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="42" customHeight="1">
@@ -3081,10 +3082,10 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="B58" s="33" t="str">
-        <x:v>2001219-3</x:v>
+        <x:v>2001231-2</x:v>
       </x:c>
       <x:c r="C58" s="39" t="str">
-        <x:v>أدلة الأحكام الشرعية (1)</x:v>
+        <x:v>أحاديث الأحكام (1)</x:v>
       </x:c>
       <x:c r="D58" s="39" t="str">
         <x:v>الشريعة</x:v>
@@ -3110,7 +3111,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L58" s="39" t="str">
-        <x:v>2001219-3||ادلةالاحكامالشرعية1</x:v>
+        <x:v>2001231-2||احاديثالاحكام1</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="42" customHeight="1">
@@ -3118,10 +3119,10 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="B59" s="33" t="str">
-        <x:v>2001231-2</x:v>
+        <x:v>2001280-2</x:v>
       </x:c>
       <x:c r="C59" s="39" t="str">
-        <x:v>أحاديث الأحكام (1)</x:v>
+        <x:v>أصول الدعوة والحسبة</x:v>
       </x:c>
       <x:c r="D59" s="39" t="str">
         <x:v>الشريعة</x:v>
@@ -3134,7 +3135,7 @@
 الشريعة: قديمة 39</x:v>
       </x:c>
       <x:c r="G59" s="39" t="str">
-        <x:v>3</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H59" s="39" t="n">
         <x:v>2</x:v>
@@ -3147,7 +3148,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L59" s="39" t="str">
-        <x:v>2001231-2||احاديثالاحكام1</x:v>
+        <x:v>2001280-2||اصولالدعوةوالحسبة</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="42" customHeight="1">
@@ -3155,10 +3156,10 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="B60" s="33" t="str">
-        <x:v>2001280-2</x:v>
+        <x:v>2001301-2</x:v>
       </x:c>
       <x:c r="C60" s="39" t="str">
-        <x:v>أصول الدعوة والحسبة</x:v>
+        <x:v>تدوين السنة</x:v>
       </x:c>
       <x:c r="D60" s="39" t="str">
         <x:v>الشريعة</x:v>
@@ -3184,7 +3185,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L60" s="39" t="str">
-        <x:v>2001280-2||اصولالدعوةوالحسبة</x:v>
+        <x:v>2001301-2||تدوينالسنة</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="42" customHeight="1">
@@ -3192,10 +3193,10 @@
         <x:v>56</x:v>
       </x:c>
       <x:c r="B61" s="33" t="str">
-        <x:v>2001301-2</x:v>
+        <x:v>2001332-2</x:v>
       </x:c>
       <x:c r="C61" s="39" t="str">
-        <x:v>تدوين السنة</x:v>
+        <x:v>أحاديث الأحكام (2)</x:v>
       </x:c>
       <x:c r="D61" s="39" t="str">
         <x:v>الشريعة</x:v>
@@ -3208,7 +3209,7 @@
 الشريعة: قديمة 39</x:v>
       </x:c>
       <x:c r="G61" s="39" t="str">
-        <x:v>6</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H61" s="39" t="n">
         <x:v>2</x:v>
@@ -3221,7 +3222,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L61" s="39" t="str">
-        <x:v>2001301-2||تدوينالسنة</x:v>
+        <x:v>2001332-2||احاديثالاحكام2</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="42" customHeight="1">
@@ -3229,10 +3230,10 @@
         <x:v>57</x:v>
       </x:c>
       <x:c r="B62" s="33" t="str">
-        <x:v>2001332-2</x:v>
+        <x:v>2001493-2</x:v>
       </x:c>
       <x:c r="C62" s="39" t="str">
-        <x:v>أحاديث الأحكام (2)</x:v>
+        <x:v>تخريج ودراسة الأسانيد</x:v>
       </x:c>
       <x:c r="D62" s="39" t="str">
         <x:v>الشريعة</x:v>
@@ -3245,7 +3246,7 @@
 الشريعة: قديمة 39</x:v>
       </x:c>
       <x:c r="G62" s="39" t="str">
-        <x:v>4</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="H62" s="39" t="n">
         <x:v>2</x:v>
@@ -3258,7 +3259,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L62" s="39" t="str">
-        <x:v>2001332-2||احاديثالاحكام2</x:v>
+        <x:v>2001493-2||تخريجودراسةالاسانيد</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="42" customHeight="1">
@@ -3266,10 +3267,10 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="B63" s="33" t="str">
-        <x:v>2001493-2</x:v>
+        <x:v>2003243-2</x:v>
       </x:c>
       <x:c r="C63" s="39" t="str">
-        <x:v>تخريج ودراسة الأسانيد</x:v>
+        <x:v>مبادئ القانون الإداري</x:v>
       </x:c>
       <x:c r="D63" s="39" t="str">
         <x:v>الشريعة</x:v>
@@ -3278,14 +3279,13 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F63" s="39" t="str">
-        <x:v>الشريعة: قديمة 38
-الشريعة: قديمة 39</x:v>
+        <x:v>الشريعة: قديمة 38</x:v>
       </x:c>
       <x:c r="G63" s="39" t="str">
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H63" s="39" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I63" s="39" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
@@ -3295,7 +3295,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L63" s="39" t="str">
-        <x:v>2001493-2||تخريجودراسةالاسانيد</x:v>
+        <x:v>2003243-2||مباديالقانونالاداري</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="42" customHeight="1">
@@ -3303,10 +3303,10 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="B64" s="33" t="str">
-        <x:v>2003243-2</x:v>
+        <x:v>2003325-1</x:v>
       </x:c>
       <x:c r="C64" s="39" t="str">
-        <x:v>مبادئ القانون الإداري</x:v>
+        <x:v>نظام المرافعات الشرعية</x:v>
       </x:c>
       <x:c r="D64" s="39" t="str">
         <x:v>الشريعة</x:v>
@@ -3315,13 +3315,14 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F64" s="39" t="str">
-        <x:v>الشريعة: قديمة 38</x:v>
+        <x:v>الشريعة: قديمة 38
+الشريعة: قديمة 39</x:v>
       </x:c>
       <x:c r="G64" s="39" t="str">
         <x:v>6</x:v>
       </x:c>
       <x:c r="H64" s="39" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I64" s="39" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
@@ -3331,7 +3332,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L64" s="39" t="str">
-        <x:v>2003243-2||مباديالقانونالاداري</x:v>
+        <x:v>2003325-1||نظامالمرافعاتالشرعية</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="42" customHeight="1">
@@ -3339,10 +3340,10 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="B65" s="33" t="str">
-        <x:v>2003325-1</x:v>
+        <x:v>2003328-1</x:v>
       </x:c>
       <x:c r="C65" s="39" t="str">
-        <x:v>نظام المرافعات الشرعية</x:v>
+        <x:v>نظام الإجراءات الجزائية</x:v>
       </x:c>
       <x:c r="D65" s="39" t="str">
         <x:v>الشريعة</x:v>
@@ -3368,7 +3369,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L65" s="39" t="str">
-        <x:v>2003325-1||نظامالمرافعاتالشرعية</x:v>
+        <x:v>2003328-1||نظامالاجراءاتالجزايية</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="42" customHeight="1">
@@ -3376,10 +3377,10 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="B66" s="33" t="str">
-        <x:v>2003328-1</x:v>
+        <x:v>2004301-2</x:v>
       </x:c>
       <x:c r="C66" s="39" t="str">
-        <x:v>نظام الإجراءات الجزائية</x:v>
+        <x:v>تدوين السنة</x:v>
       </x:c>
       <x:c r="D66" s="39" t="str">
         <x:v>الشريعة</x:v>
@@ -3388,14 +3389,13 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F66" s="39" t="str">
-        <x:v>الشريعة: قديمة 38
-الشريعة: قديمة 39</x:v>
+        <x:v>الشريعة: جديدة 47</x:v>
       </x:c>
       <x:c r="G66" s="39" t="str">
-        <x:v>6</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H66" s="39" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I66" s="39" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
@@ -3405,7 +3405,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L66" s="39" t="str">
-        <x:v>2003328-1||نظامالاجراءاتالجزايية</x:v>
+        <x:v>2004301-2||تدوينالسنة</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="42" customHeight="1">
@@ -3413,10 +3413,10 @@
         <x:v>62</x:v>
       </x:c>
       <x:c r="B67" s="33" t="str">
-        <x:v>2004301-2</x:v>
+        <x:v>2004476-2</x:v>
       </x:c>
       <x:c r="C67" s="39" t="str">
-        <x:v>تدوين السنة</x:v>
+        <x:v>الأديان والفرق</x:v>
       </x:c>
       <x:c r="D67" s="39" t="str">
         <x:v>الشريعة</x:v>
@@ -3428,7 +3428,7 @@
         <x:v>الشريعة: جديدة 47</x:v>
       </x:c>
       <x:c r="G67" s="39" t="str">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H67" s="39" t="n">
         <x:v>1</x:v>
@@ -3441,7 +3441,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L67" s="39" t="str">
-        <x:v>2004301-2||تدوينالسنة</x:v>
+        <x:v>2004476-2||الاديانوالفرق</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="42" customHeight="1">
@@ -3449,10 +3449,10 @@
         <x:v>63</x:v>
       </x:c>
       <x:c r="B68" s="33" t="str">
-        <x:v>2004476-2</x:v>
+        <x:v>20014201-2</x:v>
       </x:c>
       <x:c r="C68" s="39" t="str">
-        <x:v>الأديان والفرق</x:v>
+        <x:v>التدريبات العملية</x:v>
       </x:c>
       <x:c r="D68" s="39" t="str">
         <x:v>الشريعة</x:v>
@@ -3461,10 +3461,10 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F68" s="39" t="str">
-        <x:v>الشريعة: جديدة 47</x:v>
+        <x:v>الشريعة: قديمة 39</x:v>
       </x:c>
       <x:c r="G68" s="39" t="str">
-        <x:v>6</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H68" s="39" t="n">
         <x:v>1</x:v>
@@ -3477,7 +3477,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L68" s="39" t="str">
-        <x:v>2004476-2||الاديانوالفرق</x:v>
+        <x:v>20014201-2||التدريباتالعملية</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="42" customHeight="1">
@@ -3485,10 +3485,10 @@
         <x:v>64</x:v>
       </x:c>
       <x:c r="B69" s="33" t="str">
-        <x:v>20014201-2</x:v>
+        <x:v>20032202-2</x:v>
       </x:c>
       <x:c r="C69" s="39" t="str">
-        <x:v>التدريبات العملية</x:v>
+        <x:v>المدخل إلى دراسة الأنظمة</x:v>
       </x:c>
       <x:c r="D69" s="39" t="str">
         <x:v>الشريعة</x:v>
@@ -3500,7 +3500,7 @@
         <x:v>الشريعة: قديمة 39</x:v>
       </x:c>
       <x:c r="G69" s="39" t="str">
-        <x:v>8</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H69" s="39" t="n">
         <x:v>1</x:v>
@@ -3513,7 +3513,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L69" s="39" t="str">
-        <x:v>20014201-2||التدريباتالعملية</x:v>
+        <x:v>20032202-2||المدخلاليدراسةالانظمة</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="42" customHeight="1">
@@ -3521,22 +3521,22 @@
         <x:v>65</x:v>
       </x:c>
       <x:c r="B70" s="33" t="str">
-        <x:v>20032202-2</x:v>
+        <x:v>2003880-2</x:v>
       </x:c>
       <x:c r="C70" s="39" t="str">
-        <x:v>المدخل إلى دراسة الأنظمة</x:v>
+        <x:v>الأنظمة العدلية في السعودية</x:v>
       </x:c>
       <x:c r="D70" s="39" t="str">
-        <x:v>الشريعة</x:v>
+        <x:v>الفقه</x:v>
       </x:c>
       <x:c r="E70" s="39" t="str">
-        <x:v>بكالوريوس</x:v>
+        <x:v>ماجستير</x:v>
       </x:c>
       <x:c r="F70" s="39" t="str">
-        <x:v>الشريعة: قديمة 39</x:v>
+        <x:v>الفقه: جديدة 1</x:v>
       </x:c>
       <x:c r="G70" s="39" t="str">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H70" s="39" t="n">
         <x:v>1</x:v>
@@ -3549,7 +3549,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L70" s="39" t="str">
-        <x:v>20032202-2||المدخلاليدراسةالانظمة</x:v>
+        <x:v>2003880-2||الانظمةالعدليةفيالسعودية</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="42" customHeight="1">
@@ -3557,19 +3557,19 @@
         <x:v>66</x:v>
       </x:c>
       <x:c r="B71" s="33" t="str">
-        <x:v>2003880-2</x:v>
+        <x:v>2001205-2</x:v>
       </x:c>
       <x:c r="C71" s="39" t="str">
-        <x:v>الأنظمة العدلية في السعودية</x:v>
+        <x:v>الحديث (1)</x:v>
       </x:c>
       <x:c r="D71" s="39" t="str">
-        <x:v>الفقه</x:v>
+        <x:v>القراءات</x:v>
       </x:c>
       <x:c r="E71" s="39" t="str">
-        <x:v>ماجستير</x:v>
+        <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F71" s="39" t="str">
-        <x:v>الفقه: جديدة 1</x:v>
+        <x:v>القراءات: قديمة 38</x:v>
       </x:c>
       <x:c r="G71" s="39" t="str">
         <x:v>3</x:v>
@@ -3578,14 +3578,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I71" s="39" t="str">
-        <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
-      </x:c>
-      <x:c r="J71" s="39"/>
+        <x:v>يوجد توصيف مؤسسي لبرنامج القرآن وعلومه فقط</x:v>
+      </x:c>
+      <x:c r="J71" s="39" t="str">
+        <x:v>institutional-recovery-20260911/2001205-2.pdf</x:v>
+      </x:c>
       <x:c r="K71" s="39" t="str">
-        <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
+        <x:v>الحصول على دليل خاص ببرنامج القراءات، ثم ربط مخرجاته في نطاقه فقط</x:v>
       </x:c>
       <x:c r="L71" s="39" t="str">
-        <x:v>2003880-2||الانظمةالعدليةفيالسعودية</x:v>
+        <x:v>2001205-2||الحديث1</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="42" customHeight="1">
@@ -3593,10 +3595,10 @@
         <x:v>67</x:v>
       </x:c>
       <x:c r="B72" s="33" t="str">
-        <x:v>2001205-2</x:v>
+        <x:v>2001209-2</x:v>
       </x:c>
       <x:c r="C72" s="39" t="str">
-        <x:v>الحديث (1)</x:v>
+        <x:v>الحديث (2)</x:v>
       </x:c>
       <x:c r="D72" s="39" t="str">
         <x:v>القراءات</x:v>
@@ -3608,7 +3610,7 @@
         <x:v>القراءات: قديمة 38</x:v>
       </x:c>
       <x:c r="G72" s="39" t="str">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H72" s="39" t="n">
         <x:v>1</x:v>
@@ -3617,13 +3619,13 @@
         <x:v>يوجد توصيف مؤسسي لبرنامج القرآن وعلومه فقط</x:v>
       </x:c>
       <x:c r="J72" s="39" t="str">
-        <x:v>institutional-recovery-20260911/2001205-2.pdf</x:v>
+        <x:v>institutional-recovery-20260911/2001209-2.pdf</x:v>
       </x:c>
       <x:c r="K72" s="39" t="str">
         <x:v>الحصول على دليل خاص ببرنامج القراءات، ثم ربط مخرجاته في نطاقه فقط</x:v>
       </x:c>
       <x:c r="L72" s="39" t="str">
-        <x:v>2001205-2||الحديث1</x:v>
+        <x:v>2001209-2||الحديث2</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="42" customHeight="1">
@@ -3631,10 +3633,10 @@
         <x:v>68</x:v>
       </x:c>
       <x:c r="B73" s="33" t="str">
-        <x:v>2001209-2</x:v>
+        <x:v>2001221-2</x:v>
       </x:c>
       <x:c r="C73" s="39" t="str">
-        <x:v>الحديث (2)</x:v>
+        <x:v>الفقه (1)</x:v>
       </x:c>
       <x:c r="D73" s="39" t="str">
         <x:v>القراءات</x:v>
@@ -3643,25 +3645,25 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F73" s="39" t="str">
-        <x:v>القراءات: قديمة 38</x:v>
+        <x:v>القراءات: جديدة 47؛ القراءات: قديمة 38</x:v>
       </x:c>
       <x:c r="G73" s="39" t="str">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H73" s="39" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I73" s="39" t="str">
         <x:v>يوجد توصيف مؤسسي لبرنامج القرآن وعلومه فقط</x:v>
       </x:c>
       <x:c r="J73" s="39" t="str">
-        <x:v>institutional-recovery-20260911/2001209-2.pdf</x:v>
+        <x:v>institutional-recovery-20260911/2001221-2.pdf</x:v>
       </x:c>
       <x:c r="K73" s="39" t="str">
         <x:v>الحصول على دليل خاص ببرنامج القراءات، ثم ربط مخرجاته في نطاقه فقط</x:v>
       </x:c>
       <x:c r="L73" s="39" t="str">
-        <x:v>2001209-2||الحديث2</x:v>
+        <x:v>2001221-2||الفقه1</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="42" customHeight="1">
@@ -3669,10 +3671,10 @@
         <x:v>69</x:v>
       </x:c>
       <x:c r="B74" s="33" t="str">
-        <x:v>2001221-2</x:v>
+        <x:v>2001273-2</x:v>
       </x:c>
       <x:c r="C74" s="39" t="str">
-        <x:v>الفقه (1)</x:v>
+        <x:v>العقيدة (1)</x:v>
       </x:c>
       <x:c r="D74" s="39" t="str">
         <x:v>القراءات</x:v>
@@ -3681,25 +3683,23 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F74" s="39" t="str">
-        <x:v>القراءات: جديدة 47؛ القراءات: قديمة 38</x:v>
+        <x:v>القراءات: قديمة 38</x:v>
       </x:c>
       <x:c r="G74" s="39" t="str">
         <x:v>3</x:v>
       </x:c>
       <x:c r="H74" s="39" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I74" s="39" t="str">
-        <x:v>يوجد توصيف مؤسسي لبرنامج القرآن وعلومه فقط</x:v>
-      </x:c>
-      <x:c r="J74" s="39" t="str">
-        <x:v>institutional-recovery-20260911/2001221-2.pdf</x:v>
-      </x:c>
+        <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
+      </x:c>
+      <x:c r="J74" s="39"/>
       <x:c r="K74" s="39" t="str">
-        <x:v>الحصول على دليل خاص ببرنامج القراءات، ثم ربط مخرجاته في نطاقه فقط</x:v>
+        <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L74" s="39" t="str">
-        <x:v>2001221-2||الفقه1</x:v>
+        <x:v>2001273-2||العقيدة1</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="42" customHeight="1">
@@ -3707,10 +3707,10 @@
         <x:v>70</x:v>
       </x:c>
       <x:c r="B75" s="33" t="str">
-        <x:v>2001273-2</x:v>
+        <x:v>2001320-2</x:v>
       </x:c>
       <x:c r="C75" s="39" t="str">
-        <x:v>العقيدة (1)</x:v>
+        <x:v>الحديث (3)</x:v>
       </x:c>
       <x:c r="D75" s="39" t="str">
         <x:v>القراءات</x:v>
@@ -3722,20 +3722,22 @@
         <x:v>القراءات: قديمة 38</x:v>
       </x:c>
       <x:c r="G75" s="39" t="str">
-        <x:v>3</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H75" s="39" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="I75" s="39" t="str">
-        <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
-      </x:c>
-      <x:c r="J75" s="39"/>
+        <x:v>يوجد توصيف مؤسسي لبرنامج القرآن وعلومه فقط</x:v>
+      </x:c>
+      <x:c r="J75" s="39" t="str">
+        <x:v>institutional-recovery-20260911/2001320-2.pdf</x:v>
+      </x:c>
       <x:c r="K75" s="39" t="str">
-        <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
+        <x:v>الحصول على دليل خاص ببرنامج القراءات، ثم ربط مخرجاته في نطاقه فقط</x:v>
       </x:c>
       <x:c r="L75" s="39" t="str">
-        <x:v>2001273-2||العقيدة1</x:v>
+        <x:v>2001320-2||الحديث3</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="42" customHeight="1">
@@ -3743,10 +3745,10 @@
         <x:v>71</x:v>
       </x:c>
       <x:c r="B76" s="33" t="str">
-        <x:v>2001320-2</x:v>
+        <x:v>2001322-2</x:v>
       </x:c>
       <x:c r="C76" s="39" t="str">
-        <x:v>الحديث (3)</x:v>
+        <x:v>الفقه (2)</x:v>
       </x:c>
       <x:c r="D76" s="39" t="str">
         <x:v>القراءات</x:v>
@@ -3758,7 +3760,7 @@
         <x:v>القراءات: قديمة 38</x:v>
       </x:c>
       <x:c r="G76" s="39" t="str">
-        <x:v>6</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H76" s="39" t="n">
         <x:v>1</x:v>
@@ -3767,13 +3769,13 @@
         <x:v>يوجد توصيف مؤسسي لبرنامج القرآن وعلومه فقط</x:v>
       </x:c>
       <x:c r="J76" s="39" t="str">
-        <x:v>institutional-recovery-20260911/2001320-2.pdf</x:v>
+        <x:v>institutional-recovery-20260911/2001322-2.pdf</x:v>
       </x:c>
       <x:c r="K76" s="39" t="str">
         <x:v>الحصول على دليل خاص ببرنامج القراءات، ثم ربط مخرجاته في نطاقه فقط</x:v>
       </x:c>
       <x:c r="L76" s="39" t="str">
-        <x:v>2001320-2||الحديث3</x:v>
+        <x:v>2001322-2||الفقه2</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="42" customHeight="1">
@@ -3781,10 +3783,10 @@
         <x:v>72</x:v>
       </x:c>
       <x:c r="B77" s="33" t="str">
-        <x:v>2001322-2</x:v>
+        <x:v>2002111-3</x:v>
       </x:c>
       <x:c r="C77" s="39" t="str">
-        <x:v>الفقه (2)</x:v>
+        <x:v>عرض القراءات السبع (١)</x:v>
       </x:c>
       <x:c r="D77" s="39" t="str">
         <x:v>القراءات</x:v>
@@ -3793,25 +3795,23 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F77" s="39" t="str">
-        <x:v>القراءات: قديمة 38</x:v>
+        <x:v>القراءات: جديدة 47</x:v>
       </x:c>
       <x:c r="G77" s="39" t="str">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H77" s="39" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="I77" s="39" t="str">
-        <x:v>يوجد توصيف مؤسسي لبرنامج القرآن وعلومه فقط</x:v>
-      </x:c>
-      <x:c r="J77" s="39" t="str">
-        <x:v>institutional-recovery-20260911/2001322-2.pdf</x:v>
-      </x:c>
+        <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
+      </x:c>
+      <x:c r="J77" s="39"/>
       <x:c r="K77" s="39" t="str">
-        <x:v>الحصول على دليل خاص ببرنامج القراءات، ثم ربط مخرجاته في نطاقه فقط</x:v>
+        <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L77" s="39" t="str">
-        <x:v>2001322-2||الفقه2</x:v>
+        <x:v>2002111-3||عرضالقراءاتالسبع١</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="42" customHeight="1">
@@ -3819,10 +3819,10 @@
         <x:v>73</x:v>
       </x:c>
       <x:c r="B78" s="33" t="str">
-        <x:v>2002111-3</x:v>
+        <x:v>2002112-3</x:v>
       </x:c>
       <x:c r="C78" s="39" t="str">
-        <x:v>عرض القراءات السبع (١)</x:v>
+        <x:v>عرض القراءات السبع (٢)</x:v>
       </x:c>
       <x:c r="D78" s="39" t="str">
         <x:v>القراءات</x:v>
@@ -3834,7 +3834,7 @@
         <x:v>القراءات: جديدة 47</x:v>
       </x:c>
       <x:c r="G78" s="39" t="str">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H78" s="39" t="n">
         <x:v>1</x:v>
@@ -3847,7 +3847,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L78" s="39" t="str">
-        <x:v>2002111-3||عرضالقراءاتالسبع١</x:v>
+        <x:v>2002112-3||عرضالقراءاتالسبع٢</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="42" customHeight="1">
@@ -3855,10 +3855,10 @@
         <x:v>74</x:v>
       </x:c>
       <x:c r="B79" s="33" t="str">
-        <x:v>2002112-3</x:v>
+        <x:v>2002113-3</x:v>
       </x:c>
       <x:c r="C79" s="39" t="str">
-        <x:v>عرض القراءات السبع (٢)</x:v>
+        <x:v>عرض القراءات السبع (٣)</x:v>
       </x:c>
       <x:c r="D79" s="39" t="str">
         <x:v>القراءات</x:v>
@@ -3870,7 +3870,7 @@
         <x:v>القراءات: جديدة 47</x:v>
       </x:c>
       <x:c r="G79" s="39" t="str">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H79" s="39" t="n">
         <x:v>1</x:v>
@@ -3883,7 +3883,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L79" s="39" t="str">
-        <x:v>2002112-3||عرضالقراءاتالسبع٢</x:v>
+        <x:v>2002113-3||عرضالقراءاتالسبع٣</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="42" customHeight="1">
@@ -3891,10 +3891,10 @@
         <x:v>75</x:v>
       </x:c>
       <x:c r="B80" s="33" t="str">
-        <x:v>2002113-3</x:v>
+        <x:v>2002114-3</x:v>
       </x:c>
       <x:c r="C80" s="39" t="str">
-        <x:v>عرض القراءات السبع (٣)</x:v>
+        <x:v>عرض القراءات السبع (٤)</x:v>
       </x:c>
       <x:c r="D80" s="39" t="str">
         <x:v>القراءات</x:v>
@@ -3906,7 +3906,7 @@
         <x:v>القراءات: جديدة 47</x:v>
       </x:c>
       <x:c r="G80" s="39" t="str">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H80" s="39" t="n">
         <x:v>1</x:v>
@@ -3919,7 +3919,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L80" s="39" t="str">
-        <x:v>2002113-3||عرضالقراءاتالسبع٣</x:v>
+        <x:v>2002114-3||عرضالقراءاتالسبع٤</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="42" customHeight="1">
@@ -3927,10 +3927,10 @@
         <x:v>76</x:v>
       </x:c>
       <x:c r="B81" s="33" t="str">
-        <x:v>2002114-3</x:v>
+        <x:v>2002238-2</x:v>
       </x:c>
       <x:c r="C81" s="39" t="str">
-        <x:v>عرض القراءات السبع (٤)</x:v>
+        <x:v>الوقف والابتداء</x:v>
       </x:c>
       <x:c r="D81" s="39" t="str">
         <x:v>القراءات</x:v>
@@ -3942,7 +3942,7 @@
         <x:v>القراءات: جديدة 47</x:v>
       </x:c>
       <x:c r="G81" s="39" t="str">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H81" s="39" t="n">
         <x:v>1</x:v>
@@ -3955,7 +3955,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L81" s="39" t="str">
-        <x:v>2002114-3||عرضالقراءاتالسبع٤</x:v>
+        <x:v>2002238-2||الوقفوالابتداء</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="42" customHeight="1">
@@ -3963,10 +3963,10 @@
         <x:v>77</x:v>
       </x:c>
       <x:c r="B82" s="33" t="str">
-        <x:v>2002238-2</x:v>
+        <x:v>2002239-2</x:v>
       </x:c>
       <x:c r="C82" s="39" t="str">
-        <x:v>الوقف والابتداء</x:v>
+        <x:v>مصادر ومناهج المؤلفين في القراءات</x:v>
       </x:c>
       <x:c r="D82" s="39" t="str">
         <x:v>القراءات</x:v>
@@ -3991,7 +3991,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L82" s="39" t="str">
-        <x:v>2002238-2||الوقفوالابتداء</x:v>
+        <x:v>2002239-2||مصادرومناهجالمولفينفيالقراءات</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="42" customHeight="1">
@@ -3999,10 +3999,10 @@
         <x:v>78</x:v>
       </x:c>
       <x:c r="B83" s="33" t="str">
-        <x:v>2002239-2</x:v>
+        <x:v>2002266-6</x:v>
       </x:c>
       <x:c r="C83" s="39" t="str">
-        <x:v>مصادر ومناهج المؤلفين في القراءات</x:v>
+        <x:v>التدريب التعاوني</x:v>
       </x:c>
       <x:c r="D83" s="39" t="str">
         <x:v>القراءات</x:v>
@@ -4014,7 +4014,7 @@
         <x:v>القراءات: جديدة 47</x:v>
       </x:c>
       <x:c r="G83" s="39" t="str">
-        <x:v>5</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H83" s="39" t="n">
         <x:v>1</x:v>
@@ -4027,7 +4027,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L83" s="39" t="str">
-        <x:v>2002239-2||مصادرومناهجالمولفينفيالقراءات</x:v>
+        <x:v>2002266-6||التدريبالتعاوني</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="42" customHeight="1">
@@ -4035,10 +4035,10 @@
         <x:v>79</x:v>
       </x:c>
       <x:c r="B84" s="33" t="str">
-        <x:v>2002266-6</x:v>
+        <x:v>2002280-2</x:v>
       </x:c>
       <x:c r="C84" s="39" t="str">
-        <x:v>التدريب التعاوني</x:v>
+        <x:v>تدريبات على الجمع والكيفيات</x:v>
       </x:c>
       <x:c r="D84" s="39" t="str">
         <x:v>القراءات</x:v>
@@ -4050,7 +4050,7 @@
         <x:v>القراءات: جديدة 47</x:v>
       </x:c>
       <x:c r="G84" s="39" t="str">
-        <x:v>8</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H84" s="39" t="n">
         <x:v>1</x:v>
@@ -4063,7 +4063,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L84" s="39" t="str">
-        <x:v>2002266-6||التدريبالتعاوني</x:v>
+        <x:v>2002280-2||تدريباتعليالجمعوالكيفيات</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="42" customHeight="1">
@@ -4071,10 +4071,10 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="B85" s="33" t="str">
-        <x:v>2002280-2</x:v>
+        <x:v>2002352-2</x:v>
       </x:c>
       <x:c r="C85" s="39" t="str">
-        <x:v>تدريبات على الجمع والكيفيات</x:v>
+        <x:v>التفسير التحليلي (2)</x:v>
       </x:c>
       <x:c r="D85" s="39" t="str">
         <x:v>القراءات</x:v>
@@ -4086,7 +4086,7 @@
         <x:v>القراءات: جديدة 47</x:v>
       </x:c>
       <x:c r="G85" s="39" t="str">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H85" s="39" t="n">
         <x:v>1</x:v>
@@ -4099,7 +4099,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L85" s="39" t="str">
-        <x:v>2002280-2||تدريباتعليالجمعوالكيفيات</x:v>
+        <x:v>2002352-2||التفسيرالتحليلي2</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="42" customHeight="1">
@@ -4107,10 +4107,10 @@
         <x:v>81</x:v>
       </x:c>
       <x:c r="B86" s="33" t="str">
-        <x:v>2002352-2</x:v>
+        <x:v>2002460-2</x:v>
       </x:c>
       <x:c r="C86" s="39" t="str">
-        <x:v>التفسير التحليلي (2)</x:v>
+        <x:v>عرض القراءات الثلاث (١)</x:v>
       </x:c>
       <x:c r="D86" s="39" t="str">
         <x:v>القراءات</x:v>
@@ -4122,7 +4122,7 @@
         <x:v>القراءات: جديدة 47</x:v>
       </x:c>
       <x:c r="G86" s="39" t="str">
-        <x:v>4</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="H86" s="39" t="n">
         <x:v>1</x:v>
@@ -4135,7 +4135,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L86" s="39" t="str">
-        <x:v>2002352-2||التفسيرالتحليلي2</x:v>
+        <x:v>2002460-2||عرضالقراءاتالثلاث١</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="42" customHeight="1">
@@ -4143,10 +4143,10 @@
         <x:v>82</x:v>
       </x:c>
       <x:c r="B87" s="33" t="str">
-        <x:v>2002460-2</x:v>
+        <x:v>2002461-2</x:v>
       </x:c>
       <x:c r="C87" s="39" t="str">
-        <x:v>عرض القراءات الثلاث (١)</x:v>
+        <x:v>عرض القراءات الثلاث (٢)</x:v>
       </x:c>
       <x:c r="D87" s="39" t="str">
         <x:v>القراءات</x:v>
@@ -4158,7 +4158,7 @@
         <x:v>القراءات: جديدة 47</x:v>
       </x:c>
       <x:c r="G87" s="39" t="str">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H87" s="39" t="n">
         <x:v>1</x:v>
@@ -4171,7 +4171,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L87" s="39" t="str">
-        <x:v>2002460-2||عرضالقراءاتالثلاث١</x:v>
+        <x:v>2002461-2||عرضالقراءاتالثلاث٢</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="42" customHeight="1">
@@ -4179,25 +4179,26 @@
         <x:v>83</x:v>
       </x:c>
       <x:c r="B88" s="33" t="str">
-        <x:v>2002461-2</x:v>
+        <x:v>2004102-2</x:v>
       </x:c>
       <x:c r="C88" s="39" t="str">
-        <x:v>عرض القراءات الثلاث (٢)</x:v>
+        <x:v>مصطلح الحديث</x:v>
       </x:c>
       <x:c r="D88" s="39" t="str">
-        <x:v>القراءات</x:v>
+        <x:v>القراءات، القرآن وعلومه</x:v>
       </x:c>
       <x:c r="E88" s="39" t="str">
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F88" s="39" t="str">
-        <x:v>القراءات: جديدة 47</x:v>
+        <x:v>القراءات: جديدة 47
+القرآن وعلومه: جديدة 47</x:v>
       </x:c>
       <x:c r="G88" s="39" t="str">
-        <x:v>8</x:v>
+        <x:v>2، 3</x:v>
       </x:c>
       <x:c r="H88" s="39" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I88" s="39" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
@@ -4207,7 +4208,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L88" s="39" t="str">
-        <x:v>2002461-2||عرضالقراءاتالثلاث٢</x:v>
+        <x:v>2004102-2||مصطلحالحديث</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="42" customHeight="1">
@@ -4215,10 +4216,10 @@
         <x:v>84</x:v>
       </x:c>
       <x:c r="B89" s="33" t="str">
-        <x:v>2004102-2</x:v>
+        <x:v>2004320-2</x:v>
       </x:c>
       <x:c r="C89" s="39" t="str">
-        <x:v>مصطلح الحديث</x:v>
+        <x:v>الحديث (3)</x:v>
       </x:c>
       <x:c r="D89" s="39" t="str">
         <x:v>القراءات، القرآن وعلومه</x:v>
@@ -4231,7 +4232,7 @@
 القرآن وعلومه: جديدة 47</x:v>
       </x:c>
       <x:c r="G89" s="39" t="str">
-        <x:v>2، 3</x:v>
+        <x:v>5، 6</x:v>
       </x:c>
       <x:c r="H89" s="39" t="n">
         <x:v>2</x:v>
@@ -4244,7 +4245,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L89" s="39" t="str">
-        <x:v>2004102-2||مصطلحالحديث</x:v>
+        <x:v>2004320-2||الحديث3</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="42" customHeight="1">
@@ -4252,26 +4253,25 @@
         <x:v>85</x:v>
       </x:c>
       <x:c r="B90" s="33" t="str">
-        <x:v>2004320-2</x:v>
+        <x:v>101221-2</x:v>
       </x:c>
       <x:c r="C90" s="39" t="str">
-        <x:v>الحديث (3)</x:v>
+        <x:v>الفقه (1)</x:v>
       </x:c>
       <x:c r="D90" s="39" t="str">
-        <x:v>القراءات، القرآن وعلومه</x:v>
+        <x:v>القرآن وعلومه</x:v>
       </x:c>
       <x:c r="E90" s="39" t="str">
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F90" s="39" t="str">
-        <x:v>القراءات: جديدة 47
-القرآن وعلومه: جديدة 47</x:v>
+        <x:v>القرآن وعلومه: قديمة 39</x:v>
       </x:c>
       <x:c r="G90" s="39" t="str">
-        <x:v>5، 6</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H90" s="39" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I90" s="39" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
@@ -4281,7 +4281,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L90" s="39" t="str">
-        <x:v>2004320-2||الحديث3</x:v>
+        <x:v>101221-2||الفقه1</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="42" customHeight="1">
@@ -4289,10 +4289,10 @@
         <x:v>86</x:v>
       </x:c>
       <x:c r="B91" s="33" t="str">
-        <x:v>101221-2</x:v>
+        <x:v>2002266-5</x:v>
       </x:c>
       <x:c r="C91" s="39" t="str">
-        <x:v>الفقه (1)</x:v>
+        <x:v>التدريب التعاوني</x:v>
       </x:c>
       <x:c r="D91" s="39" t="str">
         <x:v>القرآن وعلومه</x:v>
@@ -4301,10 +4301,10 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F91" s="39" t="str">
-        <x:v>القرآن وعلومه: قديمة 39</x:v>
+        <x:v>القرآن وعلومه: جديدة 47</x:v>
       </x:c>
       <x:c r="G91" s="39" t="str">
-        <x:v>3</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H91" s="39" t="n">
         <x:v>1</x:v>
@@ -4317,7 +4317,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L91" s="39" t="str">
-        <x:v>101221-2||الفقه1</x:v>
+        <x:v>2002266-5||التدريبالتعاوني</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="42" customHeight="1">
@@ -4325,10 +4325,10 @@
         <x:v>87</x:v>
       </x:c>
       <x:c r="B92" s="33" t="str">
-        <x:v>2002266-5</x:v>
+        <x:v>20024101-2</x:v>
       </x:c>
       <x:c r="C92" s="39" t="str">
-        <x:v>التدريب التعاوني</x:v>
+        <x:v>قاعة بحث</x:v>
       </x:c>
       <x:c r="D92" s="39" t="str">
         <x:v>القرآن وعلومه</x:v>
@@ -4340,7 +4340,7 @@
         <x:v>القرآن وعلومه: جديدة 47</x:v>
       </x:c>
       <x:c r="G92" s="39" t="str">
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="H92" s="39" t="n">
         <x:v>1</x:v>
@@ -4353,44 +4353,22 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L92" s="39" t="str">
-        <x:v>2002266-5||التدريبالتعاوني</x:v>
+        <x:v>20024101-2||قاعةبحث</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="42" customHeight="1">
-      <x:c r="A93" s="33" t="n">
-        <x:v>88</x:v>
-      </x:c>
-      <x:c r="B93" s="33" t="str">
-        <x:v>20024101-2</x:v>
-      </x:c>
-      <x:c r="C93" s="39" t="str">
-        <x:v>قاعة بحث</x:v>
-      </x:c>
-      <x:c r="D93" s="39" t="str">
-        <x:v>القرآن وعلومه</x:v>
-      </x:c>
-      <x:c r="E93" s="39" t="str">
-        <x:v>بكالوريوس</x:v>
-      </x:c>
-      <x:c r="F93" s="39" t="str">
-        <x:v>القرآن وعلومه: جديدة 47</x:v>
-      </x:c>
-      <x:c r="G93" s="39" t="str">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="H93" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I93" s="39" t="str">
-        <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
-      </x:c>
+      <x:c r="A93" s="33"/>
+      <x:c r="B93" s="33"/>
+      <x:c r="C93" s="39"/>
+      <x:c r="D93" s="39"/>
+      <x:c r="E93" s="39"/>
+      <x:c r="F93" s="39"/>
+      <x:c r="G93" s="39"/>
+      <x:c r="H93" s="39"/>
+      <x:c r="I93" s="39"/>
       <x:c r="J93" s="39"/>
-      <x:c r="K93" s="39" t="str">
-        <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
-      </x:c>
-      <x:c r="L93" s="39" t="str">
-        <x:v>20024101-2||قاعةبحث</x:v>
-      </x:c>
+      <x:c r="K93" s="39"/>
+      <x:c r="L93" s="39"/>
     </x:row>
     <x:row r="94" ht="42" customHeight="1">
       <x:c r="A94" s="33"/>
@@ -4651,7 +4629,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R138168772ed64510"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R447243e16813405a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4718,7 +4696,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>عدد المواضع: 102. كل صف يمثل ظهور مقرر في برنامج وخطة وإصدار محدد.</x:v>
+        <x:v>عدد المواضع: 101. كل صف يمثل ظهور مقرر في برنامج وخطة وإصدار محدد.</x:v>
       </x:c>
       <x:c r="B3"/>
       <x:c r="C3"/>
@@ -6394,13 +6372,13 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="G41" s="43" t="str">
-        <x:v>2004269-4</x:v>
+        <x:v>2004272-2</x:v>
       </x:c>
       <x:c r="H41" s="42" t="str">
-        <x:v>التخريج ودراسة الأسانيد</x:v>
+        <x:v>العمل الخيري</x:v>
       </x:c>
       <x:c r="I41" s="43" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J41" s="42" t="str">
         <x:v>نظري</x:v>
@@ -6416,7 +6394,7 @@
       </x:c>
       <x:c r="N41" s="42"/>
       <x:c r="O41" s="42" t="str">
-        <x:v>2004269-4||التخريجودراسةالاسانيد</x:v>
+        <x:v>2004272-2||العملالخيري</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="34" customHeight="1">
@@ -6439,10 +6417,10 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="G42" s="43" t="str">
-        <x:v>2004272-2</x:v>
+        <x:v>20043111-2</x:v>
       </x:c>
       <x:c r="H42" s="42" t="str">
-        <x:v>العمل الخيري</x:v>
+        <x:v>الأمن الفكري</x:v>
       </x:c>
       <x:c r="I42" s="43" t="n">
         <x:v>2</x:v>
@@ -6451,7 +6429,7 @@
         <x:v>نظري</x:v>
       </x:c>
       <x:c r="K42" s="42" t="str">
-        <x:v>إجبارية القسم</x:v>
+        <x:v>اختيارية القسم</x:v>
       </x:c>
       <x:c r="L42" s="42" t="str">
         <x:v>الإسلامية 47.pdf</x:v>
@@ -6461,7 +6439,7 @@
       </x:c>
       <x:c r="N42" s="42"/>
       <x:c r="O42" s="42" t="str">
-        <x:v>2004272-2||العملالخيري</x:v>
+        <x:v>20043111-2||الامنالفكري</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="34" customHeight="1">
@@ -6481,13 +6459,13 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="F43" s="43" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G43" s="43" t="str">
-        <x:v>20043111-2</x:v>
+        <x:v>2001270-2</x:v>
       </x:c>
       <x:c r="H43" s="42" t="str">
-        <x:v>الأمن الفكري</x:v>
+        <x:v>فقه النوازل</x:v>
       </x:c>
       <x:c r="I43" s="43" t="n">
         <x:v>2</x:v>
@@ -6496,7 +6474,7 @@
         <x:v>نظري</x:v>
       </x:c>
       <x:c r="K43" s="42" t="str">
-        <x:v>اختيارية القسم</x:v>
+        <x:v>إجبارية القسم</x:v>
       </x:c>
       <x:c r="L43" s="42" t="str">
         <x:v>الإسلامية 47.pdf</x:v>
@@ -6506,7 +6484,7 @@
       </x:c>
       <x:c r="N43" s="42"/>
       <x:c r="O43" s="42" t="str">
-        <x:v>20043111-2||الامنالفكري</x:v>
+        <x:v>2001270-2||فقهالنوازل</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="34" customHeight="1">
@@ -6529,16 +6507,16 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G44" s="43" t="str">
-        <x:v>2001270-2</x:v>
+        <x:v>20044220-4</x:v>
       </x:c>
       <x:c r="H44" s="42" t="str">
-        <x:v>فقه النوازل</x:v>
+        <x:v>التدريب التعاوني</x:v>
       </x:c>
       <x:c r="I44" s="43" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="J44" s="42" t="str">
-        <x:v>نظري</x:v>
+        <x:v>تدريب</x:v>
       </x:c>
       <x:c r="K44" s="42" t="str">
         <x:v>إجبارية القسم</x:v>
@@ -6551,7 +6529,7 @@
       </x:c>
       <x:c r="N44" s="42"/>
       <x:c r="O44" s="42" t="str">
-        <x:v>2001270-2||فقهالنوازل</x:v>
+        <x:v>20044220-4||التدريبالتعاوني</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="34" customHeight="1">
@@ -6565,38 +6543,38 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="D45" s="42" t="str">
-        <x:v>جديدة</x:v>
+        <x:v>قديمة</x:v>
       </x:c>
       <x:c r="E45" s="43" t="n">
-        <x:v>47</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="F45" s="43" t="n">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G45" s="43" t="str">
-        <x:v>20044220-4</x:v>
+        <x:v>20043105-2</x:v>
       </x:c>
       <x:c r="H45" s="42" t="str">
-        <x:v>التدريب التعاوني</x:v>
+        <x:v>الفقه المقارن</x:v>
       </x:c>
       <x:c r="I45" s="43" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J45" s="42" t="str">
-        <x:v>تدريب</x:v>
+        <x:v>نظري</x:v>
       </x:c>
       <x:c r="K45" s="42" t="str">
         <x:v>إجبارية القسم</x:v>
       </x:c>
       <x:c r="L45" s="42" t="str">
-        <x:v>الإسلامية 47.pdf</x:v>
+        <x:v>الدراسات الإسلامية 39.pdf</x:v>
       </x:c>
       <x:c r="M45" s="42" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
       </x:c>
       <x:c r="N45" s="42"/>
       <x:c r="O45" s="42" t="str">
-        <x:v>20044220-4||التدريبالتعاوني</x:v>
+        <x:v>20043105-2||الفقهالمقارن</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="34" customHeight="1">
@@ -6619,10 +6597,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G46" s="43" t="str">
-        <x:v>20043105-2</x:v>
+        <x:v>20043108-2</x:v>
       </x:c>
       <x:c r="H46" s="42" t="str">
-        <x:v>الفقه المقارن</x:v>
+        <x:v>علم المواريث (1)</x:v>
       </x:c>
       <x:c r="I46" s="43" t="n">
         <x:v>2</x:v>
@@ -6641,7 +6619,7 @@
       </x:c>
       <x:c r="N46" s="42"/>
       <x:c r="O46" s="42" t="str">
-        <x:v>20043105-2||الفقهالمقارن</x:v>
+        <x:v>20043108-2||علمالمواريث1</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="34" customHeight="1">
@@ -6661,13 +6639,13 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="F47" s="43" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G47" s="43" t="str">
-        <x:v>20043108-2</x:v>
+        <x:v>20043202-2</x:v>
       </x:c>
       <x:c r="H47" s="42" t="str">
-        <x:v>علم المواريث (1)</x:v>
+        <x:v>القواعد الفقهية</x:v>
       </x:c>
       <x:c r="I47" s="43" t="n">
         <x:v>2</x:v>
@@ -6686,7 +6664,7 @@
       </x:c>
       <x:c r="N47" s="42"/>
       <x:c r="O47" s="42" t="str">
-        <x:v>20043108-2||علمالمواريث1</x:v>
+        <x:v>20043202-2||القواعدالفقهية</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="34" customHeight="1">
@@ -6706,13 +6684,13 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="F48" s="43" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G48" s="43" t="str">
-        <x:v>20043202-2</x:v>
+        <x:v>20044101-2</x:v>
       </x:c>
       <x:c r="H48" s="42" t="str">
-        <x:v>القواعد الفقهية</x:v>
+        <x:v>أصول فقه (3)</x:v>
       </x:c>
       <x:c r="I48" s="43" t="n">
         <x:v>2</x:v>
@@ -6731,7 +6709,7 @@
       </x:c>
       <x:c r="N48" s="42"/>
       <x:c r="O48" s="42" t="str">
-        <x:v>20043202-2||القواعدالفقهية</x:v>
+        <x:v>20044101-2||اصولفقه3</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="34" customHeight="1">
@@ -6751,13 +6729,13 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="F49" s="43" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G49" s="43" t="str">
-        <x:v>20044101-2</x:v>
+        <x:v>20044206-2</x:v>
       </x:c>
       <x:c r="H49" s="42" t="str">
-        <x:v>أصول فقه (3)</x:v>
+        <x:v>علم المواريث (2)</x:v>
       </x:c>
       <x:c r="I49" s="43" t="n">
         <x:v>2</x:v>
@@ -6776,7 +6754,7 @@
       </x:c>
       <x:c r="N49" s="42"/>
       <x:c r="O49" s="42" t="str">
-        <x:v>20044101-2||اصولفقه3</x:v>
+        <x:v>20044206-2||علمالمواريث2</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="34" customHeight="1">
@@ -6784,25 +6762,25 @@
         <x:v>45</x:v>
       </x:c>
       <x:c r="B50" s="42" t="str">
-        <x:v>الدراسات الإسلامية</x:v>
+        <x:v>الشريعة</x:v>
       </x:c>
       <x:c r="C50" s="42" t="str">
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="D50" s="42" t="str">
-        <x:v>قديمة</x:v>
+        <x:v>جديدة</x:v>
       </x:c>
       <x:c r="E50" s="43" t="n">
-        <x:v>39</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="F50" s="43" t="n">
-        <x:v>8</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G50" s="43" t="str">
-        <x:v>20044206-2</x:v>
+        <x:v>2004301-2</x:v>
       </x:c>
       <x:c r="H50" s="42" t="str">
-        <x:v>علم المواريث (2)</x:v>
+        <x:v>تدوين السنة</x:v>
       </x:c>
       <x:c r="I50" s="43" t="n">
         <x:v>2</x:v>
@@ -6811,17 +6789,17 @@
         <x:v>نظري</x:v>
       </x:c>
       <x:c r="K50" s="42" t="str">
-        <x:v>إجبارية القسم</x:v>
+        <x:v>متطلبات الكلية</x:v>
       </x:c>
       <x:c r="L50" s="42" t="str">
-        <x:v>الدراسات الإسلامية 39.pdf</x:v>
+        <x:v>الشريعة 47.pdf</x:v>
       </x:c>
       <x:c r="M50" s="42" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
       </x:c>
       <x:c r="N50" s="42"/>
       <x:c r="O50" s="42" t="str">
-        <x:v>20044206-2||علمالمواريث2</x:v>
+        <x:v>2004301-2||تدوينالسنة</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="34" customHeight="1">
@@ -6841,13 +6819,13 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="F51" s="43" t="n">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G51" s="43" t="str">
-        <x:v>2004301-2</x:v>
+        <x:v>2004476-2</x:v>
       </x:c>
       <x:c r="H51" s="42" t="str">
-        <x:v>تدوين السنة</x:v>
+        <x:v>الأديان والفرق</x:v>
       </x:c>
       <x:c r="I51" s="43" t="n">
         <x:v>2</x:v>
@@ -6866,7 +6844,7 @@
       </x:c>
       <x:c r="N51" s="42"/>
       <x:c r="O51" s="42" t="str">
-        <x:v>2004301-2||تدوينالسنة</x:v>
+        <x:v>2004476-2||الاديانوالفرق</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="34" customHeight="1">
@@ -6880,19 +6858,19 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="D52" s="42" t="str">
-        <x:v>جديدة</x:v>
+        <x:v>قديمة</x:v>
       </x:c>
       <x:c r="E52" s="43" t="n">
-        <x:v>47</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="F52" s="43" t="n">
-        <x:v>6</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G52" s="43" t="str">
-        <x:v>2004476-2</x:v>
+        <x:v>2001193-2</x:v>
       </x:c>
       <x:c r="H52" s="42" t="str">
-        <x:v>الأديان والفرق</x:v>
+        <x:v>علوم الحديث (1)</x:v>
       </x:c>
       <x:c r="I52" s="43" t="n">
         <x:v>2</x:v>
@@ -6901,17 +6879,17 @@
         <x:v>نظري</x:v>
       </x:c>
       <x:c r="K52" s="42" t="str">
-        <x:v>متطلبات الكلية</x:v>
+        <x:v>إجبارية القسم</x:v>
       </x:c>
       <x:c r="L52" s="42" t="str">
-        <x:v>الشريعة 47.pdf</x:v>
+        <x:v>خطط الإصدارات السابقة.pdf</x:v>
       </x:c>
       <x:c r="M52" s="42" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
       </x:c>
       <x:c r="N52" s="42"/>
       <x:c r="O52" s="42" t="str">
-        <x:v>2004476-2||الاديانوالفرق</x:v>
+        <x:v>2001193-2||علومالحديث1</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="34" customHeight="1">
@@ -6931,13 +6909,13 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="F53" s="43" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G53" s="43" t="str">
-        <x:v>2001193-2</x:v>
+        <x:v>2001192-2</x:v>
       </x:c>
       <x:c r="H53" s="42" t="str">
-        <x:v>علوم الحديث (1)</x:v>
+        <x:v>علوم الحديث (2)</x:v>
       </x:c>
       <x:c r="I53" s="43" t="n">
         <x:v>2</x:v>
@@ -6956,7 +6934,7 @@
       </x:c>
       <x:c r="N53" s="42"/>
       <x:c r="O53" s="42" t="str">
-        <x:v>2001193-2||علومالحديث1</x:v>
+        <x:v>2001192-2||علومالحديث2</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="34" customHeight="1">
@@ -6976,16 +6954,16 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="F54" s="43" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G54" s="43" t="str">
-        <x:v>2001192-2</x:v>
+        <x:v>2001219-3</x:v>
       </x:c>
       <x:c r="H54" s="42" t="str">
-        <x:v>علوم الحديث (2)</x:v>
+        <x:v>أدلة الأحكام الشرعية (1)</x:v>
       </x:c>
       <x:c r="I54" s="43" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="J54" s="42" t="str">
         <x:v>نظري</x:v>
@@ -7001,7 +6979,7 @@
       </x:c>
       <x:c r="N54" s="42"/>
       <x:c r="O54" s="42" t="str">
-        <x:v>2001192-2||علومالحديث2</x:v>
+        <x:v>2001219-3||ادلةالاحكامالشرعية1</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="34" customHeight="1">
@@ -7024,13 +7002,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G55" s="43" t="str">
-        <x:v>2001219-3</x:v>
+        <x:v>2001231-2</x:v>
       </x:c>
       <x:c r="H55" s="42" t="str">
-        <x:v>أدلة الأحكام الشرعية (1)</x:v>
+        <x:v>أحاديث الأحكام (1)</x:v>
       </x:c>
       <x:c r="I55" s="43" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J55" s="42" t="str">
         <x:v>نظري</x:v>
@@ -7046,7 +7024,7 @@
       </x:c>
       <x:c r="N55" s="42"/>
       <x:c r="O55" s="42" t="str">
-        <x:v>2001219-3||ادلةالاحكامالشرعية1</x:v>
+        <x:v>2001231-2||احاديثالاحكام1</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="34" customHeight="1">
@@ -7066,16 +7044,16 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="F56" s="43" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G56" s="43" t="str">
-        <x:v>2001231-2</x:v>
+        <x:v>2001217-4</x:v>
       </x:c>
       <x:c r="H56" s="42" t="str">
-        <x:v>أحاديث الأحكام (1)</x:v>
+        <x:v>أدلة الأحكام الشرعية (2)</x:v>
       </x:c>
       <x:c r="I56" s="43" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="J56" s="42" t="str">
         <x:v>نظري</x:v>
@@ -7091,7 +7069,7 @@
       </x:c>
       <x:c r="N56" s="42"/>
       <x:c r="O56" s="42" t="str">
-        <x:v>2001231-2||احاديثالاحكام1</x:v>
+        <x:v>2001217-4||ادلةالاحكامالشرعية2</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="34" customHeight="1">
@@ -7114,13 +7092,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G57" s="43" t="str">
-        <x:v>2001217-4</x:v>
+        <x:v>2001218-2</x:v>
       </x:c>
       <x:c r="H57" s="42" t="str">
-        <x:v>أدلة الأحكام الشرعية (2)</x:v>
+        <x:v>قاعة بحث (تطبيقي)</x:v>
       </x:c>
       <x:c r="I57" s="43" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J57" s="42" t="str">
         <x:v>نظري</x:v>
@@ -7136,7 +7114,7 @@
       </x:c>
       <x:c r="N57" s="42"/>
       <x:c r="O57" s="42" t="str">
-        <x:v>2001217-4||ادلةالاحكامالشرعية2</x:v>
+        <x:v>2001218-2||قاعةبحثتطبيقي</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="34" customHeight="1">
@@ -7159,10 +7137,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G58" s="43" t="str">
-        <x:v>2001218-2</x:v>
+        <x:v>2001332-2</x:v>
       </x:c>
       <x:c r="H58" s="42" t="str">
-        <x:v>قاعة بحث (تطبيقي)</x:v>
+        <x:v>أحاديث الأحكام (2)</x:v>
       </x:c>
       <x:c r="I58" s="43" t="n">
         <x:v>2</x:v>
@@ -7181,7 +7159,7 @@
       </x:c>
       <x:c r="N58" s="42"/>
       <x:c r="O58" s="42" t="str">
-        <x:v>2001218-2||قاعةبحثتطبيقي</x:v>
+        <x:v>2001332-2||احاديثالاحكام2</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="34" customHeight="1">
@@ -7201,13 +7179,13 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="F59" s="43" t="n">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G59" s="43" t="str">
-        <x:v>2001332-2</x:v>
+        <x:v>2001280-2</x:v>
       </x:c>
       <x:c r="H59" s="42" t="str">
-        <x:v>أحاديث الأحكام (2)</x:v>
+        <x:v>أصول الدعوة والحسبة</x:v>
       </x:c>
       <x:c r="I59" s="43" t="n">
         <x:v>2</x:v>
@@ -7226,7 +7204,7 @@
       </x:c>
       <x:c r="N59" s="42"/>
       <x:c r="O59" s="42" t="str">
-        <x:v>2001332-2||احاديثالاحكام2</x:v>
+        <x:v>2001280-2||اصولالدعوةوالحسبة</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="34" customHeight="1">
@@ -7249,10 +7227,10 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G60" s="43" t="str">
-        <x:v>2001280-2</x:v>
+        <x:v>2001301-2</x:v>
       </x:c>
       <x:c r="H60" s="42" t="str">
-        <x:v>أصول الدعوة والحسبة</x:v>
+        <x:v>تدوين السنة</x:v>
       </x:c>
       <x:c r="I60" s="43" t="n">
         <x:v>2</x:v>
@@ -7271,7 +7249,7 @@
       </x:c>
       <x:c r="N60" s="42"/>
       <x:c r="O60" s="42" t="str">
-        <x:v>2001280-2||اصولالدعوةوالحسبة</x:v>
+        <x:v>2001301-2||تدوينالسنة</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="34" customHeight="1">
@@ -7294,10 +7272,10 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G61" s="43" t="str">
-        <x:v>2001301-2</x:v>
+        <x:v>2003243-2</x:v>
       </x:c>
       <x:c r="H61" s="42" t="str">
-        <x:v>تدوين السنة</x:v>
+        <x:v>مبادئ القانون الإداري</x:v>
       </x:c>
       <x:c r="I61" s="43" t="n">
         <x:v>2</x:v>
@@ -7316,7 +7294,7 @@
       </x:c>
       <x:c r="N61" s="42"/>
       <x:c r="O61" s="42" t="str">
-        <x:v>2001301-2||تدوينالسنة</x:v>
+        <x:v>2003243-2||مباديالقانونالاداري</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="34" customHeight="1">
@@ -7339,13 +7317,13 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G62" s="43" t="str">
-        <x:v>2003243-2</x:v>
+        <x:v>2003325-1</x:v>
       </x:c>
       <x:c r="H62" s="42" t="str">
-        <x:v>مبادئ القانون الإداري</x:v>
+        <x:v>نظام المرافعات الشرعية</x:v>
       </x:c>
       <x:c r="I62" s="43" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J62" s="42" t="str">
         <x:v>نظري</x:v>
@@ -7361,7 +7339,7 @@
       </x:c>
       <x:c r="N62" s="42"/>
       <x:c r="O62" s="42" t="str">
-        <x:v>2003243-2||مباديالقانونالاداري</x:v>
+        <x:v>2003325-1||نظامالمرافعاتالشرعية</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="34" customHeight="1">
@@ -7384,10 +7362,10 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G63" s="43" t="str">
-        <x:v>2003325-1</x:v>
+        <x:v>2003328-1</x:v>
       </x:c>
       <x:c r="H63" s="42" t="str">
-        <x:v>نظام المرافعات الشرعية</x:v>
+        <x:v>نظام الإجراءات الجزائية</x:v>
       </x:c>
       <x:c r="I63" s="43" t="n">
         <x:v>1</x:v>
@@ -7406,7 +7384,7 @@
       </x:c>
       <x:c r="N63" s="42"/>
       <x:c r="O63" s="42" t="str">
-        <x:v>2003325-1||نظامالمرافعاتالشرعية</x:v>
+        <x:v>2003328-1||نظامالاجراءاتالجزايية</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="34" customHeight="1">
@@ -7426,16 +7404,16 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="F64" s="43" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G64" s="43" t="str">
-        <x:v>2003328-1</x:v>
+        <x:v>2001493-2</x:v>
       </x:c>
       <x:c r="H64" s="42" t="str">
-        <x:v>نظام الإجراءات الجزائية</x:v>
+        <x:v>تخريج ودراسة الأسانيد</x:v>
       </x:c>
       <x:c r="I64" s="43" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J64" s="42" t="str">
         <x:v>نظري</x:v>
@@ -7451,7 +7429,7 @@
       </x:c>
       <x:c r="N64" s="42"/>
       <x:c r="O64" s="42" t="str">
-        <x:v>2003328-1||نظامالاجراءاتالجزايية</x:v>
+        <x:v>2001493-2||تخريجودراسةالاسانيد</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="34" customHeight="1">
@@ -7468,16 +7446,16 @@
         <x:v>قديمة</x:v>
       </x:c>
       <x:c r="E65" s="43" t="n">
-        <x:v>38</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="F65" s="43" t="n">
-        <x:v>7</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G65" s="43" t="str">
-        <x:v>2001493-2</x:v>
+        <x:v>2001193-2</x:v>
       </x:c>
       <x:c r="H65" s="42" t="str">
-        <x:v>تخريج ودراسة الأسانيد</x:v>
+        <x:v>علوم الحديث (1)</x:v>
       </x:c>
       <x:c r="I65" s="43" t="n">
         <x:v>2</x:v>
@@ -7489,14 +7467,14 @@
         <x:v>إجبارية القسم</x:v>
       </x:c>
       <x:c r="L65" s="42" t="str">
-        <x:v>خطط الإصدارات السابقة.pdf</x:v>
+        <x:v>الشريعة 39.pdf</x:v>
       </x:c>
       <x:c r="M65" s="42" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
       </x:c>
       <x:c r="N65" s="42"/>
       <x:c r="O65" s="42" t="str">
-        <x:v>2001493-2||تخريجودراسةالاسانيد</x:v>
+        <x:v>2001193-2||علومالحديث1</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="34" customHeight="1">
@@ -7516,13 +7494,13 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="F66" s="43" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G66" s="43" t="str">
-        <x:v>2001193-2</x:v>
+        <x:v>2001192-2</x:v>
       </x:c>
       <x:c r="H66" s="42" t="str">
-        <x:v>علوم الحديث (1)</x:v>
+        <x:v>علوم الحديث (2)</x:v>
       </x:c>
       <x:c r="I66" s="43" t="n">
         <x:v>2</x:v>
@@ -7541,7 +7519,7 @@
       </x:c>
       <x:c r="N66" s="42"/>
       <x:c r="O66" s="42" t="str">
-        <x:v>2001193-2||علومالحديث1</x:v>
+        <x:v>2001192-2||علومالحديث2</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="34" customHeight="1">
@@ -7561,16 +7539,16 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="F67" s="43" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G67" s="43" t="str">
-        <x:v>2001192-2</x:v>
+        <x:v>2001219-3</x:v>
       </x:c>
       <x:c r="H67" s="42" t="str">
-        <x:v>علوم الحديث (2)</x:v>
+        <x:v>أدلة الأحكام الشرعية (1)</x:v>
       </x:c>
       <x:c r="I67" s="43" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="J67" s="42" t="str">
         <x:v>نظري</x:v>
@@ -7586,7 +7564,7 @@
       </x:c>
       <x:c r="N67" s="42"/>
       <x:c r="O67" s="42" t="str">
-        <x:v>2001192-2||علومالحديث2</x:v>
+        <x:v>2001219-3||ادلةالاحكامالشرعية1</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="34" customHeight="1">
@@ -7609,13 +7587,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G68" s="43" t="str">
-        <x:v>2001219-3</x:v>
+        <x:v>2001231-2</x:v>
       </x:c>
       <x:c r="H68" s="42" t="str">
-        <x:v>أدلة الأحكام الشرعية (1)</x:v>
+        <x:v>أحاديث الأحكام (1)</x:v>
       </x:c>
       <x:c r="I68" s="43" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J68" s="42" t="str">
         <x:v>نظري</x:v>
@@ -7631,7 +7609,7 @@
       </x:c>
       <x:c r="N68" s="42"/>
       <x:c r="O68" s="42" t="str">
-        <x:v>2001219-3||ادلةالاحكامالشرعية1</x:v>
+        <x:v>2001231-2||احاديثالاحكام1</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="34" customHeight="1">
@@ -7651,16 +7629,16 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="F69" s="43" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G69" s="43" t="str">
-        <x:v>2001231-2</x:v>
+        <x:v>2001217-4</x:v>
       </x:c>
       <x:c r="H69" s="42" t="str">
-        <x:v>أحاديث الأحكام (1)</x:v>
+        <x:v>أدلة الأحكام الشرعية (2)</x:v>
       </x:c>
       <x:c r="I69" s="43" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="J69" s="42" t="str">
         <x:v>نظري</x:v>
@@ -7676,7 +7654,7 @@
       </x:c>
       <x:c r="N69" s="42"/>
       <x:c r="O69" s="42" t="str">
-        <x:v>2001231-2||احاديثالاحكام1</x:v>
+        <x:v>2001217-4||ادلةالاحكامالشرعية2</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="34" customHeight="1">
@@ -7699,13 +7677,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G70" s="43" t="str">
-        <x:v>2001217-4</x:v>
+        <x:v>2001332-2</x:v>
       </x:c>
       <x:c r="H70" s="42" t="str">
-        <x:v>أدلة الأحكام الشرعية (2)</x:v>
+        <x:v>أحاديث الأحكام (2)</x:v>
       </x:c>
       <x:c r="I70" s="43" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J70" s="42" t="str">
         <x:v>نظري</x:v>
@@ -7721,7 +7699,7 @@
       </x:c>
       <x:c r="N70" s="42"/>
       <x:c r="O70" s="42" t="str">
-        <x:v>2001217-4||ادلةالاحكامالشرعية2</x:v>
+        <x:v>2001332-2||احاديثالاحكام2</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="34" customHeight="1">
@@ -7744,10 +7722,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G71" s="43" t="str">
-        <x:v>2001332-2</x:v>
+        <x:v>20032202-2</x:v>
       </x:c>
       <x:c r="H71" s="42" t="str">
-        <x:v>أحاديث الأحكام (2)</x:v>
+        <x:v>المدخل إلى دراسة الأنظمة</x:v>
       </x:c>
       <x:c r="I71" s="43" t="n">
         <x:v>2</x:v>
@@ -7766,7 +7744,7 @@
       </x:c>
       <x:c r="N71" s="42"/>
       <x:c r="O71" s="42" t="str">
-        <x:v>2001332-2||احاديثالاحكام2</x:v>
+        <x:v>20032202-2||المدخلاليدراسةالانظمة</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="34" customHeight="1">
@@ -7786,13 +7764,13 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="F72" s="43" t="n">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G72" s="43" t="str">
-        <x:v>20032202-2</x:v>
+        <x:v>2001280-2</x:v>
       </x:c>
       <x:c r="H72" s="42" t="str">
-        <x:v>المدخل إلى دراسة الأنظمة</x:v>
+        <x:v>أصول الدعوة والحسبة</x:v>
       </x:c>
       <x:c r="I72" s="43" t="n">
         <x:v>2</x:v>
@@ -7811,7 +7789,7 @@
       </x:c>
       <x:c r="N72" s="42"/>
       <x:c r="O72" s="42" t="str">
-        <x:v>20032202-2||المدخلاليدراسةالانظمة</x:v>
+        <x:v>2001280-2||اصولالدعوةوالحسبة</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="34" customHeight="1">
@@ -7834,10 +7812,10 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G73" s="43" t="str">
-        <x:v>2001280-2</x:v>
+        <x:v>2001301-2</x:v>
       </x:c>
       <x:c r="H73" s="42" t="str">
-        <x:v>أصول الدعوة والحسبة</x:v>
+        <x:v>تدوين السنة</x:v>
       </x:c>
       <x:c r="I73" s="43" t="n">
         <x:v>2</x:v>
@@ -7856,7 +7834,7 @@
       </x:c>
       <x:c r="N73" s="42"/>
       <x:c r="O73" s="42" t="str">
-        <x:v>2001280-2||اصولالدعوةوالحسبة</x:v>
+        <x:v>2001301-2||تدوينالسنة</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="34" customHeight="1">
@@ -7879,13 +7857,13 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G74" s="43" t="str">
-        <x:v>2001301-2</x:v>
+        <x:v>2003325-1</x:v>
       </x:c>
       <x:c r="H74" s="42" t="str">
-        <x:v>تدوين السنة</x:v>
+        <x:v>نظام المرافعات الشرعية</x:v>
       </x:c>
       <x:c r="I74" s="43" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J74" s="42" t="str">
         <x:v>نظري</x:v>
@@ -7901,7 +7879,7 @@
       </x:c>
       <x:c r="N74" s="42"/>
       <x:c r="O74" s="42" t="str">
-        <x:v>2001301-2||تدوينالسنة</x:v>
+        <x:v>2003325-1||نظامالمرافعاتالشرعية</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="34" customHeight="1">
@@ -7924,10 +7902,10 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G75" s="43" t="str">
-        <x:v>2003325-1</x:v>
+        <x:v>2003328-1</x:v>
       </x:c>
       <x:c r="H75" s="42" t="str">
-        <x:v>نظام المرافعات الشرعية</x:v>
+        <x:v>نظام الإجراءات الجزائية</x:v>
       </x:c>
       <x:c r="I75" s="43" t="n">
         <x:v>1</x:v>
@@ -7946,7 +7924,7 @@
       </x:c>
       <x:c r="N75" s="42"/>
       <x:c r="O75" s="42" t="str">
-        <x:v>2003325-1||نظامالمرافعاتالشرعية</x:v>
+        <x:v>2003328-1||نظامالاجراءاتالجزايية</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="34" customHeight="1">
@@ -7966,16 +7944,16 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="F76" s="43" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G76" s="43" t="str">
-        <x:v>2003328-1</x:v>
+        <x:v>2001493-2</x:v>
       </x:c>
       <x:c r="H76" s="42" t="str">
-        <x:v>نظام الإجراءات الجزائية</x:v>
+        <x:v>تخريج ودراسة الأسانيد</x:v>
       </x:c>
       <x:c r="I76" s="43" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J76" s="42" t="str">
         <x:v>نظري</x:v>
@@ -7991,7 +7969,7 @@
       </x:c>
       <x:c r="N76" s="42"/>
       <x:c r="O76" s="42" t="str">
-        <x:v>2003328-1||نظامالاجراءاتالجزايية</x:v>
+        <x:v>2001493-2||تخريجودراسةالاسانيد</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="34" customHeight="1">
@@ -8011,13 +7989,13 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="F77" s="43" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G77" s="43" t="str">
-        <x:v>2001493-2</x:v>
+        <x:v>20014201-2</x:v>
       </x:c>
       <x:c r="H77" s="42" t="str">
-        <x:v>تخريج ودراسة الأسانيد</x:v>
+        <x:v>التدريبات العملية</x:v>
       </x:c>
       <x:c r="I77" s="43" t="n">
         <x:v>2</x:v>
@@ -8036,7 +8014,7 @@
       </x:c>
       <x:c r="N77" s="42"/>
       <x:c r="O77" s="42" t="str">
-        <x:v>2001493-2||تخريجودراسةالاسانيد</x:v>
+        <x:v>20014201-2||التدريباتالعملية</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="34" customHeight="1">
@@ -8044,25 +8022,25 @@
         <x:v>73</x:v>
       </x:c>
       <x:c r="B78" s="42" t="str">
-        <x:v>الشريعة</x:v>
+        <x:v>القراءات</x:v>
       </x:c>
       <x:c r="C78" s="42" t="str">
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="D78" s="42" t="str">
-        <x:v>قديمة</x:v>
+        <x:v>جديدة</x:v>
       </x:c>
       <x:c r="E78" s="43" t="n">
-        <x:v>39</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="F78" s="43" t="n">
-        <x:v>8</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G78" s="43" t="str">
-        <x:v>20014201-2</x:v>
+        <x:v>2001221-2</x:v>
       </x:c>
       <x:c r="H78" s="42" t="str">
-        <x:v>التدريبات العملية</x:v>
+        <x:v>الفقه (1)</x:v>
       </x:c>
       <x:c r="I78" s="43" t="n">
         <x:v>2</x:v>
@@ -8071,17 +8049,17 @@
         <x:v>نظري</x:v>
       </x:c>
       <x:c r="K78" s="42" t="str">
-        <x:v>إجبارية القسم</x:v>
+        <x:v>متطلبات الكلية</x:v>
       </x:c>
       <x:c r="L78" s="42" t="str">
-        <x:v>الشريعة 39.pdf</x:v>
+        <x:v>القراءات 47.pdf</x:v>
       </x:c>
       <x:c r="M78" s="42" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
       </x:c>
       <x:c r="N78" s="42"/>
       <x:c r="O78" s="42" t="str">
-        <x:v>20014201-2||التدريباتالعملية</x:v>
+        <x:v>2001221-2||الفقه1</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="34" customHeight="1">
@@ -8104,13 +8082,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G79" s="43" t="str">
-        <x:v>2001221-2</x:v>
+        <x:v>2002111-3</x:v>
       </x:c>
       <x:c r="H79" s="42" t="str">
-        <x:v>الفقه (1)</x:v>
+        <x:v>عرض القراءات السبع (١)</x:v>
       </x:c>
       <x:c r="I79" s="43" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="J79" s="42" t="str">
         <x:v>نظري</x:v>
@@ -8126,7 +8104,7 @@
       </x:c>
       <x:c r="N79" s="42"/>
       <x:c r="O79" s="42" t="str">
-        <x:v>2001221-2||الفقه1</x:v>
+        <x:v>2002111-3||عرضالقراءاتالسبع١</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="34" customHeight="1">
@@ -8149,13 +8127,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G80" s="43" t="str">
-        <x:v>2002111-3</x:v>
+        <x:v>2002280-2</x:v>
       </x:c>
       <x:c r="H80" s="42" t="str">
-        <x:v>عرض القراءات السبع (١)</x:v>
+        <x:v>تدريبات على الجمع والكيفيات</x:v>
       </x:c>
       <x:c r="I80" s="43" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J80" s="42" t="str">
         <x:v>نظري</x:v>
@@ -8171,7 +8149,7 @@
       </x:c>
       <x:c r="N80" s="42"/>
       <x:c r="O80" s="42" t="str">
-        <x:v>2002111-3||عرضالقراءاتالسبع١</x:v>
+        <x:v>2002280-2||تدريباتعليالجمعوالكيفيات</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="34" customHeight="1">
@@ -8194,10 +8172,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G81" s="43" t="str">
-        <x:v>2002280-2</x:v>
+        <x:v>2004102-2</x:v>
       </x:c>
       <x:c r="H81" s="42" t="str">
-        <x:v>تدريبات على الجمع والكيفيات</x:v>
+        <x:v>مصطلح الحديث</x:v>
       </x:c>
       <x:c r="I81" s="43" t="n">
         <x:v>2</x:v>
@@ -8216,7 +8194,7 @@
       </x:c>
       <x:c r="N81" s="42"/>
       <x:c r="O81" s="42" t="str">
-        <x:v>2002280-2||تدريباتعليالجمعوالكيفيات</x:v>
+        <x:v>2004102-2||مصطلحالحديث</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="34" customHeight="1">
@@ -8236,16 +8214,16 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="F82" s="43" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G82" s="43" t="str">
+        <x:v>2002112-3</x:v>
+      </x:c>
+      <x:c r="H82" s="42" t="str">
+        <x:v>عرض القراءات السبع (٢)</x:v>
+      </x:c>
+      <x:c r="I82" s="43" t="n">
         <x:v>3</x:v>
-      </x:c>
-      <x:c r="G82" s="43" t="str">
-        <x:v>2004102-2</x:v>
-      </x:c>
-      <x:c r="H82" s="42" t="str">
-        <x:v>مصطلح الحديث</x:v>
-      </x:c>
-      <x:c r="I82" s="43" t="n">
-        <x:v>2</x:v>
       </x:c>
       <x:c r="J82" s="42" t="str">
         <x:v>نظري</x:v>
@@ -8261,7 +8239,7 @@
       </x:c>
       <x:c r="N82" s="42"/>
       <x:c r="O82" s="42" t="str">
-        <x:v>2004102-2||مصطلحالحديث</x:v>
+        <x:v>2002112-3||عرضالقراءاتالسبع٢</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="34" customHeight="1">
@@ -8284,13 +8262,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G83" s="43" t="str">
-        <x:v>2002112-3</x:v>
+        <x:v>2002352-2</x:v>
       </x:c>
       <x:c r="H83" s="42" t="str">
-        <x:v>عرض القراءات السبع (٢)</x:v>
+        <x:v>التفسير التحليلي (2)</x:v>
       </x:c>
       <x:c r="I83" s="43" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J83" s="42" t="str">
         <x:v>نظري</x:v>
@@ -8306,7 +8284,7 @@
       </x:c>
       <x:c r="N83" s="42"/>
       <x:c r="O83" s="42" t="str">
-        <x:v>2002112-3||عرضالقراءاتالسبع٢</x:v>
+        <x:v>2002352-2||التفسيرالتحليلي2</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="34" customHeight="1">
@@ -8326,16 +8304,16 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="F84" s="43" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G84" s="43" t="str">
-        <x:v>2002352-2</x:v>
+        <x:v>2002113-3</x:v>
       </x:c>
       <x:c r="H84" s="42" t="str">
-        <x:v>التفسير التحليلي (2)</x:v>
+        <x:v>عرض القراءات السبع (٣)</x:v>
       </x:c>
       <x:c r="I84" s="43" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="J84" s="42" t="str">
         <x:v>نظري</x:v>
@@ -8351,7 +8329,7 @@
       </x:c>
       <x:c r="N84" s="42"/>
       <x:c r="O84" s="42" t="str">
-        <x:v>2002352-2||التفسيرالتحليلي2</x:v>
+        <x:v>2002113-3||عرضالقراءاتالسبع٣</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="34" customHeight="1">
@@ -8374,13 +8352,13 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G85" s="43" t="str">
-        <x:v>2002113-3</x:v>
+        <x:v>2002238-2</x:v>
       </x:c>
       <x:c r="H85" s="42" t="str">
-        <x:v>عرض القراءات السبع (٣)</x:v>
+        <x:v>الوقف والابتداء</x:v>
       </x:c>
       <x:c r="I85" s="43" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J85" s="42" t="str">
         <x:v>نظري</x:v>
@@ -8396,7 +8374,7 @@
       </x:c>
       <x:c r="N85" s="42"/>
       <x:c r="O85" s="42" t="str">
-        <x:v>2002113-3||عرضالقراءاتالسبع٣</x:v>
+        <x:v>2002238-2||الوقفوالابتداء</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="34" customHeight="1">
@@ -8419,10 +8397,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G86" s="43" t="str">
-        <x:v>2002238-2</x:v>
+        <x:v>2002239-2</x:v>
       </x:c>
       <x:c r="H86" s="42" t="str">
-        <x:v>الوقف والابتداء</x:v>
+        <x:v>مصادر ومناهج المؤلفين في القراءات</x:v>
       </x:c>
       <x:c r="I86" s="43" t="n">
         <x:v>2</x:v>
@@ -8441,7 +8419,7 @@
       </x:c>
       <x:c r="N86" s="42"/>
       <x:c r="O86" s="42" t="str">
-        <x:v>2002238-2||الوقفوالابتداء</x:v>
+        <x:v>2002239-2||مصادرومناهجالمولفينفيالقراءات</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="34" customHeight="1">
@@ -8461,16 +8439,16 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="F87" s="43" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G87" s="43" t="str">
-        <x:v>2002239-2</x:v>
+        <x:v>2002114-3</x:v>
       </x:c>
       <x:c r="H87" s="42" t="str">
-        <x:v>مصادر ومناهج المؤلفين في القراءات</x:v>
+        <x:v>عرض القراءات السبع (٤)</x:v>
       </x:c>
       <x:c r="I87" s="43" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="J87" s="42" t="str">
         <x:v>نظري</x:v>
@@ -8486,7 +8464,7 @@
       </x:c>
       <x:c r="N87" s="42"/>
       <x:c r="O87" s="42" t="str">
-        <x:v>2002239-2||مصادرومناهجالمولفينفيالقراءات</x:v>
+        <x:v>2002114-3||عرضالقراءاتالسبع٤</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="34" customHeight="1">
@@ -8509,13 +8487,13 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G88" s="43" t="str">
-        <x:v>2002114-3</x:v>
+        <x:v>2004320-2</x:v>
       </x:c>
       <x:c r="H88" s="42" t="str">
-        <x:v>عرض القراءات السبع (٤)</x:v>
+        <x:v>الحديث (3)</x:v>
       </x:c>
       <x:c r="I88" s="43" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J88" s="42" t="str">
         <x:v>نظري</x:v>
@@ -8531,7 +8509,7 @@
       </x:c>
       <x:c r="N88" s="42"/>
       <x:c r="O88" s="42" t="str">
-        <x:v>2002114-3||عرضالقراءاتالسبع٤</x:v>
+        <x:v>2004320-2||الحديث3</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="34" customHeight="1">
@@ -8551,13 +8529,13 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="F89" s="43" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G89" s="43" t="str">
-        <x:v>2004320-2</x:v>
+        <x:v>2002460-2</x:v>
       </x:c>
       <x:c r="H89" s="42" t="str">
-        <x:v>الحديث (3)</x:v>
+        <x:v>عرض القراءات الثلاث (١)</x:v>
       </x:c>
       <x:c r="I89" s="43" t="n">
         <x:v>2</x:v>
@@ -8576,7 +8554,7 @@
       </x:c>
       <x:c r="N89" s="42"/>
       <x:c r="O89" s="42" t="str">
-        <x:v>2004320-2||الحديث3</x:v>
+        <x:v>2002460-2||عرضالقراءاتالثلاث١</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="34" customHeight="1">
@@ -8596,19 +8574,19 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="F90" s="43" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G90" s="43" t="str">
-        <x:v>2002460-2</x:v>
+        <x:v>2002266-6</x:v>
       </x:c>
       <x:c r="H90" s="42" t="str">
-        <x:v>عرض القراءات الثلاث (١)</x:v>
+        <x:v>التدريب التعاوني</x:v>
       </x:c>
       <x:c r="I90" s="43" t="n">
-        <x:v>2</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="J90" s="42" t="str">
-        <x:v>نظري</x:v>
+        <x:v>تدريب</x:v>
       </x:c>
       <x:c r="K90" s="42" t="str">
         <x:v>متطلبات الكلية</x:v>
@@ -8621,7 +8599,7 @@
       </x:c>
       <x:c r="N90" s="42"/>
       <x:c r="O90" s="42" t="str">
-        <x:v>2002460-2||عرضالقراءاتالثلاث١</x:v>
+        <x:v>2002266-6||التدريبالتعاوني</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="34" customHeight="1">
@@ -8644,16 +8622,16 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G91" s="43" t="str">
-        <x:v>2002266-6</x:v>
+        <x:v>2002461-2</x:v>
       </x:c>
       <x:c r="H91" s="42" t="str">
-        <x:v>التدريب التعاوني</x:v>
+        <x:v>عرض القراءات الثلاث (٢)</x:v>
       </x:c>
       <x:c r="I91" s="43" t="n">
-        <x:v>6</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J91" s="42" t="str">
-        <x:v>تدريب</x:v>
+        <x:v>نظري</x:v>
       </x:c>
       <x:c r="K91" s="42" t="str">
         <x:v>متطلبات الكلية</x:v>
@@ -8666,7 +8644,7 @@
       </x:c>
       <x:c r="N91" s="42"/>
       <x:c r="O91" s="42" t="str">
-        <x:v>2002266-6||التدريبالتعاوني</x:v>
+        <x:v>2002461-2||عرضالقراءاتالثلاث٢</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="34" customHeight="1">
@@ -8680,19 +8658,19 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="D92" s="42" t="str">
-        <x:v>جديدة</x:v>
+        <x:v>قديمة</x:v>
       </x:c>
       <x:c r="E92" s="43" t="n">
-        <x:v>47</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="F92" s="43" t="n">
-        <x:v>8</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G92" s="43" t="str">
-        <x:v>2002461-2</x:v>
+        <x:v>2001205-2</x:v>
       </x:c>
       <x:c r="H92" s="42" t="str">
-        <x:v>عرض القراءات الثلاث (٢)</x:v>
+        <x:v>الحديث (1)</x:v>
       </x:c>
       <x:c r="I92" s="43" t="n">
         <x:v>2</x:v>
@@ -8701,17 +8679,17 @@
         <x:v>نظري</x:v>
       </x:c>
       <x:c r="K92" s="42" t="str">
-        <x:v>متطلبات الكلية</x:v>
+        <x:v>إجبارية القسم</x:v>
       </x:c>
       <x:c r="L92" s="42" t="str">
-        <x:v>القراءات 47.pdf</x:v>
+        <x:v>القراءات 38.pdf</x:v>
       </x:c>
       <x:c r="M92" s="42" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
       </x:c>
       <x:c r="N92" s="42"/>
       <x:c r="O92" s="42" t="str">
-        <x:v>2002461-2||عرضالقراءاتالثلاث٢</x:v>
+        <x:v>2001205-2||الحديث1</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="34" customHeight="1">
@@ -8734,10 +8712,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G93" s="43" t="str">
-        <x:v>2001205-2</x:v>
+        <x:v>2001221-2</x:v>
       </x:c>
       <x:c r="H93" s="42" t="str">
-        <x:v>الحديث (1)</x:v>
+        <x:v>الفقه (1)</x:v>
       </x:c>
       <x:c r="I93" s="43" t="n">
         <x:v>2</x:v>
@@ -8756,7 +8734,7 @@
       </x:c>
       <x:c r="N93" s="42"/>
       <x:c r="O93" s="42" t="str">
-        <x:v>2001205-2||الحديث1</x:v>
+        <x:v>2001221-2||الفقه1</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="34" customHeight="1">
@@ -8779,10 +8757,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G94" s="43" t="str">
-        <x:v>2001221-2</x:v>
+        <x:v>2001273-2</x:v>
       </x:c>
       <x:c r="H94" s="42" t="str">
-        <x:v>الفقه (1)</x:v>
+        <x:v>العقيدة (1)</x:v>
       </x:c>
       <x:c r="I94" s="43" t="n">
         <x:v>2</x:v>
@@ -8801,7 +8779,7 @@
       </x:c>
       <x:c r="N94" s="42"/>
       <x:c r="O94" s="42" t="str">
-        <x:v>2001221-2||الفقه1</x:v>
+        <x:v>2001273-2||العقيدة1</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="34" customHeight="1">
@@ -8821,13 +8799,13 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="F95" s="43" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G95" s="43" t="str">
-        <x:v>2001273-2</x:v>
+        <x:v>2001209-2</x:v>
       </x:c>
       <x:c r="H95" s="42" t="str">
-        <x:v>العقيدة (1)</x:v>
+        <x:v>الحديث (2)</x:v>
       </x:c>
       <x:c r="I95" s="43" t="n">
         <x:v>2</x:v>
@@ -8846,7 +8824,7 @@
       </x:c>
       <x:c r="N95" s="42"/>
       <x:c r="O95" s="42" t="str">
-        <x:v>2001273-2||العقيدة1</x:v>
+        <x:v>2001209-2||الحديث2</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="34" customHeight="1">
@@ -8869,10 +8847,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G96" s="43" t="str">
-        <x:v>2001209-2</x:v>
+        <x:v>2001322-2</x:v>
       </x:c>
       <x:c r="H96" s="42" t="str">
-        <x:v>الحديث (2)</x:v>
+        <x:v>الفقه (2)</x:v>
       </x:c>
       <x:c r="I96" s="43" t="n">
         <x:v>2</x:v>
@@ -8891,7 +8869,7 @@
       </x:c>
       <x:c r="N96" s="42"/>
       <x:c r="O96" s="42" t="str">
-        <x:v>2001209-2||الحديث2</x:v>
+        <x:v>2001322-2||الفقه2</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="34" customHeight="1">
@@ -8911,13 +8889,13 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="F97" s="43" t="n">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G97" s="43" t="str">
-        <x:v>2001322-2</x:v>
+        <x:v>2001320-2</x:v>
       </x:c>
       <x:c r="H97" s="42" t="str">
-        <x:v>الفقه (2)</x:v>
+        <x:v>الحديث (3)</x:v>
       </x:c>
       <x:c r="I97" s="43" t="n">
         <x:v>2</x:v>
@@ -8936,7 +8914,7 @@
       </x:c>
       <x:c r="N97" s="42"/>
       <x:c r="O97" s="42" t="str">
-        <x:v>2001322-2||الفقه2</x:v>
+        <x:v>2001320-2||الحديث3</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="34" customHeight="1">
@@ -8944,25 +8922,25 @@
         <x:v>93</x:v>
       </x:c>
       <x:c r="B98" s="42" t="str">
-        <x:v>القراءات</x:v>
+        <x:v>القرآن وعلومه</x:v>
       </x:c>
       <x:c r="C98" s="42" t="str">
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="D98" s="42" t="str">
-        <x:v>قديمة</x:v>
+        <x:v>جديدة</x:v>
       </x:c>
       <x:c r="E98" s="43" t="n">
-        <x:v>38</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="F98" s="43" t="n">
-        <x:v>6</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G98" s="43" t="str">
-        <x:v>2001320-2</x:v>
+        <x:v>2004102-2</x:v>
       </x:c>
       <x:c r="H98" s="42" t="str">
-        <x:v>الحديث (3)</x:v>
+        <x:v>مصطلح الحديث</x:v>
       </x:c>
       <x:c r="I98" s="43" t="n">
         <x:v>2</x:v>
@@ -8971,17 +8949,17 @@
         <x:v>نظري</x:v>
       </x:c>
       <x:c r="K98" s="42" t="str">
-        <x:v>إجبارية القسم</x:v>
+        <x:v>متطلبات الكلية</x:v>
       </x:c>
       <x:c r="L98" s="42" t="str">
-        <x:v>القراءات 38.pdf</x:v>
+        <x:v>القرآن وعلومه 47.pdf</x:v>
       </x:c>
       <x:c r="M98" s="42" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
       </x:c>
       <x:c r="N98" s="42"/>
       <x:c r="O98" s="42" t="str">
-        <x:v>2001320-2||الحديث3</x:v>
+        <x:v>2004102-2||مصطلحالحديث</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="34" customHeight="1">
@@ -9001,13 +8979,13 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="F99" s="43" t="n">
-        <x:v>2</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G99" s="43" t="str">
-        <x:v>2004102-2</x:v>
+        <x:v>2004320-2</x:v>
       </x:c>
       <x:c r="H99" s="42" t="str">
-        <x:v>مصطلح الحديث</x:v>
+        <x:v>الحديث (3)</x:v>
       </x:c>
       <x:c r="I99" s="43" t="n">
         <x:v>2</x:v>
@@ -9026,7 +9004,7 @@
       </x:c>
       <x:c r="N99" s="42"/>
       <x:c r="O99" s="42" t="str">
-        <x:v>2004102-2||مصطلحالحديث</x:v>
+        <x:v>2004320-2||الحديث3</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="34" customHeight="1">
@@ -9046,13 +9024,13 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="F100" s="43" t="n">
-        <x:v>5</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G100" s="43" t="str">
-        <x:v>2004320-2</x:v>
+        <x:v>20024101-2</x:v>
       </x:c>
       <x:c r="H100" s="42" t="str">
-        <x:v>الحديث (3)</x:v>
+        <x:v>قاعة بحث</x:v>
       </x:c>
       <x:c r="I100" s="43" t="n">
         <x:v>2</x:v>
@@ -9061,7 +9039,7 @@
         <x:v>نظري</x:v>
       </x:c>
       <x:c r="K100" s="42" t="str">
-        <x:v>متطلبات الكلية</x:v>
+        <x:v>إجبارية القسم</x:v>
       </x:c>
       <x:c r="L100" s="42" t="str">
         <x:v>القرآن وعلومه 47.pdf</x:v>
@@ -9071,7 +9049,7 @@
       </x:c>
       <x:c r="N100" s="42"/>
       <x:c r="O100" s="42" t="str">
-        <x:v>2004320-2||الحديث3</x:v>
+        <x:v>20024101-2||قاعةبحث</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="34" customHeight="1">
@@ -9091,19 +9069,19 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="F101" s="43" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G101" s="43" t="str">
-        <x:v>20024101-2</x:v>
+        <x:v>2002266-5</x:v>
       </x:c>
       <x:c r="H101" s="42" t="str">
-        <x:v>قاعة بحث</x:v>
+        <x:v>التدريب التعاوني</x:v>
       </x:c>
       <x:c r="I101" s="43" t="n">
-        <x:v>2</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="J101" s="42" t="str">
-        <x:v>نظري</x:v>
+        <x:v>تدريب</x:v>
       </x:c>
       <x:c r="K101" s="42" t="str">
         <x:v>إجبارية القسم</x:v>
@@ -9116,7 +9094,7 @@
       </x:c>
       <x:c r="N101" s="42"/>
       <x:c r="O101" s="42" t="str">
-        <x:v>20024101-2||قاعةبحث</x:v>
+        <x:v>2002266-5||التدريبالتعاوني</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="34" customHeight="1">
@@ -9130,38 +9108,38 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="D102" s="42" t="str">
-        <x:v>جديدة</x:v>
+        <x:v>قديمة</x:v>
       </x:c>
       <x:c r="E102" s="43" t="n">
-        <x:v>47</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="F102" s="43" t="n">
-        <x:v>8</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G102" s="43" t="str">
-        <x:v>2002266-5</x:v>
+        <x:v>101221-2</x:v>
       </x:c>
       <x:c r="H102" s="42" t="str">
-        <x:v>التدريب التعاوني</x:v>
+        <x:v>الفقه (1)</x:v>
       </x:c>
       <x:c r="I102" s="43" t="n">
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J102" s="42" t="str">
-        <x:v>تدريب</x:v>
+        <x:v>نظري</x:v>
       </x:c>
       <x:c r="K102" s="42" t="str">
         <x:v>إجبارية القسم</x:v>
       </x:c>
       <x:c r="L102" s="42" t="str">
-        <x:v>القرآن وعلومه 47.pdf</x:v>
+        <x:v>القرآن وعلومه 39.pdf</x:v>
       </x:c>
       <x:c r="M102" s="42" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
       </x:c>
       <x:c r="N102" s="42"/>
       <x:c r="O102" s="42" t="str">
-        <x:v>2002266-5||التدريبالتعاوني</x:v>
+        <x:v>101221-2||الفقه1</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="34" customHeight="1">
@@ -9169,25 +9147,25 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="B103" s="42" t="str">
-        <x:v>القرآن وعلومه</x:v>
+        <x:v>أصول الفقه</x:v>
       </x:c>
       <x:c r="C103" s="42" t="str">
-        <x:v>بكالوريوس</x:v>
+        <x:v>دكتوراه</x:v>
       </x:c>
       <x:c r="D103" s="42" t="str">
-        <x:v>قديمة</x:v>
+        <x:v>جديدة</x:v>
       </x:c>
       <x:c r="E103" s="43" t="n">
-        <x:v>39</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F103" s="43" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G103" s="43" t="str">
-        <x:v>101221-2</x:v>
+        <x:v>2001901-2</x:v>
       </x:c>
       <x:c r="H103" s="42" t="str">
-        <x:v>الفقه (1)</x:v>
+        <x:v>دراسات مقاصدية</x:v>
       </x:c>
       <x:c r="I103" s="43" t="n">
         <x:v>2</x:v>
@@ -9199,14 +9177,14 @@
         <x:v>إجبارية القسم</x:v>
       </x:c>
       <x:c r="L103" s="42" t="str">
-        <x:v>القرآن وعلومه 39.pdf</x:v>
+        <x:v>الدكتوراه في أصول الفقه.pdf</x:v>
       </x:c>
       <x:c r="M103" s="42" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
       </x:c>
       <x:c r="N103" s="42"/>
       <x:c r="O103" s="42" t="str">
-        <x:v>101221-2||الفقه1</x:v>
+        <x:v>2001901-2||دراساتمقاصدية</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="34" customHeight="1">
@@ -9229,13 +9207,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G104" s="43" t="str">
-        <x:v>2001901-2</x:v>
+        <x:v>2001902-3</x:v>
       </x:c>
       <x:c r="H104" s="42" t="str">
-        <x:v>دراسات مقاصدية</x:v>
+        <x:v>دراسة تحليلية أصولية</x:v>
       </x:c>
       <x:c r="I104" s="43" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="J104" s="42" t="str">
         <x:v>نظري</x:v>
@@ -9251,7 +9229,7 @@
       </x:c>
       <x:c r="N104" s="42"/>
       <x:c r="O104" s="42" t="str">
-        <x:v>2001901-2||دراساتمقاصدية</x:v>
+        <x:v>2001902-3||دراسةتحليليةاصولية</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="34" customHeight="1">
@@ -9274,13 +9252,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G105" s="43" t="str">
-        <x:v>2001902-3</x:v>
+        <x:v>2001903-4</x:v>
       </x:c>
       <x:c r="H105" s="42" t="str">
-        <x:v>دراسة تحليلية أصولية</x:v>
+        <x:v>الاجتهاد الاستدلالي والفتوى</x:v>
       </x:c>
       <x:c r="I105" s="43" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="J105" s="42" t="str">
         <x:v>نظري</x:v>
@@ -9296,7 +9274,7 @@
       </x:c>
       <x:c r="N105" s="42"/>
       <x:c r="O105" s="42" t="str">
-        <x:v>2001902-3||دراسةتحليليةاصولية</x:v>
+        <x:v>2001903-4||الاجتهادالاستدلاليوالفتوي</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="34" customHeight="1">
@@ -9304,10 +9282,10 @@
         <x:v>101</x:v>
       </x:c>
       <x:c r="B106" s="42" t="str">
-        <x:v>أصول الفقه</x:v>
+        <x:v>الفقه</x:v>
       </x:c>
       <x:c r="C106" s="42" t="str">
-        <x:v>دكتوراه</x:v>
+        <x:v>ماجستير</x:v>
       </x:c>
       <x:c r="D106" s="42" t="str">
         <x:v>جديدة</x:v>
@@ -9316,16 +9294,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F106" s="43" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G106" s="43" t="str">
-        <x:v>2001903-4</x:v>
+        <x:v>2003880-2</x:v>
       </x:c>
       <x:c r="H106" s="42" t="str">
-        <x:v>الاجتهاد الاستدلالي والفتوى</x:v>
+        <x:v>الأنظمة العدلية في السعودية</x:v>
       </x:c>
       <x:c r="I106" s="43" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J106" s="42" t="str">
         <x:v>نظري</x:v>
@@ -9334,60 +9312,32 @@
         <x:v>إجبارية القسم</x:v>
       </x:c>
       <x:c r="L106" s="42" t="str">
-        <x:v>الدكتوراه في أصول الفقه.pdf</x:v>
+        <x:v>الماجستير في الفقه.pdf</x:v>
       </x:c>
       <x:c r="M106" s="42" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
       </x:c>
       <x:c r="N106" s="42"/>
       <x:c r="O106" s="42" t="str">
-        <x:v>2001903-4||الاجتهادالاستدلاليوالفتوي</x:v>
+        <x:v>2003880-2||الانظمةالعدليةفيالسعودية</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="34" customHeight="1">
-      <x:c r="A107" s="33" t="n">
-        <x:v>102</x:v>
-      </x:c>
-      <x:c r="B107" s="42" t="str">
-        <x:v>الفقه</x:v>
-      </x:c>
-      <x:c r="C107" s="42" t="str">
-        <x:v>ماجستير</x:v>
-      </x:c>
-      <x:c r="D107" s="42" t="str">
-        <x:v>جديدة</x:v>
-      </x:c>
-      <x:c r="E107" s="43" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F107" s="43" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="G107" s="43" t="str">
-        <x:v>2003880-2</x:v>
-      </x:c>
-      <x:c r="H107" s="42" t="str">
-        <x:v>الأنظمة العدلية في السعودية</x:v>
-      </x:c>
-      <x:c r="I107" s="43" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="J107" s="42" t="str">
-        <x:v>نظري</x:v>
-      </x:c>
-      <x:c r="K107" s="42" t="str">
-        <x:v>إجبارية القسم</x:v>
-      </x:c>
-      <x:c r="L107" s="42" t="str">
-        <x:v>الماجستير في الفقه.pdf</x:v>
-      </x:c>
-      <x:c r="M107" s="42" t="str">
-        <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
-      </x:c>
+      <x:c r="A107" s="33"/>
+      <x:c r="B107" s="42"/>
+      <x:c r="C107" s="42"/>
+      <x:c r="D107" s="42"/>
+      <x:c r="E107" s="43"/>
+      <x:c r="F107" s="43"/>
+      <x:c r="G107" s="43"/>
+      <x:c r="H107" s="42"/>
+      <x:c r="I107" s="43"/>
+      <x:c r="J107" s="42"/>
+      <x:c r="K107" s="42"/>
+      <x:c r="L107" s="42"/>
+      <x:c r="M107" s="42"/>
       <x:c r="N107" s="42"/>
-      <x:c r="O107" s="42" t="str">
-        <x:v>2003880-2||الانظمةالعدليةفيالسعودية</x:v>
-      </x:c>
+      <x:c r="O107" s="42"/>
     </x:row>
     <x:row r="108" ht="34" customHeight="1">
       <x:c r="A108" s="33"/>
@@ -10042,7 +9992,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36dcf663c92e4973"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa4771fb47dc4535"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update new-plan course specifications from supplied sources
</commit_message>
<xml_diff>
--- a/قائمة_المقررات_التخصصية_المفقودة_2026-09-10.xlsx
+++ b/قائمة_المقررات_التخصصية_المفقودة_2026-09-10.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الملخص" sheetId="1" r:id="R65f444d090ce449c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="المقررات المفقودة" sheetId="2" r:id="R49a600e8d9104a13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="مواضع الخطط" sheetId="3" r:id="R40c4a15f9b4246eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الملخص" sheetId="1" r:id="R4b2b3bceb43e4f27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="المقررات المفقودة" sheetId="2" r:id="Re404f21483db43b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="مواضع الخطط" sheetId="3" r:id="Rc711a69e5aac4b45"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -274,7 +274,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="MissingCourseIdentities" displayName="MissingCourseIdentities" ref="A5:L92" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="MissingCourseIdentities" displayName="MissingCourseIdentities" ref="A5:L90" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="م"/>
     <x:tableColumn id="2" name="رمز المقرر"/>
@@ -294,7 +294,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="MissingCourseOccurrences" displayName="MissingCourseOccurrences" ref="A5:O106" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="MissingCourseOccurrences" displayName="MissingCourseOccurrences" ref="A5:O104" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="15">
     <x:tableColumn id="1" name="م"/>
     <x:tableColumn id="2" name="البرنامج"/>
@@ -551,7 +551,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>المصدر: data.json في مستودع التوصيفات، بتاريخ 2026-09-28. النطاق: رموز 200* والاستثناء القديم 101221-2، دون الرسالة والاختبار الشامل أو مقررات الأقسام الخارجية.</x:v>
+        <x:v>المصدر: data.json في مستودع التوصيفات، بتاريخ 2026-10-02. النطاق: رموز 200* والاستثناء القديم 101221-2، دون الرسالة والاختبار الشامل أو مقررات الأقسام الخارجية.</x:v>
       </x:c>
       <x:c r="B3"/>
       <x:c r="C3"/>
@@ -790,16 +790,16 @@
         <x:v>127</x:v>
       </x:c>
       <x:c r="E12" s="30" t="n">
-        <x:v>104</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="F12" s="30" t="n">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="G12" s="36" t="n">
-        <x:v>0.8188976377952756</x:v>
+        <x:v>0.8267716535433071</x:v>
       </x:c>
       <x:c r="H12" s="30" t="n">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="I12" s="33" t="str">
         <x:v>يحتاج استكمال</x:v>
@@ -819,16 +819,16 @@
         <x:v>113</x:v>
       </x:c>
       <x:c r="E13" s="30" t="n">
-        <x:v>93</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="F13" s="30" t="n">
-        <x:v>20</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="G13" s="36" t="n">
-        <x:v>0.8230088495575221</x:v>
+        <x:v>0.831858407079646</x:v>
       </x:c>
       <x:c r="H13" s="30" t="n">
-        <x:v>19</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="I13" s="33" t="str">
         <x:v>يحتاج استكمال</x:v>
@@ -1047,16 +1047,16 @@
         <x:v>756</x:v>
       </x:c>
       <x:c r="E21" s="31" t="n">
-        <x:v>655</x:v>
+        <x:v>657</x:v>
       </x:c>
       <x:c r="F21" s="31" t="n">
-        <x:v>101</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="G21" s="37" t="n">
-        <x:v>0.8664021164021164</x:v>
+        <x:v>0.8690476190476191</x:v>
       </x:c>
       <x:c r="H21" s="31" t="n">
-        <x:v>87</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="I21" s="34" t="str">
         <x:v>قائمة العمل الحالية</x:v>
@@ -1133,7 +1133,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>عدد الهويات الفريدة: 87. قد يظهر المقرر نفسه في أكثر من برنامج أو خطة، وتوضح الأعمدة جميع المواضع المتأثرة.</x:v>
+        <x:v>عدد الهويات الفريدة: 85. قد يظهر المقرر نفسه في أكثر من برنامج أو خطة، وتوضح الأعمدة جميع المواضع المتأثرة.</x:v>
       </x:c>
       <x:c r="B3"/>
       <x:c r="C3"/>
@@ -2214,10 +2214,10 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="B34" s="33" t="str">
-        <x:v>2002310-3</x:v>
+        <x:v>2004211-4</x:v>
       </x:c>
       <x:c r="C34" s="39" t="str">
-        <x:v>التفسير التحليلي (٣)</x:v>
+        <x:v>العقيدة (1)</x:v>
       </x:c>
       <x:c r="D34" s="39" t="str">
         <x:v>الدراسات الإسلامية</x:v>
@@ -2229,7 +2229,7 @@
         <x:v>الدراسات الإسلامية: جديدة 47</x:v>
       </x:c>
       <x:c r="G34" s="39" t="str">
-        <x:v>6</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H34" s="39" t="n">
         <x:v>1</x:v>
@@ -2242,7 +2242,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L34" s="39" t="str">
-        <x:v>2002310-3||التفسيرالتحليلي٣</x:v>
+        <x:v>2004211-4||العقيدة1</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="42" customHeight="1">
@@ -2250,10 +2250,10 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="B35" s="33" t="str">
-        <x:v>2004211-4</x:v>
+        <x:v>2004252-4</x:v>
       </x:c>
       <x:c r="C35" s="39" t="str">
-        <x:v>العقيدة (1)</x:v>
+        <x:v>الحديث التحليلي (1)</x:v>
       </x:c>
       <x:c r="D35" s="39" t="str">
         <x:v>الدراسات الإسلامية</x:v>
@@ -2265,7 +2265,7 @@
         <x:v>الدراسات الإسلامية: جديدة 47</x:v>
       </x:c>
       <x:c r="G35" s="39" t="str">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H35" s="39" t="n">
         <x:v>1</x:v>
@@ -2278,7 +2278,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L35" s="39" t="str">
-        <x:v>2004211-4||العقيدة1</x:v>
+        <x:v>2004252-4||الحديثالتحليلي1</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="42" customHeight="1">
@@ -2286,10 +2286,10 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="B36" s="33" t="str">
-        <x:v>2004252-4</x:v>
+        <x:v>2004256-2</x:v>
       </x:c>
       <x:c r="C36" s="39" t="str">
-        <x:v>الحديث التحليلي (1)</x:v>
+        <x:v>الحديث التحليلي (٢)</x:v>
       </x:c>
       <x:c r="D36" s="39" t="str">
         <x:v>الدراسات الإسلامية</x:v>
@@ -2301,7 +2301,7 @@
         <x:v>الدراسات الإسلامية: جديدة 47</x:v>
       </x:c>
       <x:c r="G36" s="39" t="str">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H36" s="39" t="n">
         <x:v>1</x:v>
@@ -2314,7 +2314,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L36" s="39" t="str">
-        <x:v>2004252-4||الحديثالتحليلي1</x:v>
+        <x:v>2004256-2||الحديثالتحليلي٢</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="42" customHeight="1">
@@ -2322,10 +2322,10 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="B37" s="33" t="str">
-        <x:v>2004256-2</x:v>
+        <x:v>2004262-2</x:v>
       </x:c>
       <x:c r="C37" s="39" t="str">
-        <x:v>الحديث التحليلي (٢)</x:v>
+        <x:v>الدعوة والحسبة</x:v>
       </x:c>
       <x:c r="D37" s="39" t="str">
         <x:v>الدراسات الإسلامية</x:v>
@@ -2337,7 +2337,7 @@
         <x:v>الدراسات الإسلامية: جديدة 47</x:v>
       </x:c>
       <x:c r="G37" s="39" t="str">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H37" s="39" t="n">
         <x:v>1</x:v>
@@ -2350,7 +2350,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L37" s="39" t="str">
-        <x:v>2004256-2||الحديثالتحليلي٢</x:v>
+        <x:v>2004262-2||الدعوةوالحسبة</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="42" customHeight="1">
@@ -2358,10 +2358,10 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="B38" s="33" t="str">
-        <x:v>2004262-2</x:v>
+        <x:v>2004272-2</x:v>
       </x:c>
       <x:c r="C38" s="39" t="str">
-        <x:v>الدعوة والحسبة</x:v>
+        <x:v>العمل الخيري</x:v>
       </x:c>
       <x:c r="D38" s="39" t="str">
         <x:v>الدراسات الإسلامية</x:v>
@@ -2373,7 +2373,7 @@
         <x:v>الدراسات الإسلامية: جديدة 47</x:v>
       </x:c>
       <x:c r="G38" s="39" t="str">
-        <x:v>5</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="H38" s="39" t="n">
         <x:v>1</x:v>
@@ -2386,7 +2386,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L38" s="39" t="str">
-        <x:v>2004262-2||الدعوةوالحسبة</x:v>
+        <x:v>2004272-2||العملالخيري</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="42" customHeight="1">
@@ -2394,10 +2394,10 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="B39" s="33" t="str">
-        <x:v>2004272-2</x:v>
+        <x:v>2004305-4</x:v>
       </x:c>
       <x:c r="C39" s="39" t="str">
-        <x:v>العمل الخيري</x:v>
+        <x:v>أحاديث الأحكام (١)</x:v>
       </x:c>
       <x:c r="D39" s="39" t="str">
         <x:v>الدراسات الإسلامية</x:v>
@@ -2409,7 +2409,7 @@
         <x:v>الدراسات الإسلامية: جديدة 47</x:v>
       </x:c>
       <x:c r="G39" s="39" t="str">
-        <x:v>7</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H39" s="39" t="n">
         <x:v>1</x:v>
@@ -2422,7 +2422,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L39" s="39" t="str">
-        <x:v>2004272-2||العملالخيري</x:v>
+        <x:v>2004305-4||احاديثالاحكام١</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="42" customHeight="1">
@@ -2430,10 +2430,10 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="B40" s="33" t="str">
-        <x:v>2004305-4</x:v>
+        <x:v>20013101-3</x:v>
       </x:c>
       <x:c r="C40" s="39" t="str">
-        <x:v>أحاديث الأحكام (١)</x:v>
+        <x:v>الفقه (٤)</x:v>
       </x:c>
       <x:c r="D40" s="39" t="str">
         <x:v>الدراسات الإسلامية</x:v>
@@ -2445,7 +2445,7 @@
         <x:v>الدراسات الإسلامية: جديدة 47</x:v>
       </x:c>
       <x:c r="G40" s="39" t="str">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H40" s="39" t="n">
         <x:v>1</x:v>
@@ -2458,7 +2458,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L40" s="39" t="str">
-        <x:v>2004305-4||احاديثالاحكام١</x:v>
+        <x:v>20013101-3||الفقه٤</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="42" customHeight="1">
@@ -2466,10 +2466,10 @@
         <x:v>36</x:v>
       </x:c>
       <x:c r="B41" s="33" t="str">
-        <x:v>20013101-3</x:v>
+        <x:v>20013201-4</x:v>
       </x:c>
       <x:c r="C41" s="39" t="str">
-        <x:v>الفقه (٤)</x:v>
+        <x:v>الفقه (٥)</x:v>
       </x:c>
       <x:c r="D41" s="39" t="str">
         <x:v>الدراسات الإسلامية</x:v>
@@ -2481,7 +2481,7 @@
         <x:v>الدراسات الإسلامية: جديدة 47</x:v>
       </x:c>
       <x:c r="G41" s="39" t="str">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H41" s="39" t="n">
         <x:v>1</x:v>
@@ -2494,7 +2494,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L41" s="39" t="str">
-        <x:v>20013101-3||الفقه٤</x:v>
+        <x:v>20013201-4||الفقه٥</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="42" customHeight="1">
@@ -2502,10 +2502,10 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="B42" s="33" t="str">
-        <x:v>20013201-4</x:v>
+        <x:v>20042111-2</x:v>
       </x:c>
       <x:c r="C42" s="39" t="str">
-        <x:v>الفقه (٥)</x:v>
+        <x:v>العقيدة (٢)</x:v>
       </x:c>
       <x:c r="D42" s="39" t="str">
         <x:v>الدراسات الإسلامية</x:v>
@@ -2517,7 +2517,7 @@
         <x:v>الدراسات الإسلامية: جديدة 47</x:v>
       </x:c>
       <x:c r="G42" s="39" t="str">
-        <x:v>6</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H42" s="39" t="n">
         <x:v>1</x:v>
@@ -2530,7 +2530,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L42" s="39" t="str">
-        <x:v>20013201-4||الفقه٥</x:v>
+        <x:v>20042111-2||العقيدة٢</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="42" customHeight="1">
@@ -2538,10 +2538,10 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="B43" s="33" t="str">
-        <x:v>20042111-2</x:v>
+        <x:v>20043105-2</x:v>
       </x:c>
       <x:c r="C43" s="39" t="str">
-        <x:v>العقيدة (٢)</x:v>
+        <x:v>الفقه المقارن</x:v>
       </x:c>
       <x:c r="D43" s="39" t="str">
         <x:v>الدراسات الإسلامية</x:v>
@@ -2550,10 +2550,10 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F43" s="39" t="str">
-        <x:v>الدراسات الإسلامية: جديدة 47</x:v>
+        <x:v>الدراسات الإسلامية: قديمة 39</x:v>
       </x:c>
       <x:c r="G43" s="39" t="str">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H43" s="39" t="n">
         <x:v>1</x:v>
@@ -2566,7 +2566,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L43" s="39" t="str">
-        <x:v>20042111-2||العقيدة٢</x:v>
+        <x:v>20043105-2||الفقهالمقارن</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="42" customHeight="1">
@@ -2574,10 +2574,10 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="B44" s="33" t="str">
-        <x:v>20043105-2</x:v>
+        <x:v>20043108-2</x:v>
       </x:c>
       <x:c r="C44" s="39" t="str">
-        <x:v>الفقه المقارن</x:v>
+        <x:v>علم المواريث (1)</x:v>
       </x:c>
       <x:c r="D44" s="39" t="str">
         <x:v>الدراسات الإسلامية</x:v>
@@ -2602,7 +2602,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L44" s="39" t="str">
-        <x:v>20043105-2||الفقهالمقارن</x:v>
+        <x:v>20043108-2||علمالمواريث1</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="42" customHeight="1">
@@ -2610,10 +2610,10 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="B45" s="33" t="str">
-        <x:v>20043108-2</x:v>
+        <x:v>20043109-2</x:v>
       </x:c>
       <x:c r="C45" s="39" t="str">
-        <x:v>علم المواريث (1)</x:v>
+        <x:v>دراسات في سير السلف</x:v>
       </x:c>
       <x:c r="D45" s="39" t="str">
         <x:v>الدراسات الإسلامية</x:v>
@@ -2622,7 +2622,7 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F45" s="39" t="str">
-        <x:v>الدراسات الإسلامية: قديمة 39</x:v>
+        <x:v>الدراسات الإسلامية: جديدة 47</x:v>
       </x:c>
       <x:c r="G45" s="39" t="str">
         <x:v>5</x:v>
@@ -2638,7 +2638,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L45" s="39" t="str">
-        <x:v>20043108-2||علمالمواريث1</x:v>
+        <x:v>20043109-2||دراساتفيسيرالسلف</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="42" customHeight="1">
@@ -2646,10 +2646,10 @@
         <x:v>41</x:v>
       </x:c>
       <x:c r="B46" s="33" t="str">
-        <x:v>20043109-2</x:v>
+        <x:v>20043110-2</x:v>
       </x:c>
       <x:c r="C46" s="39" t="str">
-        <x:v>دراسات في سير السلف</x:v>
+        <x:v>محاسن الإسلام</x:v>
       </x:c>
       <x:c r="D46" s="39" t="str">
         <x:v>الدراسات الإسلامية</x:v>
@@ -2674,7 +2674,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L46" s="39" t="str">
-        <x:v>20043109-2||دراساتفيسيرالسلف</x:v>
+        <x:v>20043110-2||محاسنالاسلام</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="42" customHeight="1">
@@ -2682,10 +2682,10 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="B47" s="33" t="str">
-        <x:v>20043110-2</x:v>
+        <x:v>20043111-2</x:v>
       </x:c>
       <x:c r="C47" s="39" t="str">
-        <x:v>محاسن الإسلام</x:v>
+        <x:v>الأمن الفكري</x:v>
       </x:c>
       <x:c r="D47" s="39" t="str">
         <x:v>الدراسات الإسلامية</x:v>
@@ -2697,7 +2697,7 @@
         <x:v>الدراسات الإسلامية: جديدة 47</x:v>
       </x:c>
       <x:c r="G47" s="39" t="str">
-        <x:v>5</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="H47" s="39" t="n">
         <x:v>1</x:v>
@@ -2710,7 +2710,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L47" s="39" t="str">
-        <x:v>20043110-2||محاسنالاسلام</x:v>
+        <x:v>20043111-2||الامنالفكري</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="42" customHeight="1">
@@ -2718,10 +2718,10 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="B48" s="33" t="str">
-        <x:v>20043111-2</x:v>
+        <x:v>20043202-2</x:v>
       </x:c>
       <x:c r="C48" s="39" t="str">
-        <x:v>الأمن الفكري</x:v>
+        <x:v>القواعد الفقهية</x:v>
       </x:c>
       <x:c r="D48" s="39" t="str">
         <x:v>الدراسات الإسلامية</x:v>
@@ -2730,10 +2730,10 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F48" s="39" t="str">
-        <x:v>الدراسات الإسلامية: جديدة 47</x:v>
+        <x:v>الدراسات الإسلامية: قديمة 39</x:v>
       </x:c>
       <x:c r="G48" s="39" t="str">
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H48" s="39" t="n">
         <x:v>1</x:v>
@@ -2746,7 +2746,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L48" s="39" t="str">
-        <x:v>20043111-2||الامنالفكري</x:v>
+        <x:v>20043202-2||القواعدالفقهية</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="42" customHeight="1">
@@ -2754,10 +2754,10 @@
         <x:v>44</x:v>
       </x:c>
       <x:c r="B49" s="33" t="str">
-        <x:v>20043202-2</x:v>
+        <x:v>20044101-2</x:v>
       </x:c>
       <x:c r="C49" s="39" t="str">
-        <x:v>القواعد الفقهية</x:v>
+        <x:v>أصول فقه (3)</x:v>
       </x:c>
       <x:c r="D49" s="39" t="str">
         <x:v>الدراسات الإسلامية</x:v>
@@ -2769,7 +2769,7 @@
         <x:v>الدراسات الإسلامية: قديمة 39</x:v>
       </x:c>
       <x:c r="G49" s="39" t="str">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="H49" s="39" t="n">
         <x:v>1</x:v>
@@ -2782,7 +2782,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L49" s="39" t="str">
-        <x:v>20043202-2||القواعدالفقهية</x:v>
+        <x:v>20044101-2||اصولفقه3</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="42" customHeight="1">
@@ -2790,10 +2790,10 @@
         <x:v>45</x:v>
       </x:c>
       <x:c r="B50" s="33" t="str">
-        <x:v>20044101-2</x:v>
+        <x:v>20044206-2</x:v>
       </x:c>
       <x:c r="C50" s="39" t="str">
-        <x:v>أصول فقه (3)</x:v>
+        <x:v>علم المواريث (2)</x:v>
       </x:c>
       <x:c r="D50" s="39" t="str">
         <x:v>الدراسات الإسلامية</x:v>
@@ -2805,7 +2805,7 @@
         <x:v>الدراسات الإسلامية: قديمة 39</x:v>
       </x:c>
       <x:c r="G50" s="39" t="str">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H50" s="39" t="n">
         <x:v>1</x:v>
@@ -2818,7 +2818,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L50" s="39" t="str">
-        <x:v>20044101-2||اصولفقه3</x:v>
+        <x:v>20044206-2||علمالمواريث2</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="42" customHeight="1">
@@ -2826,10 +2826,10 @@
         <x:v>46</x:v>
       </x:c>
       <x:c r="B51" s="33" t="str">
-        <x:v>20044206-2</x:v>
+        <x:v>20044220-4</x:v>
       </x:c>
       <x:c r="C51" s="39" t="str">
-        <x:v>علم المواريث (2)</x:v>
+        <x:v>التدريب التعاوني</x:v>
       </x:c>
       <x:c r="D51" s="39" t="str">
         <x:v>الدراسات الإسلامية</x:v>
@@ -2838,7 +2838,7 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F51" s="39" t="str">
-        <x:v>الدراسات الإسلامية: قديمة 39</x:v>
+        <x:v>الدراسات الإسلامية: جديدة 47</x:v>
       </x:c>
       <x:c r="G51" s="39" t="str">
         <x:v>8</x:v>
@@ -2854,7 +2854,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L51" s="39" t="str">
-        <x:v>20044206-2||علمالمواريث2</x:v>
+        <x:v>20044220-4||التدريبالتعاوني</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="42" customHeight="1">
@@ -2862,25 +2862,26 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="B52" s="33" t="str">
-        <x:v>20044220-4</x:v>
+        <x:v>2001192-2</x:v>
       </x:c>
       <x:c r="C52" s="39" t="str">
-        <x:v>التدريب التعاوني</x:v>
+        <x:v>علوم الحديث (2)</x:v>
       </x:c>
       <x:c r="D52" s="39" t="str">
-        <x:v>الدراسات الإسلامية</x:v>
+        <x:v>الشريعة</x:v>
       </x:c>
       <x:c r="E52" s="39" t="str">
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F52" s="39" t="str">
-        <x:v>الدراسات الإسلامية: جديدة 47</x:v>
+        <x:v>الشريعة: قديمة 38
+الشريعة: قديمة 39</x:v>
       </x:c>
       <x:c r="G52" s="39" t="str">
-        <x:v>8</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H52" s="39" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I52" s="39" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
@@ -2890,7 +2891,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L52" s="39" t="str">
-        <x:v>20044220-4||التدريبالتعاوني</x:v>
+        <x:v>2001192-2||علومالحديث2</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="42" customHeight="1">
@@ -2898,10 +2899,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="B53" s="33" t="str">
-        <x:v>2001192-2</x:v>
+        <x:v>2001193-2</x:v>
       </x:c>
       <x:c r="C53" s="39" t="str">
-        <x:v>علوم الحديث (2)</x:v>
+        <x:v>علوم الحديث (1)</x:v>
       </x:c>
       <x:c r="D53" s="39" t="str">
         <x:v>الشريعة</x:v>
@@ -2914,7 +2915,7 @@
 الشريعة: قديمة 39</x:v>
       </x:c>
       <x:c r="G53" s="39" t="str">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H53" s="39" t="n">
         <x:v>2</x:v>
@@ -2927,7 +2928,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L53" s="39" t="str">
-        <x:v>2001192-2||علومالحديث2</x:v>
+        <x:v>2001193-2||علومالحديث1</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="42" customHeight="1">
@@ -2935,10 +2936,10 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="B54" s="33" t="str">
-        <x:v>2001193-2</x:v>
+        <x:v>2001217-4</x:v>
       </x:c>
       <x:c r="C54" s="39" t="str">
-        <x:v>علوم الحديث (1)</x:v>
+        <x:v>أدلة الأحكام الشرعية (2)</x:v>
       </x:c>
       <x:c r="D54" s="39" t="str">
         <x:v>الشريعة</x:v>
@@ -2951,7 +2952,7 @@
 الشريعة: قديمة 39</x:v>
       </x:c>
       <x:c r="G54" s="39" t="str">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H54" s="39" t="n">
         <x:v>2</x:v>
@@ -2964,7 +2965,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L54" s="39" t="str">
-        <x:v>2001193-2||علومالحديث1</x:v>
+        <x:v>2001217-4||ادلةالاحكامالشرعية2</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="42" customHeight="1">
@@ -2972,10 +2973,10 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="B55" s="33" t="str">
-        <x:v>2001217-4</x:v>
+        <x:v>2001218-2</x:v>
       </x:c>
       <x:c r="C55" s="39" t="str">
-        <x:v>أدلة الأحكام الشرعية (2)</x:v>
+        <x:v>قاعة بحث (تطبيقي)</x:v>
       </x:c>
       <x:c r="D55" s="39" t="str">
         <x:v>الشريعة</x:v>
@@ -2984,14 +2985,13 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F55" s="39" t="str">
-        <x:v>الشريعة: قديمة 38
-الشريعة: قديمة 39</x:v>
+        <x:v>الشريعة: قديمة 38</x:v>
       </x:c>
       <x:c r="G55" s="39" t="str">
         <x:v>4</x:v>
       </x:c>
       <x:c r="H55" s="39" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I55" s="39" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
@@ -3001,7 +3001,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L55" s="39" t="str">
-        <x:v>2001217-4||ادلةالاحكامالشرعية2</x:v>
+        <x:v>2001218-2||قاعةبحثتطبيقي</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="42" customHeight="1">
@@ -3009,10 +3009,10 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="B56" s="33" t="str">
-        <x:v>2001218-2</x:v>
+        <x:v>2001219-3</x:v>
       </x:c>
       <x:c r="C56" s="39" t="str">
-        <x:v>قاعة بحث (تطبيقي)</x:v>
+        <x:v>أدلة الأحكام الشرعية (1)</x:v>
       </x:c>
       <x:c r="D56" s="39" t="str">
         <x:v>الشريعة</x:v>
@@ -3021,13 +3021,14 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F56" s="39" t="str">
-        <x:v>الشريعة: قديمة 38</x:v>
+        <x:v>الشريعة: قديمة 38
+الشريعة: قديمة 39</x:v>
       </x:c>
       <x:c r="G56" s="39" t="str">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H56" s="39" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I56" s="39" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
@@ -3037,7 +3038,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L56" s="39" t="str">
-        <x:v>2001218-2||قاعةبحثتطبيقي</x:v>
+        <x:v>2001219-3||ادلةالاحكامالشرعية1</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="42" customHeight="1">
@@ -3045,10 +3046,10 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="B57" s="33" t="str">
-        <x:v>2001219-3</x:v>
+        <x:v>2001231-2</x:v>
       </x:c>
       <x:c r="C57" s="39" t="str">
-        <x:v>أدلة الأحكام الشرعية (1)</x:v>
+        <x:v>أحاديث الأحكام (1)</x:v>
       </x:c>
       <x:c r="D57" s="39" t="str">
         <x:v>الشريعة</x:v>
@@ -3074,7 +3075,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L57" s="39" t="str">
-        <x:v>2001219-3||ادلةالاحكامالشرعية1</x:v>
+        <x:v>2001231-2||احاديثالاحكام1</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="42" customHeight="1">
@@ -3082,10 +3083,10 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="B58" s="33" t="str">
-        <x:v>2001231-2</x:v>
+        <x:v>2001280-2</x:v>
       </x:c>
       <x:c r="C58" s="39" t="str">
-        <x:v>أحاديث الأحكام (1)</x:v>
+        <x:v>أصول الدعوة والحسبة</x:v>
       </x:c>
       <x:c r="D58" s="39" t="str">
         <x:v>الشريعة</x:v>
@@ -3098,7 +3099,7 @@
 الشريعة: قديمة 39</x:v>
       </x:c>
       <x:c r="G58" s="39" t="str">
-        <x:v>3</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H58" s="39" t="n">
         <x:v>2</x:v>
@@ -3111,7 +3112,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L58" s="39" t="str">
-        <x:v>2001231-2||احاديثالاحكام1</x:v>
+        <x:v>2001280-2||اصولالدعوةوالحسبة</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="42" customHeight="1">
@@ -3119,10 +3120,10 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="B59" s="33" t="str">
-        <x:v>2001280-2</x:v>
+        <x:v>2001301-2</x:v>
       </x:c>
       <x:c r="C59" s="39" t="str">
-        <x:v>أصول الدعوة والحسبة</x:v>
+        <x:v>تدوين السنة</x:v>
       </x:c>
       <x:c r="D59" s="39" t="str">
         <x:v>الشريعة</x:v>
@@ -3148,7 +3149,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L59" s="39" t="str">
-        <x:v>2001280-2||اصولالدعوةوالحسبة</x:v>
+        <x:v>2001301-2||تدوينالسنة</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="42" customHeight="1">
@@ -3156,10 +3157,10 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="B60" s="33" t="str">
-        <x:v>2001301-2</x:v>
+        <x:v>2001332-2</x:v>
       </x:c>
       <x:c r="C60" s="39" t="str">
-        <x:v>تدوين السنة</x:v>
+        <x:v>أحاديث الأحكام (2)</x:v>
       </x:c>
       <x:c r="D60" s="39" t="str">
         <x:v>الشريعة</x:v>
@@ -3172,7 +3173,7 @@
 الشريعة: قديمة 39</x:v>
       </x:c>
       <x:c r="G60" s="39" t="str">
-        <x:v>6</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H60" s="39" t="n">
         <x:v>2</x:v>
@@ -3185,7 +3186,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L60" s="39" t="str">
-        <x:v>2001301-2||تدوينالسنة</x:v>
+        <x:v>2001332-2||احاديثالاحكام2</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="42" customHeight="1">
@@ -3193,10 +3194,10 @@
         <x:v>56</x:v>
       </x:c>
       <x:c r="B61" s="33" t="str">
-        <x:v>2001332-2</x:v>
+        <x:v>2001493-2</x:v>
       </x:c>
       <x:c r="C61" s="39" t="str">
-        <x:v>أحاديث الأحكام (2)</x:v>
+        <x:v>تخريج ودراسة الأسانيد</x:v>
       </x:c>
       <x:c r="D61" s="39" t="str">
         <x:v>الشريعة</x:v>
@@ -3209,7 +3210,7 @@
 الشريعة: قديمة 39</x:v>
       </x:c>
       <x:c r="G61" s="39" t="str">
-        <x:v>4</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="H61" s="39" t="n">
         <x:v>2</x:v>
@@ -3222,7 +3223,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L61" s="39" t="str">
-        <x:v>2001332-2||احاديثالاحكام2</x:v>
+        <x:v>2001493-2||تخريجودراسةالاسانيد</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="42" customHeight="1">
@@ -3230,10 +3231,10 @@
         <x:v>57</x:v>
       </x:c>
       <x:c r="B62" s="33" t="str">
-        <x:v>2001493-2</x:v>
+        <x:v>2003243-2</x:v>
       </x:c>
       <x:c r="C62" s="39" t="str">
-        <x:v>تخريج ودراسة الأسانيد</x:v>
+        <x:v>مبادئ القانون الإداري</x:v>
       </x:c>
       <x:c r="D62" s="39" t="str">
         <x:v>الشريعة</x:v>
@@ -3242,14 +3243,13 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F62" s="39" t="str">
-        <x:v>الشريعة: قديمة 38
-الشريعة: قديمة 39</x:v>
+        <x:v>الشريعة: قديمة 38</x:v>
       </x:c>
       <x:c r="G62" s="39" t="str">
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H62" s="39" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I62" s="39" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
@@ -3259,7 +3259,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L62" s="39" t="str">
-        <x:v>2001493-2||تخريجودراسةالاسانيد</x:v>
+        <x:v>2003243-2||مباديالقانونالاداري</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="42" customHeight="1">
@@ -3267,10 +3267,10 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="B63" s="33" t="str">
-        <x:v>2003243-2</x:v>
+        <x:v>2003325-1</x:v>
       </x:c>
       <x:c r="C63" s="39" t="str">
-        <x:v>مبادئ القانون الإداري</x:v>
+        <x:v>نظام المرافعات الشرعية</x:v>
       </x:c>
       <x:c r="D63" s="39" t="str">
         <x:v>الشريعة</x:v>
@@ -3279,13 +3279,14 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F63" s="39" t="str">
-        <x:v>الشريعة: قديمة 38</x:v>
+        <x:v>الشريعة: قديمة 38
+الشريعة: قديمة 39</x:v>
       </x:c>
       <x:c r="G63" s="39" t="str">
         <x:v>6</x:v>
       </x:c>
       <x:c r="H63" s="39" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I63" s="39" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
@@ -3295,7 +3296,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L63" s="39" t="str">
-        <x:v>2003243-2||مباديالقانونالاداري</x:v>
+        <x:v>2003325-1||نظامالمرافعاتالشرعية</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="42" customHeight="1">
@@ -3303,10 +3304,10 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="B64" s="33" t="str">
-        <x:v>2003325-1</x:v>
+        <x:v>2003328-1</x:v>
       </x:c>
       <x:c r="C64" s="39" t="str">
-        <x:v>نظام المرافعات الشرعية</x:v>
+        <x:v>نظام الإجراءات الجزائية</x:v>
       </x:c>
       <x:c r="D64" s="39" t="str">
         <x:v>الشريعة</x:v>
@@ -3332,7 +3333,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L64" s="39" t="str">
-        <x:v>2003325-1||نظامالمرافعاتالشرعية</x:v>
+        <x:v>2003328-1||نظامالاجراءاتالجزايية</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="42" customHeight="1">
@@ -3340,10 +3341,10 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="B65" s="33" t="str">
-        <x:v>2003328-1</x:v>
+        <x:v>2004301-2</x:v>
       </x:c>
       <x:c r="C65" s="39" t="str">
-        <x:v>نظام الإجراءات الجزائية</x:v>
+        <x:v>تدوين السنة</x:v>
       </x:c>
       <x:c r="D65" s="39" t="str">
         <x:v>الشريعة</x:v>
@@ -3352,14 +3353,13 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F65" s="39" t="str">
-        <x:v>الشريعة: قديمة 38
-الشريعة: قديمة 39</x:v>
+        <x:v>الشريعة: جديدة 47</x:v>
       </x:c>
       <x:c r="G65" s="39" t="str">
-        <x:v>6</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H65" s="39" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I65" s="39" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
@@ -3369,7 +3369,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L65" s="39" t="str">
-        <x:v>2003328-1||نظامالاجراءاتالجزايية</x:v>
+        <x:v>2004301-2||تدوينالسنة</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="42" customHeight="1">
@@ -3377,10 +3377,10 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="B66" s="33" t="str">
-        <x:v>2004301-2</x:v>
+        <x:v>2004476-2</x:v>
       </x:c>
       <x:c r="C66" s="39" t="str">
-        <x:v>تدوين السنة</x:v>
+        <x:v>الأديان والفرق</x:v>
       </x:c>
       <x:c r="D66" s="39" t="str">
         <x:v>الشريعة</x:v>
@@ -3392,7 +3392,7 @@
         <x:v>الشريعة: جديدة 47</x:v>
       </x:c>
       <x:c r="G66" s="39" t="str">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H66" s="39" t="n">
         <x:v>1</x:v>
@@ -3405,7 +3405,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L66" s="39" t="str">
-        <x:v>2004301-2||تدوينالسنة</x:v>
+        <x:v>2004476-2||الاديانوالفرق</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="42" customHeight="1">
@@ -3413,10 +3413,10 @@
         <x:v>62</x:v>
       </x:c>
       <x:c r="B67" s="33" t="str">
-        <x:v>2004476-2</x:v>
+        <x:v>20014201-2</x:v>
       </x:c>
       <x:c r="C67" s="39" t="str">
-        <x:v>الأديان والفرق</x:v>
+        <x:v>التدريبات العملية</x:v>
       </x:c>
       <x:c r="D67" s="39" t="str">
         <x:v>الشريعة</x:v>
@@ -3425,10 +3425,10 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F67" s="39" t="str">
-        <x:v>الشريعة: جديدة 47</x:v>
+        <x:v>الشريعة: قديمة 39</x:v>
       </x:c>
       <x:c r="G67" s="39" t="str">
-        <x:v>6</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H67" s="39" t="n">
         <x:v>1</x:v>
@@ -3441,7 +3441,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L67" s="39" t="str">
-        <x:v>2004476-2||الاديانوالفرق</x:v>
+        <x:v>20014201-2||التدريباتالعملية</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="42" customHeight="1">
@@ -3449,10 +3449,10 @@
         <x:v>63</x:v>
       </x:c>
       <x:c r="B68" s="33" t="str">
-        <x:v>20014201-2</x:v>
+        <x:v>20032202-2</x:v>
       </x:c>
       <x:c r="C68" s="39" t="str">
-        <x:v>التدريبات العملية</x:v>
+        <x:v>المدخل إلى دراسة الأنظمة</x:v>
       </x:c>
       <x:c r="D68" s="39" t="str">
         <x:v>الشريعة</x:v>
@@ -3464,7 +3464,7 @@
         <x:v>الشريعة: قديمة 39</x:v>
       </x:c>
       <x:c r="G68" s="39" t="str">
-        <x:v>8</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H68" s="39" t="n">
         <x:v>1</x:v>
@@ -3477,7 +3477,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L68" s="39" t="str">
-        <x:v>20014201-2||التدريباتالعملية</x:v>
+        <x:v>20032202-2||المدخلاليدراسةالانظمة</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="42" customHeight="1">
@@ -3485,22 +3485,22 @@
         <x:v>64</x:v>
       </x:c>
       <x:c r="B69" s="33" t="str">
-        <x:v>20032202-2</x:v>
+        <x:v>2003880-2</x:v>
       </x:c>
       <x:c r="C69" s="39" t="str">
-        <x:v>المدخل إلى دراسة الأنظمة</x:v>
+        <x:v>الأنظمة العدلية في السعودية</x:v>
       </x:c>
       <x:c r="D69" s="39" t="str">
-        <x:v>الشريعة</x:v>
+        <x:v>الفقه</x:v>
       </x:c>
       <x:c r="E69" s="39" t="str">
-        <x:v>بكالوريوس</x:v>
+        <x:v>ماجستير</x:v>
       </x:c>
       <x:c r="F69" s="39" t="str">
-        <x:v>الشريعة: قديمة 39</x:v>
+        <x:v>الفقه: جديدة 1</x:v>
       </x:c>
       <x:c r="G69" s="39" t="str">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H69" s="39" t="n">
         <x:v>1</x:v>
@@ -3513,7 +3513,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L69" s="39" t="str">
-        <x:v>20032202-2||المدخلاليدراسةالانظمة</x:v>
+        <x:v>2003880-2||الانظمةالعدليةفيالسعودية</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="42" customHeight="1">
@@ -3521,19 +3521,19 @@
         <x:v>65</x:v>
       </x:c>
       <x:c r="B70" s="33" t="str">
-        <x:v>2003880-2</x:v>
+        <x:v>2001205-2</x:v>
       </x:c>
       <x:c r="C70" s="39" t="str">
-        <x:v>الأنظمة العدلية في السعودية</x:v>
+        <x:v>الحديث (1)</x:v>
       </x:c>
       <x:c r="D70" s="39" t="str">
-        <x:v>الفقه</x:v>
+        <x:v>القراءات</x:v>
       </x:c>
       <x:c r="E70" s="39" t="str">
-        <x:v>ماجستير</x:v>
+        <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F70" s="39" t="str">
-        <x:v>الفقه: جديدة 1</x:v>
+        <x:v>القراءات: قديمة 38</x:v>
       </x:c>
       <x:c r="G70" s="39" t="str">
         <x:v>3</x:v>
@@ -3542,14 +3542,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I70" s="39" t="str">
-        <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
-      </x:c>
-      <x:c r="J70" s="39"/>
+        <x:v>يوجد توصيف مؤسسي لبرنامج القرآن وعلومه فقط</x:v>
+      </x:c>
+      <x:c r="J70" s="39" t="str">
+        <x:v>institutional-recovery-20260911/2001205-2.pdf</x:v>
+      </x:c>
       <x:c r="K70" s="39" t="str">
-        <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
+        <x:v>الحصول على دليل خاص ببرنامج القراءات، ثم ربط مخرجاته في نطاقه فقط</x:v>
       </x:c>
       <x:c r="L70" s="39" t="str">
-        <x:v>2003880-2||الانظمةالعدليةفيالسعودية</x:v>
+        <x:v>2001205-2||الحديث1</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="42" customHeight="1">
@@ -3557,10 +3559,10 @@
         <x:v>66</x:v>
       </x:c>
       <x:c r="B71" s="33" t="str">
-        <x:v>2001205-2</x:v>
+        <x:v>2001209-2</x:v>
       </x:c>
       <x:c r="C71" s="39" t="str">
-        <x:v>الحديث (1)</x:v>
+        <x:v>الحديث (2)</x:v>
       </x:c>
       <x:c r="D71" s="39" t="str">
         <x:v>القراءات</x:v>
@@ -3572,7 +3574,7 @@
         <x:v>القراءات: قديمة 38</x:v>
       </x:c>
       <x:c r="G71" s="39" t="str">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H71" s="39" t="n">
         <x:v>1</x:v>
@@ -3581,13 +3583,13 @@
         <x:v>يوجد توصيف مؤسسي لبرنامج القرآن وعلومه فقط</x:v>
       </x:c>
       <x:c r="J71" s="39" t="str">
-        <x:v>institutional-recovery-20260911/2001205-2.pdf</x:v>
+        <x:v>institutional-recovery-20260911/2001209-2.pdf</x:v>
       </x:c>
       <x:c r="K71" s="39" t="str">
         <x:v>الحصول على دليل خاص ببرنامج القراءات، ثم ربط مخرجاته في نطاقه فقط</x:v>
       </x:c>
       <x:c r="L71" s="39" t="str">
-        <x:v>2001205-2||الحديث1</x:v>
+        <x:v>2001209-2||الحديث2</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="42" customHeight="1">
@@ -3595,10 +3597,10 @@
         <x:v>67</x:v>
       </x:c>
       <x:c r="B72" s="33" t="str">
-        <x:v>2001209-2</x:v>
+        <x:v>2001221-2</x:v>
       </x:c>
       <x:c r="C72" s="39" t="str">
-        <x:v>الحديث (2)</x:v>
+        <x:v>الفقه (1)</x:v>
       </x:c>
       <x:c r="D72" s="39" t="str">
         <x:v>القراءات</x:v>
@@ -3607,25 +3609,25 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F72" s="39" t="str">
-        <x:v>القراءات: قديمة 38</x:v>
+        <x:v>القراءات: جديدة 47؛ القراءات: قديمة 38</x:v>
       </x:c>
       <x:c r="G72" s="39" t="str">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H72" s="39" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I72" s="39" t="str">
         <x:v>يوجد توصيف مؤسسي لبرنامج القرآن وعلومه فقط</x:v>
       </x:c>
       <x:c r="J72" s="39" t="str">
-        <x:v>institutional-recovery-20260911/2001209-2.pdf</x:v>
+        <x:v>institutional-recovery-20260911/2001221-2.pdf</x:v>
       </x:c>
       <x:c r="K72" s="39" t="str">
         <x:v>الحصول على دليل خاص ببرنامج القراءات، ثم ربط مخرجاته في نطاقه فقط</x:v>
       </x:c>
       <x:c r="L72" s="39" t="str">
-        <x:v>2001209-2||الحديث2</x:v>
+        <x:v>2001221-2||الفقه1</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="42" customHeight="1">
@@ -3633,10 +3635,10 @@
         <x:v>68</x:v>
       </x:c>
       <x:c r="B73" s="33" t="str">
-        <x:v>2001221-2</x:v>
+        <x:v>2001273-2</x:v>
       </x:c>
       <x:c r="C73" s="39" t="str">
-        <x:v>الفقه (1)</x:v>
+        <x:v>العقيدة (1)</x:v>
       </x:c>
       <x:c r="D73" s="39" t="str">
         <x:v>القراءات</x:v>
@@ -3645,25 +3647,23 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F73" s="39" t="str">
-        <x:v>القراءات: جديدة 47؛ القراءات: قديمة 38</x:v>
+        <x:v>القراءات: قديمة 38</x:v>
       </x:c>
       <x:c r="G73" s="39" t="str">
         <x:v>3</x:v>
       </x:c>
       <x:c r="H73" s="39" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I73" s="39" t="str">
-        <x:v>يوجد توصيف مؤسسي لبرنامج القرآن وعلومه فقط</x:v>
-      </x:c>
-      <x:c r="J73" s="39" t="str">
-        <x:v>institutional-recovery-20260911/2001221-2.pdf</x:v>
-      </x:c>
+        <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
+      </x:c>
+      <x:c r="J73" s="39"/>
       <x:c r="K73" s="39" t="str">
-        <x:v>الحصول على دليل خاص ببرنامج القراءات، ثم ربط مخرجاته في نطاقه فقط</x:v>
+        <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L73" s="39" t="str">
-        <x:v>2001221-2||الفقه1</x:v>
+        <x:v>2001273-2||العقيدة1</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="42" customHeight="1">
@@ -3671,10 +3671,10 @@
         <x:v>69</x:v>
       </x:c>
       <x:c r="B74" s="33" t="str">
-        <x:v>2001273-2</x:v>
+        <x:v>2001320-2</x:v>
       </x:c>
       <x:c r="C74" s="39" t="str">
-        <x:v>العقيدة (1)</x:v>
+        <x:v>الحديث (3)</x:v>
       </x:c>
       <x:c r="D74" s="39" t="str">
         <x:v>القراءات</x:v>
@@ -3686,20 +3686,22 @@
         <x:v>القراءات: قديمة 38</x:v>
       </x:c>
       <x:c r="G74" s="39" t="str">
-        <x:v>3</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H74" s="39" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="I74" s="39" t="str">
-        <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
-      </x:c>
-      <x:c r="J74" s="39"/>
+        <x:v>يوجد توصيف مؤسسي لبرنامج القرآن وعلومه فقط</x:v>
+      </x:c>
+      <x:c r="J74" s="39" t="str">
+        <x:v>institutional-recovery-20260911/2001320-2.pdf</x:v>
+      </x:c>
       <x:c r="K74" s="39" t="str">
-        <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
+        <x:v>الحصول على دليل خاص ببرنامج القراءات، ثم ربط مخرجاته في نطاقه فقط</x:v>
       </x:c>
       <x:c r="L74" s="39" t="str">
-        <x:v>2001273-2||العقيدة1</x:v>
+        <x:v>2001320-2||الحديث3</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="42" customHeight="1">
@@ -3707,10 +3709,10 @@
         <x:v>70</x:v>
       </x:c>
       <x:c r="B75" s="33" t="str">
-        <x:v>2001320-2</x:v>
+        <x:v>2001322-2</x:v>
       </x:c>
       <x:c r="C75" s="39" t="str">
-        <x:v>الحديث (3)</x:v>
+        <x:v>الفقه (2)</x:v>
       </x:c>
       <x:c r="D75" s="39" t="str">
         <x:v>القراءات</x:v>
@@ -3722,7 +3724,7 @@
         <x:v>القراءات: قديمة 38</x:v>
       </x:c>
       <x:c r="G75" s="39" t="str">
-        <x:v>6</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H75" s="39" t="n">
         <x:v>1</x:v>
@@ -3731,13 +3733,13 @@
         <x:v>يوجد توصيف مؤسسي لبرنامج القرآن وعلومه فقط</x:v>
       </x:c>
       <x:c r="J75" s="39" t="str">
-        <x:v>institutional-recovery-20260911/2001320-2.pdf</x:v>
+        <x:v>institutional-recovery-20260911/2001322-2.pdf</x:v>
       </x:c>
       <x:c r="K75" s="39" t="str">
         <x:v>الحصول على دليل خاص ببرنامج القراءات، ثم ربط مخرجاته في نطاقه فقط</x:v>
       </x:c>
       <x:c r="L75" s="39" t="str">
-        <x:v>2001320-2||الحديث3</x:v>
+        <x:v>2001322-2||الفقه2</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="42" customHeight="1">
@@ -3745,10 +3747,10 @@
         <x:v>71</x:v>
       </x:c>
       <x:c r="B76" s="33" t="str">
-        <x:v>2001322-2</x:v>
+        <x:v>2002111-3</x:v>
       </x:c>
       <x:c r="C76" s="39" t="str">
-        <x:v>الفقه (2)</x:v>
+        <x:v>عرض القراءات السبع (١)</x:v>
       </x:c>
       <x:c r="D76" s="39" t="str">
         <x:v>القراءات</x:v>
@@ -3757,25 +3759,23 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F76" s="39" t="str">
-        <x:v>القراءات: قديمة 38</x:v>
+        <x:v>القراءات: جديدة 47</x:v>
       </x:c>
       <x:c r="G76" s="39" t="str">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H76" s="39" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="I76" s="39" t="str">
-        <x:v>يوجد توصيف مؤسسي لبرنامج القرآن وعلومه فقط</x:v>
-      </x:c>
-      <x:c r="J76" s="39" t="str">
-        <x:v>institutional-recovery-20260911/2001322-2.pdf</x:v>
-      </x:c>
+        <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
+      </x:c>
+      <x:c r="J76" s="39"/>
       <x:c r="K76" s="39" t="str">
-        <x:v>الحصول على دليل خاص ببرنامج القراءات، ثم ربط مخرجاته في نطاقه فقط</x:v>
+        <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L76" s="39" t="str">
-        <x:v>2001322-2||الفقه2</x:v>
+        <x:v>2002111-3||عرضالقراءاتالسبع١</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="42" customHeight="1">
@@ -3783,10 +3783,10 @@
         <x:v>72</x:v>
       </x:c>
       <x:c r="B77" s="33" t="str">
-        <x:v>2002111-3</x:v>
+        <x:v>2002112-3</x:v>
       </x:c>
       <x:c r="C77" s="39" t="str">
-        <x:v>عرض القراءات السبع (١)</x:v>
+        <x:v>عرض القراءات السبع (٢)</x:v>
       </x:c>
       <x:c r="D77" s="39" t="str">
         <x:v>القراءات</x:v>
@@ -3798,7 +3798,7 @@
         <x:v>القراءات: جديدة 47</x:v>
       </x:c>
       <x:c r="G77" s="39" t="str">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H77" s="39" t="n">
         <x:v>1</x:v>
@@ -3811,7 +3811,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L77" s="39" t="str">
-        <x:v>2002111-3||عرضالقراءاتالسبع١</x:v>
+        <x:v>2002112-3||عرضالقراءاتالسبع٢</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="42" customHeight="1">
@@ -3819,10 +3819,10 @@
         <x:v>73</x:v>
       </x:c>
       <x:c r="B78" s="33" t="str">
-        <x:v>2002112-3</x:v>
+        <x:v>2002113-3</x:v>
       </x:c>
       <x:c r="C78" s="39" t="str">
-        <x:v>عرض القراءات السبع (٢)</x:v>
+        <x:v>عرض القراءات السبع (٣)</x:v>
       </x:c>
       <x:c r="D78" s="39" t="str">
         <x:v>القراءات</x:v>
@@ -3834,7 +3834,7 @@
         <x:v>القراءات: جديدة 47</x:v>
       </x:c>
       <x:c r="G78" s="39" t="str">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H78" s="39" t="n">
         <x:v>1</x:v>
@@ -3847,7 +3847,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L78" s="39" t="str">
-        <x:v>2002112-3||عرضالقراءاتالسبع٢</x:v>
+        <x:v>2002113-3||عرضالقراءاتالسبع٣</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="42" customHeight="1">
@@ -3855,10 +3855,10 @@
         <x:v>74</x:v>
       </x:c>
       <x:c r="B79" s="33" t="str">
-        <x:v>2002113-3</x:v>
+        <x:v>2002114-3</x:v>
       </x:c>
       <x:c r="C79" s="39" t="str">
-        <x:v>عرض القراءات السبع (٣)</x:v>
+        <x:v>عرض القراءات السبع (٤)</x:v>
       </x:c>
       <x:c r="D79" s="39" t="str">
         <x:v>القراءات</x:v>
@@ -3870,7 +3870,7 @@
         <x:v>القراءات: جديدة 47</x:v>
       </x:c>
       <x:c r="G79" s="39" t="str">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H79" s="39" t="n">
         <x:v>1</x:v>
@@ -3883,7 +3883,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L79" s="39" t="str">
-        <x:v>2002113-3||عرضالقراءاتالسبع٣</x:v>
+        <x:v>2002114-3||عرضالقراءاتالسبع٤</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="42" customHeight="1">
@@ -3891,10 +3891,10 @@
         <x:v>75</x:v>
       </x:c>
       <x:c r="B80" s="33" t="str">
-        <x:v>2002114-3</x:v>
+        <x:v>2002238-2</x:v>
       </x:c>
       <x:c r="C80" s="39" t="str">
-        <x:v>عرض القراءات السبع (٤)</x:v>
+        <x:v>الوقف والابتداء</x:v>
       </x:c>
       <x:c r="D80" s="39" t="str">
         <x:v>القراءات</x:v>
@@ -3906,7 +3906,7 @@
         <x:v>القراءات: جديدة 47</x:v>
       </x:c>
       <x:c r="G80" s="39" t="str">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="H80" s="39" t="n">
         <x:v>1</x:v>
@@ -3919,7 +3919,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L80" s="39" t="str">
-        <x:v>2002114-3||عرضالقراءاتالسبع٤</x:v>
+        <x:v>2002238-2||الوقفوالابتداء</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="42" customHeight="1">
@@ -3927,10 +3927,10 @@
         <x:v>76</x:v>
       </x:c>
       <x:c r="B81" s="33" t="str">
-        <x:v>2002238-2</x:v>
+        <x:v>2002239-2</x:v>
       </x:c>
       <x:c r="C81" s="39" t="str">
-        <x:v>الوقف والابتداء</x:v>
+        <x:v>مصادر ومناهج المؤلفين في القراءات</x:v>
       </x:c>
       <x:c r="D81" s="39" t="str">
         <x:v>القراءات</x:v>
@@ -3955,7 +3955,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L81" s="39" t="str">
-        <x:v>2002238-2||الوقفوالابتداء</x:v>
+        <x:v>2002239-2||مصادرومناهجالمولفينفيالقراءات</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="42" customHeight="1">
@@ -3963,10 +3963,10 @@
         <x:v>77</x:v>
       </x:c>
       <x:c r="B82" s="33" t="str">
-        <x:v>2002239-2</x:v>
+        <x:v>2002266-6</x:v>
       </x:c>
       <x:c r="C82" s="39" t="str">
-        <x:v>مصادر ومناهج المؤلفين في القراءات</x:v>
+        <x:v>التدريب التعاوني</x:v>
       </x:c>
       <x:c r="D82" s="39" t="str">
         <x:v>القراءات</x:v>
@@ -3978,7 +3978,7 @@
         <x:v>القراءات: جديدة 47</x:v>
       </x:c>
       <x:c r="G82" s="39" t="str">
-        <x:v>5</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H82" s="39" t="n">
         <x:v>1</x:v>
@@ -3991,7 +3991,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L82" s="39" t="str">
-        <x:v>2002239-2||مصادرومناهجالمولفينفيالقراءات</x:v>
+        <x:v>2002266-6||التدريبالتعاوني</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="42" customHeight="1">
@@ -3999,10 +3999,10 @@
         <x:v>78</x:v>
       </x:c>
       <x:c r="B83" s="33" t="str">
-        <x:v>2002266-6</x:v>
+        <x:v>2002280-2</x:v>
       </x:c>
       <x:c r="C83" s="39" t="str">
-        <x:v>التدريب التعاوني</x:v>
+        <x:v>تدريبات على الجمع والكيفيات</x:v>
       </x:c>
       <x:c r="D83" s="39" t="str">
         <x:v>القراءات</x:v>
@@ -4014,7 +4014,7 @@
         <x:v>القراءات: جديدة 47</x:v>
       </x:c>
       <x:c r="G83" s="39" t="str">
-        <x:v>8</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H83" s="39" t="n">
         <x:v>1</x:v>
@@ -4027,7 +4027,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L83" s="39" t="str">
-        <x:v>2002266-6||التدريبالتعاوني</x:v>
+        <x:v>2002280-2||تدريباتعليالجمعوالكيفيات</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="42" customHeight="1">
@@ -4035,10 +4035,10 @@
         <x:v>79</x:v>
       </x:c>
       <x:c r="B84" s="33" t="str">
-        <x:v>2002280-2</x:v>
+        <x:v>2002460-2</x:v>
       </x:c>
       <x:c r="C84" s="39" t="str">
-        <x:v>تدريبات على الجمع والكيفيات</x:v>
+        <x:v>عرض القراءات الثلاث (١)</x:v>
       </x:c>
       <x:c r="D84" s="39" t="str">
         <x:v>القراءات</x:v>
@@ -4050,7 +4050,7 @@
         <x:v>القراءات: جديدة 47</x:v>
       </x:c>
       <x:c r="G84" s="39" t="str">
-        <x:v>3</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="H84" s="39" t="n">
         <x:v>1</x:v>
@@ -4063,7 +4063,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L84" s="39" t="str">
-        <x:v>2002280-2||تدريباتعليالجمعوالكيفيات</x:v>
+        <x:v>2002460-2||عرضالقراءاتالثلاث١</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="42" customHeight="1">
@@ -4071,10 +4071,10 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="B85" s="33" t="str">
-        <x:v>2002352-2</x:v>
+        <x:v>2002461-2</x:v>
       </x:c>
       <x:c r="C85" s="39" t="str">
-        <x:v>التفسير التحليلي (2)</x:v>
+        <x:v>عرض القراءات الثلاث (٢)</x:v>
       </x:c>
       <x:c r="D85" s="39" t="str">
         <x:v>القراءات</x:v>
@@ -4086,7 +4086,7 @@
         <x:v>القراءات: جديدة 47</x:v>
       </x:c>
       <x:c r="G85" s="39" t="str">
-        <x:v>4</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H85" s="39" t="n">
         <x:v>1</x:v>
@@ -4099,7 +4099,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L85" s="39" t="str">
-        <x:v>2002352-2||التفسيرالتحليلي2</x:v>
+        <x:v>2002461-2||عرضالقراءاتالثلاث٢</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="42" customHeight="1">
@@ -4107,25 +4107,26 @@
         <x:v>81</x:v>
       </x:c>
       <x:c r="B86" s="33" t="str">
-        <x:v>2002460-2</x:v>
+        <x:v>2004102-2</x:v>
       </x:c>
       <x:c r="C86" s="39" t="str">
-        <x:v>عرض القراءات الثلاث (١)</x:v>
+        <x:v>مصطلح الحديث</x:v>
       </x:c>
       <x:c r="D86" s="39" t="str">
-        <x:v>القراءات</x:v>
+        <x:v>القراءات، القرآن وعلومه</x:v>
       </x:c>
       <x:c r="E86" s="39" t="str">
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F86" s="39" t="str">
-        <x:v>القراءات: جديدة 47</x:v>
+        <x:v>القراءات: جديدة 47
+القرآن وعلومه: جديدة 47</x:v>
       </x:c>
       <x:c r="G86" s="39" t="str">
-        <x:v>7</x:v>
+        <x:v>2، 3</x:v>
       </x:c>
       <x:c r="H86" s="39" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I86" s="39" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
@@ -4135,7 +4136,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L86" s="39" t="str">
-        <x:v>2002460-2||عرضالقراءاتالثلاث١</x:v>
+        <x:v>2004102-2||مصطلحالحديث</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="42" customHeight="1">
@@ -4143,25 +4144,26 @@
         <x:v>82</x:v>
       </x:c>
       <x:c r="B87" s="33" t="str">
-        <x:v>2002461-2</x:v>
+        <x:v>2004320-2</x:v>
       </x:c>
       <x:c r="C87" s="39" t="str">
-        <x:v>عرض القراءات الثلاث (٢)</x:v>
+        <x:v>الحديث (3)</x:v>
       </x:c>
       <x:c r="D87" s="39" t="str">
-        <x:v>القراءات</x:v>
+        <x:v>القراءات، القرآن وعلومه</x:v>
       </x:c>
       <x:c r="E87" s="39" t="str">
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F87" s="39" t="str">
-        <x:v>القراءات: جديدة 47</x:v>
+        <x:v>القراءات: جديدة 47
+القرآن وعلومه: جديدة 47</x:v>
       </x:c>
       <x:c r="G87" s="39" t="str">
-        <x:v>8</x:v>
+        <x:v>5، 6</x:v>
       </x:c>
       <x:c r="H87" s="39" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I87" s="39" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
@@ -4171,7 +4173,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L87" s="39" t="str">
-        <x:v>2002461-2||عرضالقراءاتالثلاث٢</x:v>
+        <x:v>2004320-2||الحديث3</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="42" customHeight="1">
@@ -4179,26 +4181,25 @@
         <x:v>83</x:v>
       </x:c>
       <x:c r="B88" s="33" t="str">
-        <x:v>2004102-2</x:v>
+        <x:v>101221-2</x:v>
       </x:c>
       <x:c r="C88" s="39" t="str">
-        <x:v>مصطلح الحديث</x:v>
+        <x:v>الفقه (1)</x:v>
       </x:c>
       <x:c r="D88" s="39" t="str">
-        <x:v>القراءات، القرآن وعلومه</x:v>
+        <x:v>القرآن وعلومه</x:v>
       </x:c>
       <x:c r="E88" s="39" t="str">
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F88" s="39" t="str">
-        <x:v>القراءات: جديدة 47
-القرآن وعلومه: جديدة 47</x:v>
+        <x:v>القرآن وعلومه: قديمة 39</x:v>
       </x:c>
       <x:c r="G88" s="39" t="str">
-        <x:v>2، 3</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H88" s="39" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I88" s="39" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
@@ -4208,7 +4209,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L88" s="39" t="str">
-        <x:v>2004102-2||مصطلحالحديث</x:v>
+        <x:v>101221-2||الفقه1</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="42" customHeight="1">
@@ -4216,26 +4217,25 @@
         <x:v>84</x:v>
       </x:c>
       <x:c r="B89" s="33" t="str">
-        <x:v>2004320-2</x:v>
+        <x:v>2002266-5</x:v>
       </x:c>
       <x:c r="C89" s="39" t="str">
-        <x:v>الحديث (3)</x:v>
+        <x:v>التدريب التعاوني</x:v>
       </x:c>
       <x:c r="D89" s="39" t="str">
-        <x:v>القراءات، القرآن وعلومه</x:v>
+        <x:v>القرآن وعلومه</x:v>
       </x:c>
       <x:c r="E89" s="39" t="str">
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F89" s="39" t="str">
-        <x:v>القراءات: جديدة 47
-القرآن وعلومه: جديدة 47</x:v>
+        <x:v>القرآن وعلومه: جديدة 47</x:v>
       </x:c>
       <x:c r="G89" s="39" t="str">
-        <x:v>5، 6</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H89" s="39" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I89" s="39" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
@@ -4245,7 +4245,7 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L89" s="39" t="str">
-        <x:v>2004320-2||الحديث3</x:v>
+        <x:v>2002266-5||التدريبالتعاوني</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="42" customHeight="1">
@@ -4253,10 +4253,10 @@
         <x:v>85</x:v>
       </x:c>
       <x:c r="B90" s="33" t="str">
-        <x:v>101221-2</x:v>
+        <x:v>20024101-2</x:v>
       </x:c>
       <x:c r="C90" s="39" t="str">
-        <x:v>الفقه (1)</x:v>
+        <x:v>قاعة بحث</x:v>
       </x:c>
       <x:c r="D90" s="39" t="str">
         <x:v>القرآن وعلومه</x:v>
@@ -4265,10 +4265,10 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="F90" s="39" t="str">
-        <x:v>القرآن وعلومه: قديمة 39</x:v>
+        <x:v>القرآن وعلومه: جديدة 47</x:v>
       </x:c>
       <x:c r="G90" s="39" t="str">
-        <x:v>3</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="H90" s="39" t="n">
         <x:v>1</x:v>
@@ -4281,80 +4281,36 @@
         <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
       </x:c>
       <x:c r="L90" s="39" t="str">
-        <x:v>101221-2||الفقه1</x:v>
+        <x:v>20024101-2||قاعةبحث</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="42" customHeight="1">
-      <x:c r="A91" s="33" t="n">
-        <x:v>86</x:v>
-      </x:c>
-      <x:c r="B91" s="33" t="str">
-        <x:v>2002266-5</x:v>
-      </x:c>
-      <x:c r="C91" s="39" t="str">
-        <x:v>التدريب التعاوني</x:v>
-      </x:c>
-      <x:c r="D91" s="39" t="str">
-        <x:v>القرآن وعلومه</x:v>
-      </x:c>
-      <x:c r="E91" s="39" t="str">
-        <x:v>بكالوريوس</x:v>
-      </x:c>
-      <x:c r="F91" s="39" t="str">
-        <x:v>القرآن وعلومه: جديدة 47</x:v>
-      </x:c>
-      <x:c r="G91" s="39" t="str">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="H91" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I91" s="39" t="str">
-        <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
-      </x:c>
+      <x:c r="A91" s="33"/>
+      <x:c r="B91" s="33"/>
+      <x:c r="C91" s="39"/>
+      <x:c r="D91" s="39"/>
+      <x:c r="E91" s="39"/>
+      <x:c r="F91" s="39"/>
+      <x:c r="G91" s="39"/>
+      <x:c r="H91" s="39"/>
+      <x:c r="I91" s="39"/>
       <x:c r="J91" s="39"/>
-      <x:c r="K91" s="39" t="str">
-        <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
-      </x:c>
-      <x:c r="L91" s="39" t="str">
-        <x:v>2002266-5||التدريبالتعاوني</x:v>
-      </x:c>
+      <x:c r="K91" s="39"/>
+      <x:c r="L91" s="39"/>
     </x:row>
     <x:row r="92" ht="42" customHeight="1">
-      <x:c r="A92" s="33" t="n">
-        <x:v>87</x:v>
-      </x:c>
-      <x:c r="B92" s="33" t="str">
-        <x:v>20024101-2</x:v>
-      </x:c>
-      <x:c r="C92" s="39" t="str">
-        <x:v>قاعة بحث</x:v>
-      </x:c>
-      <x:c r="D92" s="39" t="str">
-        <x:v>القرآن وعلومه</x:v>
-      </x:c>
-      <x:c r="E92" s="39" t="str">
-        <x:v>بكالوريوس</x:v>
-      </x:c>
-      <x:c r="F92" s="39" t="str">
-        <x:v>القرآن وعلومه: جديدة 47</x:v>
-      </x:c>
-      <x:c r="G92" s="39" t="str">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="H92" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I92" s="39" t="str">
-        <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
-      </x:c>
+      <x:c r="A92" s="33"/>
+      <x:c r="B92" s="33"/>
+      <x:c r="C92" s="39"/>
+      <x:c r="D92" s="39"/>
+      <x:c r="E92" s="39"/>
+      <x:c r="F92" s="39"/>
+      <x:c r="G92" s="39"/>
+      <x:c r="H92" s="39"/>
+      <x:c r="I92" s="39"/>
       <x:c r="J92" s="39"/>
-      <x:c r="K92" s="39" t="str">
-        <x:v>الحصول على توصيف صالح، ثم التحقق من الهوية وربط مخرجات كل برنامج على حدة</x:v>
-      </x:c>
-      <x:c r="L92" s="39" t="str">
-        <x:v>20024101-2||قاعةبحث</x:v>
-      </x:c>
+      <x:c r="K92" s="39"/>
+      <x:c r="L92" s="39"/>
     </x:row>
     <x:row r="93" ht="42" customHeight="1">
       <x:c r="A93" s="33"/>
@@ -4629,7 +4585,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R447243e16813405a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8429400768fb43d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4696,7 +4652,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>عدد المواضع: 101. كل صف يمثل ظهور مقرر في برنامج وخطة وإصدار محدد.</x:v>
+        <x:v>عدد المواضع: 99. كل صف يمثل ظهور مقرر في برنامج وخطة وإصدار محدد.</x:v>
       </x:c>
       <x:c r="B3"/>
       <x:c r="C3"/>
@@ -6282,13 +6238,13 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G39" s="43" t="str">
-        <x:v>2002310-3</x:v>
+        <x:v>20013201-4</x:v>
       </x:c>
       <x:c r="H39" s="42" t="str">
-        <x:v>التفسير التحليلي (٣)</x:v>
+        <x:v>الفقه (٥)</x:v>
       </x:c>
       <x:c r="I39" s="43" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="J39" s="42" t="str">
         <x:v>نظري</x:v>
@@ -6304,7 +6260,7 @@
       </x:c>
       <x:c r="N39" s="42"/>
       <x:c r="O39" s="42" t="str">
-        <x:v>2002310-3||التفسيرالتحليلي٣</x:v>
+        <x:v>20013201-4||الفقه٥</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="34" customHeight="1">
@@ -6324,16 +6280,16 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="F40" s="43" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G40" s="43" t="str">
-        <x:v>20013201-4</x:v>
+        <x:v>2004272-2</x:v>
       </x:c>
       <x:c r="H40" s="42" t="str">
-        <x:v>الفقه (٥)</x:v>
+        <x:v>العمل الخيري</x:v>
       </x:c>
       <x:c r="I40" s="43" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J40" s="42" t="str">
         <x:v>نظري</x:v>
@@ -6349,7 +6305,7 @@
       </x:c>
       <x:c r="N40" s="42"/>
       <x:c r="O40" s="42" t="str">
-        <x:v>20013201-4||الفقه٥</x:v>
+        <x:v>2004272-2||العملالخيري</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="34" customHeight="1">
@@ -6372,10 +6328,10 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="G41" s="43" t="str">
-        <x:v>2004272-2</x:v>
+        <x:v>20043111-2</x:v>
       </x:c>
       <x:c r="H41" s="42" t="str">
-        <x:v>العمل الخيري</x:v>
+        <x:v>الأمن الفكري</x:v>
       </x:c>
       <x:c r="I41" s="43" t="n">
         <x:v>2</x:v>
@@ -6384,7 +6340,7 @@
         <x:v>نظري</x:v>
       </x:c>
       <x:c r="K41" s="42" t="str">
-        <x:v>إجبارية القسم</x:v>
+        <x:v>اختيارية القسم</x:v>
       </x:c>
       <x:c r="L41" s="42" t="str">
         <x:v>الإسلامية 47.pdf</x:v>
@@ -6394,7 +6350,7 @@
       </x:c>
       <x:c r="N41" s="42"/>
       <x:c r="O41" s="42" t="str">
-        <x:v>2004272-2||العملالخيري</x:v>
+        <x:v>20043111-2||الامنالفكري</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="34" customHeight="1">
@@ -6414,13 +6370,13 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="F42" s="43" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G42" s="43" t="str">
-        <x:v>20043111-2</x:v>
+        <x:v>2001270-2</x:v>
       </x:c>
       <x:c r="H42" s="42" t="str">
-        <x:v>الأمن الفكري</x:v>
+        <x:v>فقه النوازل</x:v>
       </x:c>
       <x:c r="I42" s="43" t="n">
         <x:v>2</x:v>
@@ -6429,7 +6385,7 @@
         <x:v>نظري</x:v>
       </x:c>
       <x:c r="K42" s="42" t="str">
-        <x:v>اختيارية القسم</x:v>
+        <x:v>إجبارية القسم</x:v>
       </x:c>
       <x:c r="L42" s="42" t="str">
         <x:v>الإسلامية 47.pdf</x:v>
@@ -6439,7 +6395,7 @@
       </x:c>
       <x:c r="N42" s="42"/>
       <x:c r="O42" s="42" t="str">
-        <x:v>20043111-2||الامنالفكري</x:v>
+        <x:v>2001270-2||فقهالنوازل</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="34" customHeight="1">
@@ -6462,16 +6418,16 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="G43" s="43" t="str">
-        <x:v>2001270-2</x:v>
+        <x:v>20044220-4</x:v>
       </x:c>
       <x:c r="H43" s="42" t="str">
-        <x:v>فقه النوازل</x:v>
+        <x:v>التدريب التعاوني</x:v>
       </x:c>
       <x:c r="I43" s="43" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="J43" s="42" t="str">
-        <x:v>نظري</x:v>
+        <x:v>تدريب</x:v>
       </x:c>
       <x:c r="K43" s="42" t="str">
         <x:v>إجبارية القسم</x:v>
@@ -6484,7 +6440,7 @@
       </x:c>
       <x:c r="N43" s="42"/>
       <x:c r="O43" s="42" t="str">
-        <x:v>2001270-2||فقهالنوازل</x:v>
+        <x:v>20044220-4||التدريبالتعاوني</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="34" customHeight="1">
@@ -6498,38 +6454,38 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="D44" s="42" t="str">
-        <x:v>جديدة</x:v>
+        <x:v>قديمة</x:v>
       </x:c>
       <x:c r="E44" s="43" t="n">
-        <x:v>47</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="F44" s="43" t="n">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G44" s="43" t="str">
-        <x:v>20044220-4</x:v>
+        <x:v>20043105-2</x:v>
       </x:c>
       <x:c r="H44" s="42" t="str">
-        <x:v>التدريب التعاوني</x:v>
+        <x:v>الفقه المقارن</x:v>
       </x:c>
       <x:c r="I44" s="43" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J44" s="42" t="str">
-        <x:v>تدريب</x:v>
+        <x:v>نظري</x:v>
       </x:c>
       <x:c r="K44" s="42" t="str">
         <x:v>إجبارية القسم</x:v>
       </x:c>
       <x:c r="L44" s="42" t="str">
-        <x:v>الإسلامية 47.pdf</x:v>
+        <x:v>الدراسات الإسلامية 39.pdf</x:v>
       </x:c>
       <x:c r="M44" s="42" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
       </x:c>
       <x:c r="N44" s="42"/>
       <x:c r="O44" s="42" t="str">
-        <x:v>20044220-4||التدريبالتعاوني</x:v>
+        <x:v>20043105-2||الفقهالمقارن</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="34" customHeight="1">
@@ -6552,10 +6508,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G45" s="43" t="str">
-        <x:v>20043105-2</x:v>
+        <x:v>20043108-2</x:v>
       </x:c>
       <x:c r="H45" s="42" t="str">
-        <x:v>الفقه المقارن</x:v>
+        <x:v>علم المواريث (1)</x:v>
       </x:c>
       <x:c r="I45" s="43" t="n">
         <x:v>2</x:v>
@@ -6574,7 +6530,7 @@
       </x:c>
       <x:c r="N45" s="42"/>
       <x:c r="O45" s="42" t="str">
-        <x:v>20043105-2||الفقهالمقارن</x:v>
+        <x:v>20043108-2||علمالمواريث1</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="34" customHeight="1">
@@ -6594,13 +6550,13 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="F46" s="43" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G46" s="43" t="str">
-        <x:v>20043108-2</x:v>
+        <x:v>20043202-2</x:v>
       </x:c>
       <x:c r="H46" s="42" t="str">
-        <x:v>علم المواريث (1)</x:v>
+        <x:v>القواعد الفقهية</x:v>
       </x:c>
       <x:c r="I46" s="43" t="n">
         <x:v>2</x:v>
@@ -6619,7 +6575,7 @@
       </x:c>
       <x:c r="N46" s="42"/>
       <x:c r="O46" s="42" t="str">
-        <x:v>20043108-2||علمالمواريث1</x:v>
+        <x:v>20043202-2||القواعدالفقهية</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="34" customHeight="1">
@@ -6639,13 +6595,13 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="F47" s="43" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G47" s="43" t="str">
-        <x:v>20043202-2</x:v>
+        <x:v>20044101-2</x:v>
       </x:c>
       <x:c r="H47" s="42" t="str">
-        <x:v>القواعد الفقهية</x:v>
+        <x:v>أصول فقه (3)</x:v>
       </x:c>
       <x:c r="I47" s="43" t="n">
         <x:v>2</x:v>
@@ -6664,7 +6620,7 @@
       </x:c>
       <x:c r="N47" s="42"/>
       <x:c r="O47" s="42" t="str">
-        <x:v>20043202-2||القواعدالفقهية</x:v>
+        <x:v>20044101-2||اصولفقه3</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="34" customHeight="1">
@@ -6684,13 +6640,13 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="F48" s="43" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G48" s="43" t="str">
-        <x:v>20044101-2</x:v>
+        <x:v>20044206-2</x:v>
       </x:c>
       <x:c r="H48" s="42" t="str">
-        <x:v>أصول فقه (3)</x:v>
+        <x:v>علم المواريث (2)</x:v>
       </x:c>
       <x:c r="I48" s="43" t="n">
         <x:v>2</x:v>
@@ -6709,7 +6665,7 @@
       </x:c>
       <x:c r="N48" s="42"/>
       <x:c r="O48" s="42" t="str">
-        <x:v>20044101-2||اصولفقه3</x:v>
+        <x:v>20044206-2||علمالمواريث2</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="34" customHeight="1">
@@ -6717,25 +6673,25 @@
         <x:v>44</x:v>
       </x:c>
       <x:c r="B49" s="42" t="str">
-        <x:v>الدراسات الإسلامية</x:v>
+        <x:v>الشريعة</x:v>
       </x:c>
       <x:c r="C49" s="42" t="str">
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="D49" s="42" t="str">
-        <x:v>قديمة</x:v>
+        <x:v>جديدة</x:v>
       </x:c>
       <x:c r="E49" s="43" t="n">
-        <x:v>39</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="F49" s="43" t="n">
-        <x:v>8</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G49" s="43" t="str">
-        <x:v>20044206-2</x:v>
+        <x:v>2004301-2</x:v>
       </x:c>
       <x:c r="H49" s="42" t="str">
-        <x:v>علم المواريث (2)</x:v>
+        <x:v>تدوين السنة</x:v>
       </x:c>
       <x:c r="I49" s="43" t="n">
         <x:v>2</x:v>
@@ -6744,17 +6700,17 @@
         <x:v>نظري</x:v>
       </x:c>
       <x:c r="K49" s="42" t="str">
-        <x:v>إجبارية القسم</x:v>
+        <x:v>متطلبات الكلية</x:v>
       </x:c>
       <x:c r="L49" s="42" t="str">
-        <x:v>الدراسات الإسلامية 39.pdf</x:v>
+        <x:v>الشريعة 47.pdf</x:v>
       </x:c>
       <x:c r="M49" s="42" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
       </x:c>
       <x:c r="N49" s="42"/>
       <x:c r="O49" s="42" t="str">
-        <x:v>20044206-2||علمالمواريث2</x:v>
+        <x:v>2004301-2||تدوينالسنة</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="34" customHeight="1">
@@ -6774,13 +6730,13 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="F50" s="43" t="n">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G50" s="43" t="str">
-        <x:v>2004301-2</x:v>
+        <x:v>2004476-2</x:v>
       </x:c>
       <x:c r="H50" s="42" t="str">
-        <x:v>تدوين السنة</x:v>
+        <x:v>الأديان والفرق</x:v>
       </x:c>
       <x:c r="I50" s="43" t="n">
         <x:v>2</x:v>
@@ -6799,7 +6755,7 @@
       </x:c>
       <x:c r="N50" s="42"/>
       <x:c r="O50" s="42" t="str">
-        <x:v>2004301-2||تدوينالسنة</x:v>
+        <x:v>2004476-2||الاديانوالفرق</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="34" customHeight="1">
@@ -6813,19 +6769,19 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="D51" s="42" t="str">
-        <x:v>جديدة</x:v>
+        <x:v>قديمة</x:v>
       </x:c>
       <x:c r="E51" s="43" t="n">
-        <x:v>47</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="F51" s="43" t="n">
-        <x:v>6</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G51" s="43" t="str">
-        <x:v>2004476-2</x:v>
+        <x:v>2001193-2</x:v>
       </x:c>
       <x:c r="H51" s="42" t="str">
-        <x:v>الأديان والفرق</x:v>
+        <x:v>علوم الحديث (1)</x:v>
       </x:c>
       <x:c r="I51" s="43" t="n">
         <x:v>2</x:v>
@@ -6834,17 +6790,17 @@
         <x:v>نظري</x:v>
       </x:c>
       <x:c r="K51" s="42" t="str">
-        <x:v>متطلبات الكلية</x:v>
+        <x:v>إجبارية القسم</x:v>
       </x:c>
       <x:c r="L51" s="42" t="str">
-        <x:v>الشريعة 47.pdf</x:v>
+        <x:v>خطط الإصدارات السابقة.pdf</x:v>
       </x:c>
       <x:c r="M51" s="42" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
       </x:c>
       <x:c r="N51" s="42"/>
       <x:c r="O51" s="42" t="str">
-        <x:v>2004476-2||الاديانوالفرق</x:v>
+        <x:v>2001193-2||علومالحديث1</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="34" customHeight="1">
@@ -6864,13 +6820,13 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="F52" s="43" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G52" s="43" t="str">
-        <x:v>2001193-2</x:v>
+        <x:v>2001192-2</x:v>
       </x:c>
       <x:c r="H52" s="42" t="str">
-        <x:v>علوم الحديث (1)</x:v>
+        <x:v>علوم الحديث (2)</x:v>
       </x:c>
       <x:c r="I52" s="43" t="n">
         <x:v>2</x:v>
@@ -6889,7 +6845,7 @@
       </x:c>
       <x:c r="N52" s="42"/>
       <x:c r="O52" s="42" t="str">
-        <x:v>2001193-2||علومالحديث1</x:v>
+        <x:v>2001192-2||علومالحديث2</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="34" customHeight="1">
@@ -6909,16 +6865,16 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="F53" s="43" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G53" s="43" t="str">
-        <x:v>2001192-2</x:v>
+        <x:v>2001219-3</x:v>
       </x:c>
       <x:c r="H53" s="42" t="str">
-        <x:v>علوم الحديث (2)</x:v>
+        <x:v>أدلة الأحكام الشرعية (1)</x:v>
       </x:c>
       <x:c r="I53" s="43" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="J53" s="42" t="str">
         <x:v>نظري</x:v>
@@ -6934,7 +6890,7 @@
       </x:c>
       <x:c r="N53" s="42"/>
       <x:c r="O53" s="42" t="str">
-        <x:v>2001192-2||علومالحديث2</x:v>
+        <x:v>2001219-3||ادلةالاحكامالشرعية1</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="34" customHeight="1">
@@ -6957,13 +6913,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G54" s="43" t="str">
-        <x:v>2001219-3</x:v>
+        <x:v>2001231-2</x:v>
       </x:c>
       <x:c r="H54" s="42" t="str">
-        <x:v>أدلة الأحكام الشرعية (1)</x:v>
+        <x:v>أحاديث الأحكام (1)</x:v>
       </x:c>
       <x:c r="I54" s="43" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J54" s="42" t="str">
         <x:v>نظري</x:v>
@@ -6979,7 +6935,7 @@
       </x:c>
       <x:c r="N54" s="42"/>
       <x:c r="O54" s="42" t="str">
-        <x:v>2001219-3||ادلةالاحكامالشرعية1</x:v>
+        <x:v>2001231-2||احاديثالاحكام1</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="34" customHeight="1">
@@ -6999,16 +6955,16 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="F55" s="43" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G55" s="43" t="str">
-        <x:v>2001231-2</x:v>
+        <x:v>2001217-4</x:v>
       </x:c>
       <x:c r="H55" s="42" t="str">
-        <x:v>أحاديث الأحكام (1)</x:v>
+        <x:v>أدلة الأحكام الشرعية (2)</x:v>
       </x:c>
       <x:c r="I55" s="43" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="J55" s="42" t="str">
         <x:v>نظري</x:v>
@@ -7024,7 +6980,7 @@
       </x:c>
       <x:c r="N55" s="42"/>
       <x:c r="O55" s="42" t="str">
-        <x:v>2001231-2||احاديثالاحكام1</x:v>
+        <x:v>2001217-4||ادلةالاحكامالشرعية2</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="34" customHeight="1">
@@ -7047,13 +7003,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G56" s="43" t="str">
-        <x:v>2001217-4</x:v>
+        <x:v>2001218-2</x:v>
       </x:c>
       <x:c r="H56" s="42" t="str">
-        <x:v>أدلة الأحكام الشرعية (2)</x:v>
+        <x:v>قاعة بحث (تطبيقي)</x:v>
       </x:c>
       <x:c r="I56" s="43" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J56" s="42" t="str">
         <x:v>نظري</x:v>
@@ -7069,7 +7025,7 @@
       </x:c>
       <x:c r="N56" s="42"/>
       <x:c r="O56" s="42" t="str">
-        <x:v>2001217-4||ادلةالاحكامالشرعية2</x:v>
+        <x:v>2001218-2||قاعةبحثتطبيقي</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="34" customHeight="1">
@@ -7092,10 +7048,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G57" s="43" t="str">
-        <x:v>2001218-2</x:v>
+        <x:v>2001332-2</x:v>
       </x:c>
       <x:c r="H57" s="42" t="str">
-        <x:v>قاعة بحث (تطبيقي)</x:v>
+        <x:v>أحاديث الأحكام (2)</x:v>
       </x:c>
       <x:c r="I57" s="43" t="n">
         <x:v>2</x:v>
@@ -7114,7 +7070,7 @@
       </x:c>
       <x:c r="N57" s="42"/>
       <x:c r="O57" s="42" t="str">
-        <x:v>2001218-2||قاعةبحثتطبيقي</x:v>
+        <x:v>2001332-2||احاديثالاحكام2</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="34" customHeight="1">
@@ -7134,13 +7090,13 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="F58" s="43" t="n">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G58" s="43" t="str">
-        <x:v>2001332-2</x:v>
+        <x:v>2001280-2</x:v>
       </x:c>
       <x:c r="H58" s="42" t="str">
-        <x:v>أحاديث الأحكام (2)</x:v>
+        <x:v>أصول الدعوة والحسبة</x:v>
       </x:c>
       <x:c r="I58" s="43" t="n">
         <x:v>2</x:v>
@@ -7159,7 +7115,7 @@
       </x:c>
       <x:c r="N58" s="42"/>
       <x:c r="O58" s="42" t="str">
-        <x:v>2001332-2||احاديثالاحكام2</x:v>
+        <x:v>2001280-2||اصولالدعوةوالحسبة</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="34" customHeight="1">
@@ -7182,10 +7138,10 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G59" s="43" t="str">
-        <x:v>2001280-2</x:v>
+        <x:v>2001301-2</x:v>
       </x:c>
       <x:c r="H59" s="42" t="str">
-        <x:v>أصول الدعوة والحسبة</x:v>
+        <x:v>تدوين السنة</x:v>
       </x:c>
       <x:c r="I59" s="43" t="n">
         <x:v>2</x:v>
@@ -7204,7 +7160,7 @@
       </x:c>
       <x:c r="N59" s="42"/>
       <x:c r="O59" s="42" t="str">
-        <x:v>2001280-2||اصولالدعوةوالحسبة</x:v>
+        <x:v>2001301-2||تدوينالسنة</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="34" customHeight="1">
@@ -7227,10 +7183,10 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G60" s="43" t="str">
-        <x:v>2001301-2</x:v>
+        <x:v>2003243-2</x:v>
       </x:c>
       <x:c r="H60" s="42" t="str">
-        <x:v>تدوين السنة</x:v>
+        <x:v>مبادئ القانون الإداري</x:v>
       </x:c>
       <x:c r="I60" s="43" t="n">
         <x:v>2</x:v>
@@ -7249,7 +7205,7 @@
       </x:c>
       <x:c r="N60" s="42"/>
       <x:c r="O60" s="42" t="str">
-        <x:v>2001301-2||تدوينالسنة</x:v>
+        <x:v>2003243-2||مباديالقانونالاداري</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="34" customHeight="1">
@@ -7272,13 +7228,13 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G61" s="43" t="str">
-        <x:v>2003243-2</x:v>
+        <x:v>2003325-1</x:v>
       </x:c>
       <x:c r="H61" s="42" t="str">
-        <x:v>مبادئ القانون الإداري</x:v>
+        <x:v>نظام المرافعات الشرعية</x:v>
       </x:c>
       <x:c r="I61" s="43" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J61" s="42" t="str">
         <x:v>نظري</x:v>
@@ -7294,7 +7250,7 @@
       </x:c>
       <x:c r="N61" s="42"/>
       <x:c r="O61" s="42" t="str">
-        <x:v>2003243-2||مباديالقانونالاداري</x:v>
+        <x:v>2003325-1||نظامالمرافعاتالشرعية</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="34" customHeight="1">
@@ -7317,10 +7273,10 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G62" s="43" t="str">
-        <x:v>2003325-1</x:v>
+        <x:v>2003328-1</x:v>
       </x:c>
       <x:c r="H62" s="42" t="str">
-        <x:v>نظام المرافعات الشرعية</x:v>
+        <x:v>نظام الإجراءات الجزائية</x:v>
       </x:c>
       <x:c r="I62" s="43" t="n">
         <x:v>1</x:v>
@@ -7339,7 +7295,7 @@
       </x:c>
       <x:c r="N62" s="42"/>
       <x:c r="O62" s="42" t="str">
-        <x:v>2003325-1||نظامالمرافعاتالشرعية</x:v>
+        <x:v>2003328-1||نظامالاجراءاتالجزايية</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="34" customHeight="1">
@@ -7359,16 +7315,16 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="F63" s="43" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G63" s="43" t="str">
-        <x:v>2003328-1</x:v>
+        <x:v>2001493-2</x:v>
       </x:c>
       <x:c r="H63" s="42" t="str">
-        <x:v>نظام الإجراءات الجزائية</x:v>
+        <x:v>تخريج ودراسة الأسانيد</x:v>
       </x:c>
       <x:c r="I63" s="43" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J63" s="42" t="str">
         <x:v>نظري</x:v>
@@ -7384,7 +7340,7 @@
       </x:c>
       <x:c r="N63" s="42"/>
       <x:c r="O63" s="42" t="str">
-        <x:v>2003328-1||نظامالاجراءاتالجزايية</x:v>
+        <x:v>2001493-2||تخريجودراسةالاسانيد</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="34" customHeight="1">
@@ -7401,16 +7357,16 @@
         <x:v>قديمة</x:v>
       </x:c>
       <x:c r="E64" s="43" t="n">
-        <x:v>38</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="F64" s="43" t="n">
-        <x:v>7</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G64" s="43" t="str">
-        <x:v>2001493-2</x:v>
+        <x:v>2001193-2</x:v>
       </x:c>
       <x:c r="H64" s="42" t="str">
-        <x:v>تخريج ودراسة الأسانيد</x:v>
+        <x:v>علوم الحديث (1)</x:v>
       </x:c>
       <x:c r="I64" s="43" t="n">
         <x:v>2</x:v>
@@ -7422,14 +7378,14 @@
         <x:v>إجبارية القسم</x:v>
       </x:c>
       <x:c r="L64" s="42" t="str">
-        <x:v>خطط الإصدارات السابقة.pdf</x:v>
+        <x:v>الشريعة 39.pdf</x:v>
       </x:c>
       <x:c r="M64" s="42" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
       </x:c>
       <x:c r="N64" s="42"/>
       <x:c r="O64" s="42" t="str">
-        <x:v>2001493-2||تخريجودراسةالاسانيد</x:v>
+        <x:v>2001193-2||علومالحديث1</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="34" customHeight="1">
@@ -7449,13 +7405,13 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="F65" s="43" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G65" s="43" t="str">
-        <x:v>2001193-2</x:v>
+        <x:v>2001192-2</x:v>
       </x:c>
       <x:c r="H65" s="42" t="str">
-        <x:v>علوم الحديث (1)</x:v>
+        <x:v>علوم الحديث (2)</x:v>
       </x:c>
       <x:c r="I65" s="43" t="n">
         <x:v>2</x:v>
@@ -7474,7 +7430,7 @@
       </x:c>
       <x:c r="N65" s="42"/>
       <x:c r="O65" s="42" t="str">
-        <x:v>2001193-2||علومالحديث1</x:v>
+        <x:v>2001192-2||علومالحديث2</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="34" customHeight="1">
@@ -7494,16 +7450,16 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="F66" s="43" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G66" s="43" t="str">
-        <x:v>2001192-2</x:v>
+        <x:v>2001219-3</x:v>
       </x:c>
       <x:c r="H66" s="42" t="str">
-        <x:v>علوم الحديث (2)</x:v>
+        <x:v>أدلة الأحكام الشرعية (1)</x:v>
       </x:c>
       <x:c r="I66" s="43" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="J66" s="42" t="str">
         <x:v>نظري</x:v>
@@ -7519,7 +7475,7 @@
       </x:c>
       <x:c r="N66" s="42"/>
       <x:c r="O66" s="42" t="str">
-        <x:v>2001192-2||علومالحديث2</x:v>
+        <x:v>2001219-3||ادلةالاحكامالشرعية1</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="34" customHeight="1">
@@ -7542,13 +7498,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G67" s="43" t="str">
-        <x:v>2001219-3</x:v>
+        <x:v>2001231-2</x:v>
       </x:c>
       <x:c r="H67" s="42" t="str">
-        <x:v>أدلة الأحكام الشرعية (1)</x:v>
+        <x:v>أحاديث الأحكام (1)</x:v>
       </x:c>
       <x:c r="I67" s="43" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J67" s="42" t="str">
         <x:v>نظري</x:v>
@@ -7564,7 +7520,7 @@
       </x:c>
       <x:c r="N67" s="42"/>
       <x:c r="O67" s="42" t="str">
-        <x:v>2001219-3||ادلةالاحكامالشرعية1</x:v>
+        <x:v>2001231-2||احاديثالاحكام1</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="34" customHeight="1">
@@ -7584,16 +7540,16 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="F68" s="43" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G68" s="43" t="str">
-        <x:v>2001231-2</x:v>
+        <x:v>2001217-4</x:v>
       </x:c>
       <x:c r="H68" s="42" t="str">
-        <x:v>أحاديث الأحكام (1)</x:v>
+        <x:v>أدلة الأحكام الشرعية (2)</x:v>
       </x:c>
       <x:c r="I68" s="43" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="J68" s="42" t="str">
         <x:v>نظري</x:v>
@@ -7609,7 +7565,7 @@
       </x:c>
       <x:c r="N68" s="42"/>
       <x:c r="O68" s="42" t="str">
-        <x:v>2001231-2||احاديثالاحكام1</x:v>
+        <x:v>2001217-4||ادلةالاحكامالشرعية2</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="34" customHeight="1">
@@ -7632,13 +7588,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G69" s="43" t="str">
-        <x:v>2001217-4</x:v>
+        <x:v>2001332-2</x:v>
       </x:c>
       <x:c r="H69" s="42" t="str">
-        <x:v>أدلة الأحكام الشرعية (2)</x:v>
+        <x:v>أحاديث الأحكام (2)</x:v>
       </x:c>
       <x:c r="I69" s="43" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J69" s="42" t="str">
         <x:v>نظري</x:v>
@@ -7654,7 +7610,7 @@
       </x:c>
       <x:c r="N69" s="42"/>
       <x:c r="O69" s="42" t="str">
-        <x:v>2001217-4||ادلةالاحكامالشرعية2</x:v>
+        <x:v>2001332-2||احاديثالاحكام2</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="34" customHeight="1">
@@ -7677,10 +7633,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G70" s="43" t="str">
-        <x:v>2001332-2</x:v>
+        <x:v>20032202-2</x:v>
       </x:c>
       <x:c r="H70" s="42" t="str">
-        <x:v>أحاديث الأحكام (2)</x:v>
+        <x:v>المدخل إلى دراسة الأنظمة</x:v>
       </x:c>
       <x:c r="I70" s="43" t="n">
         <x:v>2</x:v>
@@ -7699,7 +7655,7 @@
       </x:c>
       <x:c r="N70" s="42"/>
       <x:c r="O70" s="42" t="str">
-        <x:v>2001332-2||احاديثالاحكام2</x:v>
+        <x:v>20032202-2||المدخلاليدراسةالانظمة</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="34" customHeight="1">
@@ -7719,13 +7675,13 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="F71" s="43" t="n">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G71" s="43" t="str">
-        <x:v>20032202-2</x:v>
+        <x:v>2001280-2</x:v>
       </x:c>
       <x:c r="H71" s="42" t="str">
-        <x:v>المدخل إلى دراسة الأنظمة</x:v>
+        <x:v>أصول الدعوة والحسبة</x:v>
       </x:c>
       <x:c r="I71" s="43" t="n">
         <x:v>2</x:v>
@@ -7744,7 +7700,7 @@
       </x:c>
       <x:c r="N71" s="42"/>
       <x:c r="O71" s="42" t="str">
-        <x:v>20032202-2||المدخلاليدراسةالانظمة</x:v>
+        <x:v>2001280-2||اصولالدعوةوالحسبة</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="34" customHeight="1">
@@ -7767,10 +7723,10 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G72" s="43" t="str">
-        <x:v>2001280-2</x:v>
+        <x:v>2001301-2</x:v>
       </x:c>
       <x:c r="H72" s="42" t="str">
-        <x:v>أصول الدعوة والحسبة</x:v>
+        <x:v>تدوين السنة</x:v>
       </x:c>
       <x:c r="I72" s="43" t="n">
         <x:v>2</x:v>
@@ -7789,7 +7745,7 @@
       </x:c>
       <x:c r="N72" s="42"/>
       <x:c r="O72" s="42" t="str">
-        <x:v>2001280-2||اصولالدعوةوالحسبة</x:v>
+        <x:v>2001301-2||تدوينالسنة</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="34" customHeight="1">
@@ -7812,13 +7768,13 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G73" s="43" t="str">
-        <x:v>2001301-2</x:v>
+        <x:v>2003325-1</x:v>
       </x:c>
       <x:c r="H73" s="42" t="str">
-        <x:v>تدوين السنة</x:v>
+        <x:v>نظام المرافعات الشرعية</x:v>
       </x:c>
       <x:c r="I73" s="43" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J73" s="42" t="str">
         <x:v>نظري</x:v>
@@ -7834,7 +7790,7 @@
       </x:c>
       <x:c r="N73" s="42"/>
       <x:c r="O73" s="42" t="str">
-        <x:v>2001301-2||تدوينالسنة</x:v>
+        <x:v>2003325-1||نظامالمرافعاتالشرعية</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="34" customHeight="1">
@@ -7857,10 +7813,10 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G74" s="43" t="str">
-        <x:v>2003325-1</x:v>
+        <x:v>2003328-1</x:v>
       </x:c>
       <x:c r="H74" s="42" t="str">
-        <x:v>نظام المرافعات الشرعية</x:v>
+        <x:v>نظام الإجراءات الجزائية</x:v>
       </x:c>
       <x:c r="I74" s="43" t="n">
         <x:v>1</x:v>
@@ -7879,7 +7835,7 @@
       </x:c>
       <x:c r="N74" s="42"/>
       <x:c r="O74" s="42" t="str">
-        <x:v>2003325-1||نظامالمرافعاتالشرعية</x:v>
+        <x:v>2003328-1||نظامالاجراءاتالجزايية</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="34" customHeight="1">
@@ -7899,16 +7855,16 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="F75" s="43" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G75" s="43" t="str">
-        <x:v>2003328-1</x:v>
+        <x:v>2001493-2</x:v>
       </x:c>
       <x:c r="H75" s="42" t="str">
-        <x:v>نظام الإجراءات الجزائية</x:v>
+        <x:v>تخريج ودراسة الأسانيد</x:v>
       </x:c>
       <x:c r="I75" s="43" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J75" s="42" t="str">
         <x:v>نظري</x:v>
@@ -7924,7 +7880,7 @@
       </x:c>
       <x:c r="N75" s="42"/>
       <x:c r="O75" s="42" t="str">
-        <x:v>2003328-1||نظامالاجراءاتالجزايية</x:v>
+        <x:v>2001493-2||تخريجودراسةالاسانيد</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="34" customHeight="1">
@@ -7944,13 +7900,13 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="F76" s="43" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G76" s="43" t="str">
-        <x:v>2001493-2</x:v>
+        <x:v>20014201-2</x:v>
       </x:c>
       <x:c r="H76" s="42" t="str">
-        <x:v>تخريج ودراسة الأسانيد</x:v>
+        <x:v>التدريبات العملية</x:v>
       </x:c>
       <x:c r="I76" s="43" t="n">
         <x:v>2</x:v>
@@ -7969,7 +7925,7 @@
       </x:c>
       <x:c r="N76" s="42"/>
       <x:c r="O76" s="42" t="str">
-        <x:v>2001493-2||تخريجودراسةالاسانيد</x:v>
+        <x:v>20014201-2||التدريباتالعملية</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="34" customHeight="1">
@@ -7977,25 +7933,25 @@
         <x:v>72</x:v>
       </x:c>
       <x:c r="B77" s="42" t="str">
-        <x:v>الشريعة</x:v>
+        <x:v>القراءات</x:v>
       </x:c>
       <x:c r="C77" s="42" t="str">
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="D77" s="42" t="str">
-        <x:v>قديمة</x:v>
+        <x:v>جديدة</x:v>
       </x:c>
       <x:c r="E77" s="43" t="n">
-        <x:v>39</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="F77" s="43" t="n">
-        <x:v>8</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G77" s="43" t="str">
-        <x:v>20014201-2</x:v>
+        <x:v>2001221-2</x:v>
       </x:c>
       <x:c r="H77" s="42" t="str">
-        <x:v>التدريبات العملية</x:v>
+        <x:v>الفقه (1)</x:v>
       </x:c>
       <x:c r="I77" s="43" t="n">
         <x:v>2</x:v>
@@ -8004,17 +7960,17 @@
         <x:v>نظري</x:v>
       </x:c>
       <x:c r="K77" s="42" t="str">
-        <x:v>إجبارية القسم</x:v>
+        <x:v>متطلبات الكلية</x:v>
       </x:c>
       <x:c r="L77" s="42" t="str">
-        <x:v>الشريعة 39.pdf</x:v>
+        <x:v>القراءات 47.pdf</x:v>
       </x:c>
       <x:c r="M77" s="42" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
       </x:c>
       <x:c r="N77" s="42"/>
       <x:c r="O77" s="42" t="str">
-        <x:v>20014201-2||التدريباتالعملية</x:v>
+        <x:v>2001221-2||الفقه1</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="34" customHeight="1">
@@ -8037,13 +7993,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G78" s="43" t="str">
-        <x:v>2001221-2</x:v>
+        <x:v>2002111-3</x:v>
       </x:c>
       <x:c r="H78" s="42" t="str">
-        <x:v>الفقه (1)</x:v>
+        <x:v>عرض القراءات السبع (١)</x:v>
       </x:c>
       <x:c r="I78" s="43" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="J78" s="42" t="str">
         <x:v>نظري</x:v>
@@ -8059,7 +8015,7 @@
       </x:c>
       <x:c r="N78" s="42"/>
       <x:c r="O78" s="42" t="str">
-        <x:v>2001221-2||الفقه1</x:v>
+        <x:v>2002111-3||عرضالقراءاتالسبع١</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="34" customHeight="1">
@@ -8082,13 +8038,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G79" s="43" t="str">
-        <x:v>2002111-3</x:v>
+        <x:v>2002280-2</x:v>
       </x:c>
       <x:c r="H79" s="42" t="str">
-        <x:v>عرض القراءات السبع (١)</x:v>
+        <x:v>تدريبات على الجمع والكيفيات</x:v>
       </x:c>
       <x:c r="I79" s="43" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J79" s="42" t="str">
         <x:v>نظري</x:v>
@@ -8104,7 +8060,7 @@
       </x:c>
       <x:c r="N79" s="42"/>
       <x:c r="O79" s="42" t="str">
-        <x:v>2002111-3||عرضالقراءاتالسبع١</x:v>
+        <x:v>2002280-2||تدريباتعليالجمعوالكيفيات</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="34" customHeight="1">
@@ -8127,10 +8083,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G80" s="43" t="str">
-        <x:v>2002280-2</x:v>
+        <x:v>2004102-2</x:v>
       </x:c>
       <x:c r="H80" s="42" t="str">
-        <x:v>تدريبات على الجمع والكيفيات</x:v>
+        <x:v>مصطلح الحديث</x:v>
       </x:c>
       <x:c r="I80" s="43" t="n">
         <x:v>2</x:v>
@@ -8149,7 +8105,7 @@
       </x:c>
       <x:c r="N80" s="42"/>
       <x:c r="O80" s="42" t="str">
-        <x:v>2002280-2||تدريباتعليالجمعوالكيفيات</x:v>
+        <x:v>2004102-2||مصطلحالحديث</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="34" customHeight="1">
@@ -8169,16 +8125,16 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="F81" s="43" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G81" s="43" t="str">
+        <x:v>2002112-3</x:v>
+      </x:c>
+      <x:c r="H81" s="42" t="str">
+        <x:v>عرض القراءات السبع (٢)</x:v>
+      </x:c>
+      <x:c r="I81" s="43" t="n">
         <x:v>3</x:v>
-      </x:c>
-      <x:c r="G81" s="43" t="str">
-        <x:v>2004102-2</x:v>
-      </x:c>
-      <x:c r="H81" s="42" t="str">
-        <x:v>مصطلح الحديث</x:v>
-      </x:c>
-      <x:c r="I81" s="43" t="n">
-        <x:v>2</x:v>
       </x:c>
       <x:c r="J81" s="42" t="str">
         <x:v>نظري</x:v>
@@ -8194,7 +8150,7 @@
       </x:c>
       <x:c r="N81" s="42"/>
       <x:c r="O81" s="42" t="str">
-        <x:v>2004102-2||مصطلحالحديث</x:v>
+        <x:v>2002112-3||عرضالقراءاتالسبع٢</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="34" customHeight="1">
@@ -8214,13 +8170,13 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="F82" s="43" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G82" s="43" t="str">
-        <x:v>2002112-3</x:v>
+        <x:v>2002113-3</x:v>
       </x:c>
       <x:c r="H82" s="42" t="str">
-        <x:v>عرض القراءات السبع (٢)</x:v>
+        <x:v>عرض القراءات السبع (٣)</x:v>
       </x:c>
       <x:c r="I82" s="43" t="n">
         <x:v>3</x:v>
@@ -8239,7 +8195,7 @@
       </x:c>
       <x:c r="N82" s="42"/>
       <x:c r="O82" s="42" t="str">
-        <x:v>2002112-3||عرضالقراءاتالسبع٢</x:v>
+        <x:v>2002113-3||عرضالقراءاتالسبع٣</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="34" customHeight="1">
@@ -8259,13 +8215,13 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="F83" s="43" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G83" s="43" t="str">
-        <x:v>2002352-2</x:v>
+        <x:v>2002238-2</x:v>
       </x:c>
       <x:c r="H83" s="42" t="str">
-        <x:v>التفسير التحليلي (2)</x:v>
+        <x:v>الوقف والابتداء</x:v>
       </x:c>
       <x:c r="I83" s="43" t="n">
         <x:v>2</x:v>
@@ -8284,7 +8240,7 @@
       </x:c>
       <x:c r="N83" s="42"/>
       <x:c r="O83" s="42" t="str">
-        <x:v>2002352-2||التفسيرالتحليلي2</x:v>
+        <x:v>2002238-2||الوقفوالابتداء</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="34" customHeight="1">
@@ -8307,13 +8263,13 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G84" s="43" t="str">
-        <x:v>2002113-3</x:v>
+        <x:v>2002239-2</x:v>
       </x:c>
       <x:c r="H84" s="42" t="str">
-        <x:v>عرض القراءات السبع (٣)</x:v>
+        <x:v>مصادر ومناهج المؤلفين في القراءات</x:v>
       </x:c>
       <x:c r="I84" s="43" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J84" s="42" t="str">
         <x:v>نظري</x:v>
@@ -8329,7 +8285,7 @@
       </x:c>
       <x:c r="N84" s="42"/>
       <x:c r="O84" s="42" t="str">
-        <x:v>2002113-3||عرضالقراءاتالسبع٣</x:v>
+        <x:v>2002239-2||مصادرومناهجالمولفينفيالقراءات</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="34" customHeight="1">
@@ -8349,16 +8305,16 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="F85" s="43" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G85" s="43" t="str">
-        <x:v>2002238-2</x:v>
+        <x:v>2002114-3</x:v>
       </x:c>
       <x:c r="H85" s="42" t="str">
-        <x:v>الوقف والابتداء</x:v>
+        <x:v>عرض القراءات السبع (٤)</x:v>
       </x:c>
       <x:c r="I85" s="43" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="J85" s="42" t="str">
         <x:v>نظري</x:v>
@@ -8374,7 +8330,7 @@
       </x:c>
       <x:c r="N85" s="42"/>
       <x:c r="O85" s="42" t="str">
-        <x:v>2002238-2||الوقفوالابتداء</x:v>
+        <x:v>2002114-3||عرضالقراءاتالسبع٤</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="34" customHeight="1">
@@ -8394,13 +8350,13 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="F86" s="43" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G86" s="43" t="str">
-        <x:v>2002239-2</x:v>
+        <x:v>2004320-2</x:v>
       </x:c>
       <x:c r="H86" s="42" t="str">
-        <x:v>مصادر ومناهج المؤلفين في القراءات</x:v>
+        <x:v>الحديث (3)</x:v>
       </x:c>
       <x:c r="I86" s="43" t="n">
         <x:v>2</x:v>
@@ -8419,7 +8375,7 @@
       </x:c>
       <x:c r="N86" s="42"/>
       <x:c r="O86" s="42" t="str">
-        <x:v>2002239-2||مصادرومناهجالمولفينفيالقراءات</x:v>
+        <x:v>2004320-2||الحديث3</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="34" customHeight="1">
@@ -8439,16 +8395,16 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="F87" s="43" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G87" s="43" t="str">
-        <x:v>2002114-3</x:v>
+        <x:v>2002460-2</x:v>
       </x:c>
       <x:c r="H87" s="42" t="str">
-        <x:v>عرض القراءات السبع (٤)</x:v>
+        <x:v>عرض القراءات الثلاث (١)</x:v>
       </x:c>
       <x:c r="I87" s="43" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J87" s="42" t="str">
         <x:v>نظري</x:v>
@@ -8464,7 +8420,7 @@
       </x:c>
       <x:c r="N87" s="42"/>
       <x:c r="O87" s="42" t="str">
-        <x:v>2002114-3||عرضالقراءاتالسبع٤</x:v>
+        <x:v>2002460-2||عرضالقراءاتالثلاث١</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="34" customHeight="1">
@@ -8484,19 +8440,19 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="F88" s="43" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G88" s="43" t="str">
+        <x:v>2002266-6</x:v>
+      </x:c>
+      <x:c r="H88" s="42" t="str">
+        <x:v>التدريب التعاوني</x:v>
+      </x:c>
+      <x:c r="I88" s="43" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="G88" s="43" t="str">
-        <x:v>2004320-2</x:v>
-      </x:c>
-      <x:c r="H88" s="42" t="str">
-        <x:v>الحديث (3)</x:v>
-      </x:c>
-      <x:c r="I88" s="43" t="n">
-        <x:v>2</x:v>
-      </x:c>
       <x:c r="J88" s="42" t="str">
-        <x:v>نظري</x:v>
+        <x:v>تدريب</x:v>
       </x:c>
       <x:c r="K88" s="42" t="str">
         <x:v>متطلبات الكلية</x:v>
@@ -8509,7 +8465,7 @@
       </x:c>
       <x:c r="N88" s="42"/>
       <x:c r="O88" s="42" t="str">
-        <x:v>2004320-2||الحديث3</x:v>
+        <x:v>2002266-6||التدريبالتعاوني</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="34" customHeight="1">
@@ -8529,13 +8485,13 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="F89" s="43" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G89" s="43" t="str">
-        <x:v>2002460-2</x:v>
+        <x:v>2002461-2</x:v>
       </x:c>
       <x:c r="H89" s="42" t="str">
-        <x:v>عرض القراءات الثلاث (١)</x:v>
+        <x:v>عرض القراءات الثلاث (٢)</x:v>
       </x:c>
       <x:c r="I89" s="43" t="n">
         <x:v>2</x:v>
@@ -8554,7 +8510,7 @@
       </x:c>
       <x:c r="N89" s="42"/>
       <x:c r="O89" s="42" t="str">
-        <x:v>2002460-2||عرضالقراءاتالثلاث١</x:v>
+        <x:v>2002461-2||عرضالقراءاتالثلاث٢</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="34" customHeight="1">
@@ -8568,38 +8524,38 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="D90" s="42" t="str">
-        <x:v>جديدة</x:v>
+        <x:v>قديمة</x:v>
       </x:c>
       <x:c r="E90" s="43" t="n">
-        <x:v>47</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="F90" s="43" t="n">
-        <x:v>8</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G90" s="43" t="str">
-        <x:v>2002266-6</x:v>
+        <x:v>2001205-2</x:v>
       </x:c>
       <x:c r="H90" s="42" t="str">
-        <x:v>التدريب التعاوني</x:v>
+        <x:v>الحديث (1)</x:v>
       </x:c>
       <x:c r="I90" s="43" t="n">
-        <x:v>6</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J90" s="42" t="str">
-        <x:v>تدريب</x:v>
+        <x:v>نظري</x:v>
       </x:c>
       <x:c r="K90" s="42" t="str">
-        <x:v>متطلبات الكلية</x:v>
+        <x:v>إجبارية القسم</x:v>
       </x:c>
       <x:c r="L90" s="42" t="str">
-        <x:v>القراءات 47.pdf</x:v>
+        <x:v>القراءات 38.pdf</x:v>
       </x:c>
       <x:c r="M90" s="42" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
       </x:c>
       <x:c r="N90" s="42"/>
       <x:c r="O90" s="42" t="str">
-        <x:v>2002266-6||التدريبالتعاوني</x:v>
+        <x:v>2001205-2||الحديث1</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="34" customHeight="1">
@@ -8613,19 +8569,19 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="D91" s="42" t="str">
-        <x:v>جديدة</x:v>
+        <x:v>قديمة</x:v>
       </x:c>
       <x:c r="E91" s="43" t="n">
-        <x:v>47</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="F91" s="43" t="n">
-        <x:v>8</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G91" s="43" t="str">
-        <x:v>2002461-2</x:v>
+        <x:v>2001221-2</x:v>
       </x:c>
       <x:c r="H91" s="42" t="str">
-        <x:v>عرض القراءات الثلاث (٢)</x:v>
+        <x:v>الفقه (1)</x:v>
       </x:c>
       <x:c r="I91" s="43" t="n">
         <x:v>2</x:v>
@@ -8634,17 +8590,17 @@
         <x:v>نظري</x:v>
       </x:c>
       <x:c r="K91" s="42" t="str">
-        <x:v>متطلبات الكلية</x:v>
+        <x:v>إجبارية القسم</x:v>
       </x:c>
       <x:c r="L91" s="42" t="str">
-        <x:v>القراءات 47.pdf</x:v>
+        <x:v>القراءات 38.pdf</x:v>
       </x:c>
       <x:c r="M91" s="42" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
       </x:c>
       <x:c r="N91" s="42"/>
       <x:c r="O91" s="42" t="str">
-        <x:v>2002461-2||عرضالقراءاتالثلاث٢</x:v>
+        <x:v>2001221-2||الفقه1</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="34" customHeight="1">
@@ -8667,10 +8623,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G92" s="43" t="str">
-        <x:v>2001205-2</x:v>
+        <x:v>2001273-2</x:v>
       </x:c>
       <x:c r="H92" s="42" t="str">
-        <x:v>الحديث (1)</x:v>
+        <x:v>العقيدة (1)</x:v>
       </x:c>
       <x:c r="I92" s="43" t="n">
         <x:v>2</x:v>
@@ -8689,7 +8645,7 @@
       </x:c>
       <x:c r="N92" s="42"/>
       <x:c r="O92" s="42" t="str">
-        <x:v>2001205-2||الحديث1</x:v>
+        <x:v>2001273-2||العقيدة1</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="34" customHeight="1">
@@ -8709,13 +8665,13 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="F93" s="43" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G93" s="43" t="str">
-        <x:v>2001221-2</x:v>
+        <x:v>2001209-2</x:v>
       </x:c>
       <x:c r="H93" s="42" t="str">
-        <x:v>الفقه (1)</x:v>
+        <x:v>الحديث (2)</x:v>
       </x:c>
       <x:c r="I93" s="43" t="n">
         <x:v>2</x:v>
@@ -8734,7 +8690,7 @@
       </x:c>
       <x:c r="N93" s="42"/>
       <x:c r="O93" s="42" t="str">
-        <x:v>2001221-2||الفقه1</x:v>
+        <x:v>2001209-2||الحديث2</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="34" customHeight="1">
@@ -8754,13 +8710,13 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="F94" s="43" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G94" s="43" t="str">
-        <x:v>2001273-2</x:v>
+        <x:v>2001322-2</x:v>
       </x:c>
       <x:c r="H94" s="42" t="str">
-        <x:v>العقيدة (1)</x:v>
+        <x:v>الفقه (2)</x:v>
       </x:c>
       <x:c r="I94" s="43" t="n">
         <x:v>2</x:v>
@@ -8779,7 +8735,7 @@
       </x:c>
       <x:c r="N94" s="42"/>
       <x:c r="O94" s="42" t="str">
-        <x:v>2001273-2||العقيدة1</x:v>
+        <x:v>2001322-2||الفقه2</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="34" customHeight="1">
@@ -8799,13 +8755,13 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="F95" s="43" t="n">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G95" s="43" t="str">
-        <x:v>2001209-2</x:v>
+        <x:v>2001320-2</x:v>
       </x:c>
       <x:c r="H95" s="42" t="str">
-        <x:v>الحديث (2)</x:v>
+        <x:v>الحديث (3)</x:v>
       </x:c>
       <x:c r="I95" s="43" t="n">
         <x:v>2</x:v>
@@ -8824,7 +8780,7 @@
       </x:c>
       <x:c r="N95" s="42"/>
       <x:c r="O95" s="42" t="str">
-        <x:v>2001209-2||الحديث2</x:v>
+        <x:v>2001320-2||الحديث3</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="34" customHeight="1">
@@ -8832,25 +8788,25 @@
         <x:v>91</x:v>
       </x:c>
       <x:c r="B96" s="42" t="str">
-        <x:v>القراءات</x:v>
+        <x:v>القرآن وعلومه</x:v>
       </x:c>
       <x:c r="C96" s="42" t="str">
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="D96" s="42" t="str">
-        <x:v>قديمة</x:v>
+        <x:v>جديدة</x:v>
       </x:c>
       <x:c r="E96" s="43" t="n">
-        <x:v>38</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="F96" s="43" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G96" s="43" t="str">
-        <x:v>2001322-2</x:v>
+        <x:v>2004102-2</x:v>
       </x:c>
       <x:c r="H96" s="42" t="str">
-        <x:v>الفقه (2)</x:v>
+        <x:v>مصطلح الحديث</x:v>
       </x:c>
       <x:c r="I96" s="43" t="n">
         <x:v>2</x:v>
@@ -8859,17 +8815,17 @@
         <x:v>نظري</x:v>
       </x:c>
       <x:c r="K96" s="42" t="str">
-        <x:v>إجبارية القسم</x:v>
+        <x:v>متطلبات الكلية</x:v>
       </x:c>
       <x:c r="L96" s="42" t="str">
-        <x:v>القراءات 38.pdf</x:v>
+        <x:v>القرآن وعلومه 47.pdf</x:v>
       </x:c>
       <x:c r="M96" s="42" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
       </x:c>
       <x:c r="N96" s="42"/>
       <x:c r="O96" s="42" t="str">
-        <x:v>2001322-2||الفقه2</x:v>
+        <x:v>2004102-2||مصطلحالحديث</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="34" customHeight="1">
@@ -8877,22 +8833,22 @@
         <x:v>92</x:v>
       </x:c>
       <x:c r="B97" s="42" t="str">
-        <x:v>القراءات</x:v>
+        <x:v>القرآن وعلومه</x:v>
       </x:c>
       <x:c r="C97" s="42" t="str">
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="D97" s="42" t="str">
-        <x:v>قديمة</x:v>
+        <x:v>جديدة</x:v>
       </x:c>
       <x:c r="E97" s="43" t="n">
-        <x:v>38</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="F97" s="43" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G97" s="43" t="str">
-        <x:v>2001320-2</x:v>
+        <x:v>2004320-2</x:v>
       </x:c>
       <x:c r="H97" s="42" t="str">
         <x:v>الحديث (3)</x:v>
@@ -8904,17 +8860,17 @@
         <x:v>نظري</x:v>
       </x:c>
       <x:c r="K97" s="42" t="str">
-        <x:v>إجبارية القسم</x:v>
+        <x:v>متطلبات الكلية</x:v>
       </x:c>
       <x:c r="L97" s="42" t="str">
-        <x:v>القراءات 38.pdf</x:v>
+        <x:v>القرآن وعلومه 47.pdf</x:v>
       </x:c>
       <x:c r="M97" s="42" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
       </x:c>
       <x:c r="N97" s="42"/>
       <x:c r="O97" s="42" t="str">
-        <x:v>2001320-2||الحديث3</x:v>
+        <x:v>2004320-2||الحديث3</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="34" customHeight="1">
@@ -8934,13 +8890,13 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="F98" s="43" t="n">
-        <x:v>2</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G98" s="43" t="str">
-        <x:v>2004102-2</x:v>
+        <x:v>20024101-2</x:v>
       </x:c>
       <x:c r="H98" s="42" t="str">
-        <x:v>مصطلح الحديث</x:v>
+        <x:v>قاعة بحث</x:v>
       </x:c>
       <x:c r="I98" s="43" t="n">
         <x:v>2</x:v>
@@ -8949,7 +8905,7 @@
         <x:v>نظري</x:v>
       </x:c>
       <x:c r="K98" s="42" t="str">
-        <x:v>متطلبات الكلية</x:v>
+        <x:v>إجبارية القسم</x:v>
       </x:c>
       <x:c r="L98" s="42" t="str">
         <x:v>القرآن وعلومه 47.pdf</x:v>
@@ -8959,7 +8915,7 @@
       </x:c>
       <x:c r="N98" s="42"/>
       <x:c r="O98" s="42" t="str">
-        <x:v>2004102-2||مصطلحالحديث</x:v>
+        <x:v>20024101-2||قاعةبحث</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="34" customHeight="1">
@@ -8979,22 +8935,22 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="F99" s="43" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G99" s="43" t="str">
+        <x:v>2002266-5</x:v>
+      </x:c>
+      <x:c r="H99" s="42" t="str">
+        <x:v>التدريب التعاوني</x:v>
+      </x:c>
+      <x:c r="I99" s="43" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G99" s="43" t="str">
-        <x:v>2004320-2</x:v>
-      </x:c>
-      <x:c r="H99" s="42" t="str">
-        <x:v>الحديث (3)</x:v>
-      </x:c>
-      <x:c r="I99" s="43" t="n">
-        <x:v>2</x:v>
-      </x:c>
       <x:c r="J99" s="42" t="str">
-        <x:v>نظري</x:v>
+        <x:v>تدريب</x:v>
       </x:c>
       <x:c r="K99" s="42" t="str">
-        <x:v>متطلبات الكلية</x:v>
+        <x:v>إجبارية القسم</x:v>
       </x:c>
       <x:c r="L99" s="42" t="str">
         <x:v>القرآن وعلومه 47.pdf</x:v>
@@ -9004,7 +8960,7 @@
       </x:c>
       <x:c r="N99" s="42"/>
       <x:c r="O99" s="42" t="str">
-        <x:v>2004320-2||الحديث3</x:v>
+        <x:v>2002266-5||التدريبالتعاوني</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="34" customHeight="1">
@@ -9018,19 +8974,19 @@
         <x:v>بكالوريوس</x:v>
       </x:c>
       <x:c r="D100" s="42" t="str">
-        <x:v>جديدة</x:v>
+        <x:v>قديمة</x:v>
       </x:c>
       <x:c r="E100" s="43" t="n">
-        <x:v>47</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="F100" s="43" t="n">
-        <x:v>7</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G100" s="43" t="str">
-        <x:v>20024101-2</x:v>
+        <x:v>101221-2</x:v>
       </x:c>
       <x:c r="H100" s="42" t="str">
-        <x:v>قاعة بحث</x:v>
+        <x:v>الفقه (1)</x:v>
       </x:c>
       <x:c r="I100" s="43" t="n">
         <x:v>2</x:v>
@@ -9042,14 +8998,14 @@
         <x:v>إجبارية القسم</x:v>
       </x:c>
       <x:c r="L100" s="42" t="str">
-        <x:v>القرآن وعلومه 47.pdf</x:v>
+        <x:v>القرآن وعلومه 39.pdf</x:v>
       </x:c>
       <x:c r="M100" s="42" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
       </x:c>
       <x:c r="N100" s="42"/>
       <x:c r="O100" s="42" t="str">
-        <x:v>20024101-2||قاعةبحث</x:v>
+        <x:v>101221-2||الفقه1</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="34" customHeight="1">
@@ -9057,44 +9013,44 @@
         <x:v>96</x:v>
       </x:c>
       <x:c r="B101" s="42" t="str">
-        <x:v>القرآن وعلومه</x:v>
+        <x:v>أصول الفقه</x:v>
       </x:c>
       <x:c r="C101" s="42" t="str">
-        <x:v>بكالوريوس</x:v>
+        <x:v>دكتوراه</x:v>
       </x:c>
       <x:c r="D101" s="42" t="str">
         <x:v>جديدة</x:v>
       </x:c>
       <x:c r="E101" s="43" t="n">
-        <x:v>47</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F101" s="43" t="n">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G101" s="43" t="str">
-        <x:v>2002266-5</x:v>
+        <x:v>2001901-2</x:v>
       </x:c>
       <x:c r="H101" s="42" t="str">
-        <x:v>التدريب التعاوني</x:v>
+        <x:v>دراسات مقاصدية</x:v>
       </x:c>
       <x:c r="I101" s="43" t="n">
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J101" s="42" t="str">
-        <x:v>تدريب</x:v>
+        <x:v>نظري</x:v>
       </x:c>
       <x:c r="K101" s="42" t="str">
         <x:v>إجبارية القسم</x:v>
       </x:c>
       <x:c r="L101" s="42" t="str">
-        <x:v>القرآن وعلومه 47.pdf</x:v>
+        <x:v>الدكتوراه في أصول الفقه.pdf</x:v>
       </x:c>
       <x:c r="M101" s="42" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
       </x:c>
       <x:c r="N101" s="42"/>
       <x:c r="O101" s="42" t="str">
-        <x:v>2002266-5||التدريبالتعاوني</x:v>
+        <x:v>2001901-2||دراساتمقاصدية</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="34" customHeight="1">
@@ -9102,28 +9058,28 @@
         <x:v>97</x:v>
       </x:c>
       <x:c r="B102" s="42" t="str">
-        <x:v>القرآن وعلومه</x:v>
+        <x:v>أصول الفقه</x:v>
       </x:c>
       <x:c r="C102" s="42" t="str">
-        <x:v>بكالوريوس</x:v>
+        <x:v>دكتوراه</x:v>
       </x:c>
       <x:c r="D102" s="42" t="str">
-        <x:v>قديمة</x:v>
+        <x:v>جديدة</x:v>
       </x:c>
       <x:c r="E102" s="43" t="n">
-        <x:v>39</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F102" s="43" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G102" s="43" t="str">
+        <x:v>2001902-3</x:v>
+      </x:c>
+      <x:c r="H102" s="42" t="str">
+        <x:v>دراسة تحليلية أصولية</x:v>
+      </x:c>
+      <x:c r="I102" s="43" t="n">
         <x:v>3</x:v>
-      </x:c>
-      <x:c r="G102" s="43" t="str">
-        <x:v>101221-2</x:v>
-      </x:c>
-      <x:c r="H102" s="42" t="str">
-        <x:v>الفقه (1)</x:v>
-      </x:c>
-      <x:c r="I102" s="43" t="n">
-        <x:v>2</x:v>
       </x:c>
       <x:c r="J102" s="42" t="str">
         <x:v>نظري</x:v>
@@ -9132,14 +9088,14 @@
         <x:v>إجبارية القسم</x:v>
       </x:c>
       <x:c r="L102" s="42" t="str">
-        <x:v>القرآن وعلومه 39.pdf</x:v>
+        <x:v>الدكتوراه في أصول الفقه.pdf</x:v>
       </x:c>
       <x:c r="M102" s="42" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
       </x:c>
       <x:c r="N102" s="42"/>
       <x:c r="O102" s="42" t="str">
-        <x:v>101221-2||الفقه1</x:v>
+        <x:v>2001902-3||دراسةتحليليةاصولية</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="34" customHeight="1">
@@ -9162,13 +9118,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G103" s="43" t="str">
-        <x:v>2001901-2</x:v>
+        <x:v>2001903-4</x:v>
       </x:c>
       <x:c r="H103" s="42" t="str">
-        <x:v>دراسات مقاصدية</x:v>
+        <x:v>الاجتهاد الاستدلالي والفتوى</x:v>
       </x:c>
       <x:c r="I103" s="43" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="J103" s="42" t="str">
         <x:v>نظري</x:v>
@@ -9184,7 +9140,7 @@
       </x:c>
       <x:c r="N103" s="42"/>
       <x:c r="O103" s="42" t="str">
-        <x:v>2001901-2||دراساتمقاصدية</x:v>
+        <x:v>2001903-4||الاجتهادالاستدلاليوالفتوي</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="34" customHeight="1">
@@ -9192,10 +9148,10 @@
         <x:v>99</x:v>
       </x:c>
       <x:c r="B104" s="42" t="str">
-        <x:v>أصول الفقه</x:v>
+        <x:v>الفقه</x:v>
       </x:c>
       <x:c r="C104" s="42" t="str">
-        <x:v>دكتوراه</x:v>
+        <x:v>ماجستير</x:v>
       </x:c>
       <x:c r="D104" s="42" t="str">
         <x:v>جديدة</x:v>
@@ -9204,16 +9160,16 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F104" s="43" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G104" s="43" t="str">
-        <x:v>2001902-3</x:v>
+        <x:v>2003880-2</x:v>
       </x:c>
       <x:c r="H104" s="42" t="str">
-        <x:v>دراسة تحليلية أصولية</x:v>
+        <x:v>الأنظمة العدلية في السعودية</x:v>
       </x:c>
       <x:c r="I104" s="43" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J104" s="42" t="str">
         <x:v>نظري</x:v>
@@ -9222,105 +9178,49 @@
         <x:v>إجبارية القسم</x:v>
       </x:c>
       <x:c r="L104" s="42" t="str">
-        <x:v>الدكتوراه في أصول الفقه.pdf</x:v>
+        <x:v>الماجستير في الفقه.pdf</x:v>
       </x:c>
       <x:c r="M104" s="42" t="str">
         <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
       </x:c>
       <x:c r="N104" s="42"/>
       <x:c r="O104" s="42" t="str">
-        <x:v>2001902-3||دراسةتحليليةاصولية</x:v>
+        <x:v>2003880-2||الانظمةالعدليةفيالسعودية</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="34" customHeight="1">
-      <x:c r="A105" s="33" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="B105" s="42" t="str">
-        <x:v>أصول الفقه</x:v>
-      </x:c>
-      <x:c r="C105" s="42" t="str">
-        <x:v>دكتوراه</x:v>
-      </x:c>
-      <x:c r="D105" s="42" t="str">
-        <x:v>جديدة</x:v>
-      </x:c>
-      <x:c r="E105" s="43" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F105" s="43" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G105" s="43" t="str">
-        <x:v>2001903-4</x:v>
-      </x:c>
-      <x:c r="H105" s="42" t="str">
-        <x:v>الاجتهاد الاستدلالي والفتوى</x:v>
-      </x:c>
-      <x:c r="I105" s="43" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="J105" s="42" t="str">
-        <x:v>نظري</x:v>
-      </x:c>
-      <x:c r="K105" s="42" t="str">
-        <x:v>إجبارية القسم</x:v>
-      </x:c>
-      <x:c r="L105" s="42" t="str">
-        <x:v>الدكتوراه في أصول الفقه.pdf</x:v>
-      </x:c>
-      <x:c r="M105" s="42" t="str">
-        <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
-      </x:c>
+      <x:c r="A105" s="33"/>
+      <x:c r="B105" s="42"/>
+      <x:c r="C105" s="42"/>
+      <x:c r="D105" s="42"/>
+      <x:c r="E105" s="43"/>
+      <x:c r="F105" s="43"/>
+      <x:c r="G105" s="43"/>
+      <x:c r="H105" s="42"/>
+      <x:c r="I105" s="43"/>
+      <x:c r="J105" s="42"/>
+      <x:c r="K105" s="42"/>
+      <x:c r="L105" s="42"/>
+      <x:c r="M105" s="42"/>
       <x:c r="N105" s="42"/>
-      <x:c r="O105" s="42" t="str">
-        <x:v>2001903-4||الاجتهادالاستدلاليوالفتوي</x:v>
-      </x:c>
+      <x:c r="O105" s="42"/>
     </x:row>
     <x:row r="106" ht="34" customHeight="1">
-      <x:c r="A106" s="33" t="n">
-        <x:v>101</x:v>
-      </x:c>
-      <x:c r="B106" s="42" t="str">
-        <x:v>الفقه</x:v>
-      </x:c>
-      <x:c r="C106" s="42" t="str">
-        <x:v>ماجستير</x:v>
-      </x:c>
-      <x:c r="D106" s="42" t="str">
-        <x:v>جديدة</x:v>
-      </x:c>
-      <x:c r="E106" s="43" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F106" s="43" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="G106" s="43" t="str">
-        <x:v>2003880-2</x:v>
-      </x:c>
-      <x:c r="H106" s="42" t="str">
-        <x:v>الأنظمة العدلية في السعودية</x:v>
-      </x:c>
-      <x:c r="I106" s="43" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="J106" s="42" t="str">
-        <x:v>نظري</x:v>
-      </x:c>
-      <x:c r="K106" s="42" t="str">
-        <x:v>إجبارية القسم</x:v>
-      </x:c>
-      <x:c r="L106" s="42" t="str">
-        <x:v>الماجستير في الفقه.pdf</x:v>
-      </x:c>
-      <x:c r="M106" s="42" t="str">
-        <x:v>لا يوجد توصيف تحت الرمز في المستودع</x:v>
-      </x:c>
+      <x:c r="A106" s="33"/>
+      <x:c r="B106" s="42"/>
+      <x:c r="C106" s="42"/>
+      <x:c r="D106" s="42"/>
+      <x:c r="E106" s="43"/>
+      <x:c r="F106" s="43"/>
+      <x:c r="G106" s="43"/>
+      <x:c r="H106" s="42"/>
+      <x:c r="I106" s="43"/>
+      <x:c r="J106" s="42"/>
+      <x:c r="K106" s="42"/>
+      <x:c r="L106" s="42"/>
+      <x:c r="M106" s="42"/>
       <x:c r="N106" s="42"/>
-      <x:c r="O106" s="42" t="str">
-        <x:v>2003880-2||الانظمةالعدليةفيالسعودية</x:v>
-      </x:c>
+      <x:c r="O106" s="42"/>
     </x:row>
     <x:row r="107" ht="34" customHeight="1">
       <x:c r="A107" s="33"/>
@@ -9992,7 +9892,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa4771fb47dc4535"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb643a2132cd54965"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>